<commit_message>
feat: actions fetch kookmin 2026-09-14T23:58Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12517" uniqueCount="3174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12493" uniqueCount="3172">
   <si>
     <t>campusCode</t>
   </si>
@@ -8671,6 +8671,9 @@
     <t>전공실기3</t>
   </si>
   <si>
+    <t>김진석</t>
+  </si>
+  <si>
     <t>이옥재</t>
   </si>
   <si>
@@ -8695,31 +8698,22 @@
     <t>플루트페다고지전공</t>
   </si>
   <si>
-    <t>697800a</t>
-  </si>
-  <si>
-    <t>플루트 전공실기Ⅰ</t>
+    <t>697810a</t>
+  </si>
+  <si>
+    <t>플루트 전공실기Ⅱ</t>
+  </si>
+  <si>
+    <t>예술관3층17호실</t>
+  </si>
+  <si>
+    <t>697850a</t>
+  </si>
+  <si>
+    <t>플루트 앙상블Ⅱ</t>
   </si>
   <si>
     <t>국성화</t>
-  </si>
-  <si>
-    <t>예술관3층10호실,예술관3층17호실</t>
-  </si>
-  <si>
-    <t>697810a</t>
-  </si>
-  <si>
-    <t>플루트 전공실기Ⅱ</t>
-  </si>
-  <si>
-    <t>예술관3층17호실</t>
-  </si>
-  <si>
-    <t>697850a</t>
-  </si>
-  <si>
-    <t>플루트 앙상블Ⅱ</t>
   </si>
   <si>
     <t>702770a</t>
@@ -9909,7 +9903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M1043"/>
+  <dimension ref="A1:M1041"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -48396,7 +48390,7 @@
         <v>2</v>
       </c>
       <c r="I939" t="s">
-        <v>2876</v>
+        <v>2886</v>
       </c>
       <c r="J939" t="s">
         <v>650</v>
@@ -48437,7 +48431,7 @@
         <v>2</v>
       </c>
       <c r="I940" t="s">
-        <v>2886</v>
+        <v>2887</v>
       </c>
       <c r="J940" t="s">
         <v>650</v>
@@ -48478,10 +48472,10 @@
         <v>2</v>
       </c>
       <c r="I941" t="s">
-        <v>2873</v>
+        <v>2865</v>
       </c>
       <c r="J941" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="K941" t="s">
         <v>21</v>
@@ -48490,7 +48484,7 @@
         <v>2879</v>
       </c>
       <c r="M941" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
     </row>
     <row r="942" spans="1:13" x14ac:dyDescent="0.25">
@@ -48510,28 +48504,28 @@
         <v>16</v>
       </c>
       <c r="F942" t="s">
-        <v>2884</v>
+        <v>2888</v>
       </c>
       <c r="G942" t="s">
-        <v>2885</v>
+        <v>2889</v>
       </c>
       <c r="H942">
         <v>2</v>
       </c>
       <c r="I942" t="s">
-        <v>2865</v>
+        <v>2890</v>
       </c>
       <c r="J942" t="s">
-        <v>642</v>
+        <v>2641</v>
       </c>
       <c r="K942" t="s">
         <v>21</v>
       </c>
       <c r="L942" t="s">
-        <v>2879</v>
+        <v>896</v>
       </c>
       <c r="M942" t="s">
-        <v>646</v>
+        <v>23</v>
       </c>
     </row>
     <row r="943" spans="1:13" x14ac:dyDescent="0.25">
@@ -48551,25 +48545,25 @@
         <v>16</v>
       </c>
       <c r="F943" t="s">
-        <v>2887</v>
+        <v>2891</v>
       </c>
       <c r="G943" t="s">
-        <v>2888</v>
+        <v>2892</v>
       </c>
       <c r="H943">
         <v>2</v>
       </c>
       <c r="I943" t="s">
-        <v>2889</v>
+        <v>2865</v>
       </c>
       <c r="J943" t="s">
-        <v>2641</v>
+        <v>2649</v>
       </c>
       <c r="K943" t="s">
         <v>21</v>
       </c>
       <c r="L943" t="s">
-        <v>896</v>
+        <v>858</v>
       </c>
       <c r="M943" t="s">
         <v>23</v>
@@ -48583,34 +48577,34 @@
         <v>2823</v>
       </c>
       <c r="C944" t="s">
-        <v>2861</v>
+        <v>2893</v>
       </c>
       <c r="D944" t="s">
-        <v>2862</v>
+        <v>2894</v>
       </c>
       <c r="E944" t="s">
         <v>16</v>
       </c>
       <c r="F944" t="s">
-        <v>2890</v>
+        <v>2895</v>
       </c>
       <c r="G944" t="s">
-        <v>2891</v>
+        <v>2896</v>
       </c>
       <c r="H944">
         <v>2</v>
       </c>
       <c r="I944" t="s">
-        <v>2865</v>
+        <v>205</v>
       </c>
       <c r="J944" t="s">
-        <v>2649</v>
+        <v>803</v>
       </c>
       <c r="K944" t="s">
         <v>21</v>
       </c>
       <c r="L944" t="s">
-        <v>858</v>
+        <v>2897</v>
       </c>
       <c r="M944" t="s">
         <v>23</v>
@@ -48624,34 +48618,34 @@
         <v>2823</v>
       </c>
       <c r="C945" t="s">
-        <v>2892</v>
+        <v>2893</v>
       </c>
       <c r="D945" t="s">
-        <v>2893</v>
+        <v>2894</v>
       </c>
       <c r="E945" t="s">
         <v>16</v>
       </c>
       <c r="F945" t="s">
-        <v>2894</v>
+        <v>2898</v>
       </c>
       <c r="G945" t="s">
-        <v>2895</v>
+        <v>2899</v>
       </c>
       <c r="H945">
         <v>2</v>
       </c>
       <c r="I945" t="s">
-        <v>2896</v>
+        <v>2900</v>
       </c>
       <c r="J945" t="s">
-        <v>809</v>
+        <v>790</v>
       </c>
       <c r="K945" t="s">
         <v>21</v>
       </c>
       <c r="L945" t="s">
-        <v>2897</v>
+        <v>2833</v>
       </c>
       <c r="M945" t="s">
         <v>23</v>
@@ -48665,34 +48659,34 @@
         <v>2823</v>
       </c>
       <c r="C946" t="s">
-        <v>2892</v>
+        <v>2893</v>
       </c>
       <c r="D946" t="s">
-        <v>2893</v>
+        <v>2894</v>
       </c>
       <c r="E946" t="s">
         <v>16</v>
       </c>
       <c r="F946" t="s">
-        <v>2898</v>
+        <v>2901</v>
       </c>
       <c r="G946" t="s">
-        <v>2899</v>
+        <v>2902</v>
       </c>
       <c r="H946">
         <v>2</v>
       </c>
       <c r="I946" t="s">
-        <v>205</v>
+        <v>2900</v>
       </c>
       <c r="J946" t="s">
-        <v>803</v>
+        <v>2903</v>
       </c>
       <c r="K946" t="s">
         <v>21</v>
       </c>
       <c r="L946" t="s">
-        <v>2900</v>
+        <v>2833</v>
       </c>
       <c r="M946" t="s">
         <v>23</v>
@@ -48706,34 +48700,34 @@
         <v>2823</v>
       </c>
       <c r="C947" t="s">
-        <v>2892</v>
+        <v>2893</v>
       </c>
       <c r="D947" t="s">
-        <v>2893</v>
+        <v>2894</v>
       </c>
       <c r="E947" t="s">
         <v>16</v>
       </c>
       <c r="F947" t="s">
-        <v>2901</v>
+        <v>2904</v>
       </c>
       <c r="G947" t="s">
-        <v>2902</v>
+        <v>2905</v>
       </c>
       <c r="H947">
         <v>2</v>
       </c>
       <c r="I947" t="s">
-        <v>2896</v>
+        <v>2906</v>
       </c>
       <c r="J947" t="s">
-        <v>790</v>
+        <v>2907</v>
       </c>
       <c r="K947" t="s">
         <v>21</v>
       </c>
       <c r="L947" t="s">
-        <v>2833</v>
+        <v>2908</v>
       </c>
       <c r="M947" t="s">
         <v>23</v>
@@ -48747,34 +48741,34 @@
         <v>2823</v>
       </c>
       <c r="C948" t="s">
-        <v>2892</v>
+        <v>2909</v>
       </c>
       <c r="D948" t="s">
-        <v>2893</v>
+        <v>2910</v>
       </c>
       <c r="E948" t="s">
         <v>16</v>
       </c>
       <c r="F948" t="s">
-        <v>2903</v>
+        <v>2911</v>
       </c>
       <c r="G948" t="s">
-        <v>2904</v>
+        <v>2878</v>
       </c>
       <c r="H948">
         <v>2</v>
       </c>
       <c r="I948" t="s">
-        <v>2896</v>
+        <v>2912</v>
       </c>
       <c r="J948" t="s">
-        <v>2905</v>
+        <v>2913</v>
       </c>
       <c r="K948" t="s">
         <v>21</v>
       </c>
       <c r="L948" t="s">
-        <v>2833</v>
+        <v>2897</v>
       </c>
       <c r="M948" t="s">
         <v>23</v>
@@ -48788,34 +48782,34 @@
         <v>2823</v>
       </c>
       <c r="C949" t="s">
-        <v>2892</v>
+        <v>2909</v>
       </c>
       <c r="D949" t="s">
-        <v>2893</v>
+        <v>2910</v>
       </c>
       <c r="E949" t="s">
         <v>16</v>
       </c>
       <c r="F949" t="s">
-        <v>2906</v>
+        <v>2914</v>
       </c>
       <c r="G949" t="s">
-        <v>2907</v>
+        <v>2915</v>
       </c>
       <c r="H949">
         <v>2</v>
       </c>
       <c r="I949" t="s">
-        <v>2908</v>
+        <v>2916</v>
       </c>
       <c r="J949" t="s">
-        <v>2909</v>
+        <v>2917</v>
       </c>
       <c r="K949" t="s">
         <v>21</v>
       </c>
       <c r="L949" t="s">
-        <v>2910</v>
+        <v>858</v>
       </c>
       <c r="M949" t="s">
         <v>23</v>
@@ -48829,34 +48823,34 @@
         <v>2823</v>
       </c>
       <c r="C950" t="s">
-        <v>2911</v>
+        <v>2909</v>
       </c>
       <c r="D950" t="s">
-        <v>2912</v>
+        <v>2910</v>
       </c>
       <c r="E950" t="s">
         <v>16</v>
       </c>
       <c r="F950" t="s">
-        <v>2913</v>
+        <v>2918</v>
       </c>
       <c r="G950" t="s">
-        <v>2878</v>
+        <v>2881</v>
       </c>
       <c r="H950">
         <v>2</v>
       </c>
       <c r="I950" t="s">
-        <v>2914</v>
+        <v>2912</v>
       </c>
       <c r="J950" t="s">
-        <v>2915</v>
+        <v>2919</v>
       </c>
       <c r="K950" t="s">
         <v>21</v>
       </c>
       <c r="L950" t="s">
-        <v>2900</v>
+        <v>2897</v>
       </c>
       <c r="M950" t="s">
         <v>23</v>
@@ -48870,34 +48864,34 @@
         <v>2823</v>
       </c>
       <c r="C951" t="s">
-        <v>2911</v>
+        <v>2909</v>
       </c>
       <c r="D951" t="s">
-        <v>2912</v>
+        <v>2910</v>
       </c>
       <c r="E951" t="s">
         <v>16</v>
       </c>
       <c r="F951" t="s">
-        <v>2916</v>
+        <v>2920</v>
       </c>
       <c r="G951" t="s">
-        <v>2917</v>
+        <v>2885</v>
       </c>
       <c r="H951">
         <v>2</v>
       </c>
       <c r="I951" t="s">
-        <v>2918</v>
+        <v>2921</v>
       </c>
       <c r="J951" t="s">
-        <v>2919</v>
+        <v>2922</v>
       </c>
       <c r="K951" t="s">
         <v>21</v>
       </c>
       <c r="L951" t="s">
-        <v>858</v>
+        <v>2897</v>
       </c>
       <c r="M951" t="s">
         <v>23</v>
@@ -48911,34 +48905,34 @@
         <v>2823</v>
       </c>
       <c r="C952" t="s">
-        <v>2911</v>
+        <v>2909</v>
       </c>
       <c r="D952" t="s">
-        <v>2912</v>
+        <v>2910</v>
       </c>
       <c r="E952" t="s">
         <v>16</v>
       </c>
       <c r="F952" t="s">
-        <v>2920</v>
+        <v>2923</v>
       </c>
       <c r="G952" t="s">
-        <v>2881</v>
+        <v>2924</v>
       </c>
       <c r="H952">
         <v>2</v>
       </c>
       <c r="I952" t="s">
-        <v>2914</v>
+        <v>2916</v>
       </c>
       <c r="J952" t="s">
-        <v>2921</v>
+        <v>2925</v>
       </c>
       <c r="K952" t="s">
         <v>21</v>
       </c>
       <c r="L952" t="s">
-        <v>2900</v>
+        <v>896</v>
       </c>
       <c r="M952" t="s">
         <v>23</v>
@@ -48952,34 +48946,34 @@
         <v>2823</v>
       </c>
       <c r="C953" t="s">
-        <v>2911</v>
+        <v>2909</v>
       </c>
       <c r="D953" t="s">
-        <v>2912</v>
+        <v>2910</v>
       </c>
       <c r="E953" t="s">
         <v>16</v>
       </c>
       <c r="F953" t="s">
-        <v>2922</v>
+        <v>2926</v>
       </c>
       <c r="G953" t="s">
-        <v>2885</v>
+        <v>2927</v>
       </c>
       <c r="H953">
         <v>2</v>
       </c>
       <c r="I953" t="s">
-        <v>2923</v>
+        <v>2912</v>
       </c>
       <c r="J953" t="s">
-        <v>2924</v>
+        <v>2928</v>
       </c>
       <c r="K953" t="s">
         <v>21</v>
       </c>
       <c r="L953" t="s">
-        <v>2900</v>
+        <v>873</v>
       </c>
       <c r="M953" t="s">
         <v>23</v>
@@ -48993,34 +48987,34 @@
         <v>2823</v>
       </c>
       <c r="C954" t="s">
-        <v>2911</v>
+        <v>2929</v>
       </c>
       <c r="D954" t="s">
-        <v>2912</v>
+        <v>2930</v>
       </c>
       <c r="E954" t="s">
         <v>16</v>
       </c>
       <c r="F954" t="s">
-        <v>2925</v>
+        <v>2931</v>
       </c>
       <c r="G954" t="s">
-        <v>2926</v>
+        <v>2932</v>
       </c>
       <c r="H954">
         <v>2</v>
       </c>
       <c r="I954" t="s">
-        <v>2918</v>
+        <v>2933</v>
       </c>
       <c r="J954" t="s">
-        <v>2927</v>
+        <v>2571</v>
       </c>
       <c r="K954" t="s">
         <v>21</v>
       </c>
       <c r="L954" t="s">
-        <v>896</v>
+        <v>697</v>
       </c>
       <c r="M954" t="s">
         <v>23</v>
@@ -49034,37 +49028,37 @@
         <v>2823</v>
       </c>
       <c r="C955" t="s">
-        <v>2911</v>
+        <v>2929</v>
       </c>
       <c r="D955" t="s">
-        <v>2912</v>
+        <v>2930</v>
       </c>
       <c r="E955" t="s">
         <v>16</v>
       </c>
       <c r="F955" t="s">
-        <v>2928</v>
+        <v>2931</v>
       </c>
       <c r="G955" t="s">
-        <v>2929</v>
+        <v>2932</v>
       </c>
       <c r="H955">
         <v>2</v>
       </c>
       <c r="I955" t="s">
-        <v>2914</v>
+        <v>2933</v>
       </c>
       <c r="J955" t="s">
-        <v>2930</v>
+        <v>2389</v>
       </c>
       <c r="K955" t="s">
         <v>21</v>
       </c>
       <c r="L955" t="s">
-        <v>873</v>
+        <v>697</v>
       </c>
       <c r="M955" t="s">
-        <v>23</v>
+        <v>640</v>
       </c>
     </row>
     <row r="956" spans="1:13" x14ac:dyDescent="0.25">
@@ -49075,34 +49069,34 @@
         <v>2823</v>
       </c>
       <c r="C956" t="s">
-        <v>2931</v>
+        <v>2929</v>
       </c>
       <c r="D956" t="s">
-        <v>2932</v>
+        <v>2930</v>
       </c>
       <c r="E956" t="s">
         <v>16</v>
       </c>
       <c r="F956" t="s">
-        <v>2933</v>
+        <v>2934</v>
       </c>
       <c r="G956" t="s">
-        <v>2934</v>
+        <v>2935</v>
       </c>
       <c r="H956">
         <v>2</v>
       </c>
       <c r="I956" t="s">
-        <v>2935</v>
+        <v>205</v>
       </c>
       <c r="J956" t="s">
-        <v>2571</v>
+        <v>2936</v>
       </c>
       <c r="K956" t="s">
         <v>21</v>
       </c>
       <c r="L956" t="s">
-        <v>697</v>
+        <v>2937</v>
       </c>
       <c r="M956" t="s">
         <v>23</v>
@@ -49116,34 +49110,34 @@
         <v>2823</v>
       </c>
       <c r="C957" t="s">
-        <v>2931</v>
+        <v>2929</v>
       </c>
       <c r="D957" t="s">
-        <v>2932</v>
+        <v>2930</v>
       </c>
       <c r="E957" t="s">
         <v>16</v>
       </c>
       <c r="F957" t="s">
-        <v>2933</v>
+        <v>2934</v>
       </c>
       <c r="G957" t="s">
-        <v>2934</v>
+        <v>2935</v>
       </c>
       <c r="H957">
         <v>2</v>
       </c>
       <c r="I957" t="s">
-        <v>2935</v>
+        <v>2938</v>
       </c>
       <c r="J957" t="s">
-        <v>2389</v>
+        <v>2571</v>
       </c>
       <c r="K957" t="s">
         <v>21</v>
       </c>
       <c r="L957" t="s">
-        <v>697</v>
+        <v>858</v>
       </c>
       <c r="M957" t="s">
         <v>640</v>
@@ -49157,37 +49151,37 @@
         <v>2823</v>
       </c>
       <c r="C958" t="s">
-        <v>2931</v>
+        <v>2929</v>
       </c>
       <c r="D958" t="s">
-        <v>2932</v>
+        <v>2930</v>
       </c>
       <c r="E958" t="s">
         <v>16</v>
       </c>
       <c r="F958" t="s">
-        <v>2936</v>
+        <v>2934</v>
       </c>
       <c r="G958" t="s">
-        <v>2937</v>
+        <v>2935</v>
       </c>
       <c r="H958">
         <v>2</v>
       </c>
       <c r="I958" t="s">
-        <v>205</v>
+        <v>2938</v>
       </c>
       <c r="J958" t="s">
-        <v>2938</v>
+        <v>2939</v>
       </c>
       <c r="K958" t="s">
         <v>21</v>
       </c>
       <c r="L958" t="s">
-        <v>2939</v>
+        <v>858</v>
       </c>
       <c r="M958" t="s">
-        <v>23</v>
+        <v>643</v>
       </c>
     </row>
     <row r="959" spans="1:13" x14ac:dyDescent="0.25">
@@ -49198,37 +49192,37 @@
         <v>2823</v>
       </c>
       <c r="C959" t="s">
-        <v>2931</v>
+        <v>2929</v>
       </c>
       <c r="D959" t="s">
-        <v>2932</v>
+        <v>2930</v>
       </c>
       <c r="E959" t="s">
         <v>16</v>
       </c>
       <c r="F959" t="s">
-        <v>2936</v>
+        <v>2940</v>
       </c>
       <c r="G959" t="s">
-        <v>2937</v>
+        <v>2941</v>
       </c>
       <c r="H959">
         <v>2</v>
       </c>
       <c r="I959" t="s">
-        <v>2940</v>
+        <v>2933</v>
       </c>
       <c r="J959" t="s">
-        <v>2571</v>
+        <v>2942</v>
       </c>
       <c r="K959" t="s">
         <v>21</v>
       </c>
       <c r="L959" t="s">
-        <v>858</v>
+        <v>896</v>
       </c>
       <c r="M959" t="s">
-        <v>640</v>
+        <v>23</v>
       </c>
     </row>
     <row r="960" spans="1:13" x14ac:dyDescent="0.25">
@@ -49239,37 +49233,37 @@
         <v>2823</v>
       </c>
       <c r="C960" t="s">
-        <v>2931</v>
+        <v>2929</v>
       </c>
       <c r="D960" t="s">
-        <v>2932</v>
+        <v>2930</v>
       </c>
       <c r="E960" t="s">
         <v>16</v>
       </c>
       <c r="F960" t="s">
-        <v>2936</v>
+        <v>2943</v>
       </c>
       <c r="G960" t="s">
-        <v>2937</v>
+        <v>2944</v>
       </c>
       <c r="H960">
         <v>2</v>
       </c>
       <c r="I960" t="s">
-        <v>2940</v>
+        <v>2933</v>
       </c>
       <c r="J960" t="s">
-        <v>2941</v>
+        <v>2548</v>
       </c>
       <c r="K960" t="s">
         <v>21</v>
       </c>
       <c r="L960" t="s">
-        <v>858</v>
+        <v>896</v>
       </c>
       <c r="M960" t="s">
-        <v>643</v>
+        <v>23</v>
       </c>
     </row>
     <row r="961" spans="1:13" x14ac:dyDescent="0.25">
@@ -49280,34 +49274,34 @@
         <v>2823</v>
       </c>
       <c r="C961" t="s">
-        <v>2931</v>
+        <v>2929</v>
       </c>
       <c r="D961" t="s">
-        <v>2932</v>
+        <v>2930</v>
       </c>
       <c r="E961" t="s">
         <v>16</v>
       </c>
       <c r="F961" t="s">
-        <v>2942</v>
+        <v>2945</v>
       </c>
       <c r="G961" t="s">
-        <v>2943</v>
+        <v>2946</v>
       </c>
       <c r="H961">
         <v>2</v>
       </c>
       <c r="I961" t="s">
-        <v>2935</v>
+        <v>2938</v>
       </c>
       <c r="J961" t="s">
-        <v>2944</v>
+        <v>2947</v>
       </c>
       <c r="K961" t="s">
         <v>21</v>
       </c>
       <c r="L961" t="s">
-        <v>896</v>
+        <v>858</v>
       </c>
       <c r="M961" t="s">
         <v>23</v>
@@ -49321,34 +49315,34 @@
         <v>2823</v>
       </c>
       <c r="C962" t="s">
-        <v>2931</v>
+        <v>2948</v>
       </c>
       <c r="D962" t="s">
-        <v>2932</v>
+        <v>2949</v>
       </c>
       <c r="E962" t="s">
         <v>16</v>
       </c>
       <c r="F962" t="s">
-        <v>2945</v>
+        <v>2950</v>
       </c>
       <c r="G962" t="s">
-        <v>2946</v>
+        <v>2951</v>
       </c>
       <c r="H962">
         <v>2</v>
       </c>
       <c r="I962" t="s">
-        <v>2935</v>
+        <v>1096</v>
       </c>
       <c r="J962" t="s">
-        <v>2548</v>
+        <v>711</v>
       </c>
       <c r="K962" t="s">
         <v>21</v>
       </c>
       <c r="L962" t="s">
-        <v>896</v>
+        <v>2952</v>
       </c>
       <c r="M962" t="s">
         <v>23</v>
@@ -49362,34 +49356,34 @@
         <v>2823</v>
       </c>
       <c r="C963" t="s">
-        <v>2931</v>
+        <v>2948</v>
       </c>
       <c r="D963" t="s">
-        <v>2932</v>
+        <v>2949</v>
       </c>
       <c r="E963" t="s">
         <v>16</v>
       </c>
       <c r="F963" t="s">
-        <v>2947</v>
+        <v>2953</v>
       </c>
       <c r="G963" t="s">
-        <v>2948</v>
+        <v>2954</v>
       </c>
       <c r="H963">
         <v>2</v>
       </c>
       <c r="I963" t="s">
-        <v>2940</v>
+        <v>2955</v>
       </c>
       <c r="J963" t="s">
-        <v>2949</v>
+        <v>710</v>
       </c>
       <c r="K963" t="s">
         <v>21</v>
       </c>
       <c r="L963" t="s">
-        <v>858</v>
+        <v>2952</v>
       </c>
       <c r="M963" t="s">
         <v>23</v>
@@ -49403,34 +49397,34 @@
         <v>2823</v>
       </c>
       <c r="C964" t="s">
-        <v>2950</v>
+        <v>2948</v>
       </c>
       <c r="D964" t="s">
-        <v>2951</v>
+        <v>2949</v>
       </c>
       <c r="E964" t="s">
         <v>16</v>
       </c>
       <c r="F964" t="s">
-        <v>2952</v>
+        <v>2956</v>
       </c>
       <c r="G964" t="s">
-        <v>2953</v>
+        <v>2957</v>
       </c>
       <c r="H964">
         <v>2</v>
       </c>
       <c r="I964" t="s">
-        <v>1096</v>
+        <v>2958</v>
       </c>
       <c r="J964" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="K964" t="s">
         <v>21</v>
       </c>
       <c r="L964" t="s">
-        <v>2954</v>
+        <v>2952</v>
       </c>
       <c r="M964" t="s">
         <v>23</v>
@@ -49438,40 +49432,40 @@
     </row>
     <row r="965" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A965" t="s">
-        <v>2822</v>
+        <v>2959</v>
       </c>
       <c r="B965" t="s">
-        <v>2823</v>
+        <v>2960</v>
       </c>
       <c r="C965" t="s">
-        <v>2950</v>
+        <v>2961</v>
       </c>
       <c r="D965" t="s">
-        <v>2951</v>
+        <v>2962</v>
       </c>
       <c r="E965" t="s">
-        <v>16</v>
+        <v>2274</v>
       </c>
       <c r="F965" t="s">
-        <v>2955</v>
+        <v>2963</v>
       </c>
       <c r="G965" t="s">
-        <v>2956</v>
+        <v>2964</v>
       </c>
       <c r="H965">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I965" t="s">
-        <v>2957</v>
+        <v>219</v>
       </c>
       <c r="J965" t="s">
-        <v>710</v>
+        <v>2965</v>
       </c>
       <c r="K965" t="s">
         <v>21</v>
       </c>
       <c r="L965" t="s">
-        <v>2954</v>
+        <v>2966</v>
       </c>
       <c r="M965" t="s">
         <v>23</v>
@@ -49479,40 +49473,40 @@
     </row>
     <row r="966" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A966" t="s">
-        <v>2822</v>
+        <v>2959</v>
       </c>
       <c r="B966" t="s">
-        <v>2823</v>
+        <v>2960</v>
       </c>
       <c r="C966" t="s">
-        <v>2950</v>
+        <v>2961</v>
       </c>
       <c r="D966" t="s">
-        <v>2951</v>
+        <v>2962</v>
       </c>
       <c r="E966" t="s">
         <v>16</v>
       </c>
       <c r="F966" t="s">
-        <v>2958</v>
+        <v>2967</v>
       </c>
       <c r="G966" t="s">
-        <v>2959</v>
+        <v>2968</v>
       </c>
       <c r="H966">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I966" t="s">
-        <v>2960</v>
+        <v>219</v>
       </c>
       <c r="J966" t="s">
-        <v>707</v>
+        <v>2969</v>
       </c>
       <c r="K966" t="s">
         <v>21</v>
       </c>
       <c r="L966" t="s">
-        <v>2954</v>
+        <v>2250</v>
       </c>
       <c r="M966" t="s">
         <v>23</v>
@@ -49520,40 +49514,40 @@
     </row>
     <row r="967" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A967" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B967" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C967" t="s">
         <v>2961</v>
       </c>
-      <c r="B967" t="s">
+      <c r="D967" t="s">
         <v>2962</v>
       </c>
-      <c r="C967" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D967" t="s">
-        <v>2964</v>
-      </c>
       <c r="E967" t="s">
-        <v>2274</v>
+        <v>16</v>
       </c>
       <c r="F967" t="s">
-        <v>2965</v>
+        <v>2970</v>
       </c>
       <c r="G967" t="s">
-        <v>2966</v>
+        <v>2971</v>
       </c>
       <c r="H967">
         <v>3</v>
       </c>
       <c r="I967" t="s">
-        <v>219</v>
+        <v>2972</v>
       </c>
       <c r="J967" t="s">
-        <v>2967</v>
+        <v>2973</v>
       </c>
       <c r="K967" t="s">
         <v>21</v>
       </c>
       <c r="L967" t="s">
-        <v>2968</v>
+        <v>2250</v>
       </c>
       <c r="M967" t="s">
         <v>23</v>
@@ -49561,40 +49555,40 @@
     </row>
     <row r="968" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A968" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B968" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C968" t="s">
         <v>2961</v>
       </c>
-      <c r="B968" t="s">
+      <c r="D968" t="s">
         <v>2962</v>
       </c>
-      <c r="C968" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D968" t="s">
-        <v>2964</v>
-      </c>
       <c r="E968" t="s">
-        <v>16</v>
+        <v>2274</v>
       </c>
       <c r="F968" t="s">
+        <v>2974</v>
+      </c>
+      <c r="G968" t="s">
+        <v>2975</v>
+      </c>
+      <c r="H968">
+        <v>3</v>
+      </c>
+      <c r="I968" t="s">
+        <v>2976</v>
+      </c>
+      <c r="J968" t="s">
         <v>2969</v>
       </c>
-      <c r="G968" t="s">
-        <v>2970</v>
-      </c>
-      <c r="H968">
-        <v>3</v>
-      </c>
-      <c r="I968" t="s">
-        <v>219</v>
-      </c>
-      <c r="J968" t="s">
-        <v>2971</v>
-      </c>
       <c r="K968" t="s">
         <v>21</v>
       </c>
       <c r="L968" t="s">
-        <v>2250</v>
+        <v>2150</v>
       </c>
       <c r="M968" t="s">
         <v>23</v>
@@ -49602,34 +49596,34 @@
     </row>
     <row r="969" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A969" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B969" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C969" t="s">
         <v>2961</v>
       </c>
-      <c r="B969" t="s">
+      <c r="D969" t="s">
         <v>2962</v>
-      </c>
-      <c r="C969" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D969" t="s">
-        <v>2964</v>
       </c>
       <c r="E969" t="s">
         <v>16</v>
       </c>
       <c r="F969" t="s">
-        <v>2972</v>
+        <v>2977</v>
       </c>
       <c r="G969" t="s">
-        <v>2973</v>
+        <v>2978</v>
       </c>
       <c r="H969">
         <v>3</v>
       </c>
       <c r="I969" t="s">
-        <v>2974</v>
+        <v>2979</v>
       </c>
       <c r="J969" t="s">
-        <v>2975</v>
+        <v>2980</v>
       </c>
       <c r="K969" t="s">
         <v>21</v>
@@ -49643,40 +49637,40 @@
     </row>
     <row r="970" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A970" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B970" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C970" t="s">
         <v>2961</v>
       </c>
-      <c r="B970" t="s">
+      <c r="D970" t="s">
         <v>2962</v>
       </c>
-      <c r="C970" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D970" t="s">
-        <v>2964</v>
-      </c>
       <c r="E970" t="s">
-        <v>2274</v>
+        <v>16</v>
       </c>
       <c r="F970" t="s">
-        <v>2976</v>
+        <v>2981</v>
       </c>
       <c r="G970" t="s">
-        <v>2977</v>
+        <v>2982</v>
       </c>
       <c r="H970">
         <v>3</v>
       </c>
       <c r="I970" t="s">
-        <v>2978</v>
+        <v>219</v>
       </c>
       <c r="J970" t="s">
-        <v>2971</v>
+        <v>205</v>
       </c>
       <c r="K970" t="s">
         <v>21</v>
       </c>
       <c r="L970" t="s">
-        <v>2150</v>
+        <v>205</v>
       </c>
       <c r="M970" t="s">
         <v>23</v>
@@ -49684,72 +49678,72 @@
     </row>
     <row r="971" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A971" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B971" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C971" t="s">
         <v>2961</v>
       </c>
-      <c r="B971" t="s">
+      <c r="D971" t="s">
         <v>2962</v>
-      </c>
-      <c r="C971" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D971" t="s">
-        <v>2964</v>
       </c>
       <c r="E971" t="s">
         <v>16</v>
       </c>
       <c r="F971" t="s">
-        <v>2979</v>
+        <v>2981</v>
       </c>
       <c r="G971" t="s">
-        <v>2980</v>
+        <v>2982</v>
       </c>
       <c r="H971">
         <v>3</v>
       </c>
       <c r="I971" t="s">
-        <v>2981</v>
+        <v>2976</v>
       </c>
       <c r="J971" t="s">
-        <v>2982</v>
+        <v>205</v>
       </c>
       <c r="K971" t="s">
         <v>21</v>
       </c>
       <c r="L971" t="s">
-        <v>2250</v>
+        <v>205</v>
       </c>
       <c r="M971" t="s">
-        <v>23</v>
+        <v>640</v>
       </c>
     </row>
     <row r="972" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A972" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B972" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C972" t="s">
         <v>2961</v>
       </c>
-      <c r="B972" t="s">
+      <c r="D972" t="s">
         <v>2962</v>
-      </c>
-      <c r="C972" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D972" t="s">
-        <v>2964</v>
       </c>
       <c r="E972" t="s">
         <v>16</v>
       </c>
       <c r="F972" t="s">
-        <v>2983</v>
+        <v>2981</v>
       </c>
       <c r="G972" t="s">
-        <v>2984</v>
+        <v>2982</v>
       </c>
       <c r="H972">
         <v>3</v>
       </c>
       <c r="I972" t="s">
-        <v>219</v>
+        <v>2972</v>
       </c>
       <c r="J972" t="s">
         <v>205</v>
@@ -49761,36 +49755,36 @@
         <v>205</v>
       </c>
       <c r="M972" t="s">
-        <v>23</v>
+        <v>643</v>
       </c>
     </row>
     <row r="973" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A973" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B973" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C973" t="s">
         <v>2961</v>
       </c>
-      <c r="B973" t="s">
+      <c r="D973" t="s">
         <v>2962</v>
-      </c>
-      <c r="C973" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D973" t="s">
-        <v>2964</v>
       </c>
       <c r="E973" t="s">
         <v>16</v>
       </c>
       <c r="F973" t="s">
-        <v>2983</v>
+        <v>2981</v>
       </c>
       <c r="G973" t="s">
-        <v>2984</v>
+        <v>2982</v>
       </c>
       <c r="H973">
         <v>3</v>
       </c>
       <c r="I973" t="s">
-        <v>2978</v>
+        <v>213</v>
       </c>
       <c r="J973" t="s">
         <v>205</v>
@@ -49802,36 +49796,36 @@
         <v>205</v>
       </c>
       <c r="M973" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="974" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A974" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B974" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C974" t="s">
         <v>2961</v>
       </c>
-      <c r="B974" t="s">
+      <c r="D974" t="s">
         <v>2962</v>
-      </c>
-      <c r="C974" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D974" t="s">
-        <v>2964</v>
       </c>
       <c r="E974" t="s">
         <v>16</v>
       </c>
       <c r="F974" t="s">
-        <v>2983</v>
+        <v>2981</v>
       </c>
       <c r="G974" t="s">
-        <v>2984</v>
+        <v>2982</v>
       </c>
       <c r="H974">
         <v>3</v>
       </c>
       <c r="I974" t="s">
-        <v>2974</v>
+        <v>216</v>
       </c>
       <c r="J974" t="s">
         <v>205</v>
@@ -49843,21 +49837,21 @@
         <v>205</v>
       </c>
       <c r="M974" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="975" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A975" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B975" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C975" t="s">
         <v>2961</v>
       </c>
-      <c r="B975" t="s">
+      <c r="D975" t="s">
         <v>2962</v>
-      </c>
-      <c r="C975" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D975" t="s">
-        <v>2964</v>
       </c>
       <c r="E975" t="s">
         <v>16</v>
@@ -49884,21 +49878,21 @@
         <v>205</v>
       </c>
       <c r="M975" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
     </row>
     <row r="976" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A976" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B976" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C976" t="s">
         <v>2961</v>
       </c>
-      <c r="B976" t="s">
+      <c r="D976" t="s">
         <v>2962</v>
-      </c>
-      <c r="C976" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D976" t="s">
-        <v>2964</v>
       </c>
       <c r="E976" t="s">
         <v>16</v>
@@ -49913,7 +49907,7 @@
         <v>3</v>
       </c>
       <c r="I976" t="s">
-        <v>216</v>
+        <v>2972</v>
       </c>
       <c r="J976" t="s">
         <v>205</v>
@@ -49925,36 +49919,36 @@
         <v>205</v>
       </c>
       <c r="M976" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="977" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A977" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B977" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C977" t="s">
         <v>2961</v>
       </c>
-      <c r="B977" t="s">
+      <c r="D977" t="s">
         <v>2962</v>
-      </c>
-      <c r="C977" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D977" t="s">
-        <v>2964</v>
       </c>
       <c r="E977" t="s">
         <v>16</v>
       </c>
       <c r="F977" t="s">
-        <v>2985</v>
+        <v>2983</v>
       </c>
       <c r="G977" t="s">
-        <v>2986</v>
+        <v>2984</v>
       </c>
       <c r="H977">
         <v>3</v>
       </c>
       <c r="I977" t="s">
-        <v>213</v>
+        <v>2976</v>
       </c>
       <c r="J977" t="s">
         <v>205</v>
@@ -49966,36 +49960,36 @@
         <v>205</v>
       </c>
       <c r="M977" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="978" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A978" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B978" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C978" t="s">
         <v>2961</v>
       </c>
-      <c r="B978" t="s">
+      <c r="D978" t="s">
         <v>2962</v>
-      </c>
-      <c r="C978" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D978" t="s">
-        <v>2964</v>
       </c>
       <c r="E978" t="s">
         <v>16</v>
       </c>
       <c r="F978" t="s">
-        <v>2985</v>
+        <v>2983</v>
       </c>
       <c r="G978" t="s">
-        <v>2986</v>
+        <v>2984</v>
       </c>
       <c r="H978">
         <v>3</v>
       </c>
       <c r="I978" t="s">
-        <v>2974</v>
+        <v>219</v>
       </c>
       <c r="J978" t="s">
         <v>205</v>
@@ -50007,21 +50001,21 @@
         <v>205</v>
       </c>
       <c r="M978" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="979" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A979" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B979" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C979" t="s">
         <v>2961</v>
       </c>
-      <c r="B979" t="s">
+      <c r="D979" t="s">
         <v>2962</v>
-      </c>
-      <c r="C979" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D979" t="s">
-        <v>2964</v>
       </c>
       <c r="E979" t="s">
         <v>16</v>
@@ -50036,98 +50030,98 @@
         <v>3</v>
       </c>
       <c r="I979" t="s">
-        <v>2978</v>
+        <v>219</v>
       </c>
       <c r="J979" t="s">
-        <v>205</v>
+        <v>2987</v>
       </c>
       <c r="K979" t="s">
         <v>21</v>
       </c>
       <c r="L979" t="s">
-        <v>205</v>
+        <v>2250</v>
       </c>
       <c r="M979" t="s">
-        <v>646</v>
+        <v>23</v>
       </c>
     </row>
     <row r="980" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A980" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B980" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C980" t="s">
         <v>2961</v>
       </c>
-      <c r="B980" t="s">
+      <c r="D980" t="s">
         <v>2962</v>
-      </c>
-      <c r="C980" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D980" t="s">
-        <v>2964</v>
       </c>
       <c r="E980" t="s">
         <v>16</v>
       </c>
       <c r="F980" t="s">
-        <v>2985</v>
+        <v>2988</v>
       </c>
       <c r="G980" t="s">
-        <v>2986</v>
+        <v>2989</v>
       </c>
       <c r="H980">
         <v>3</v>
       </c>
       <c r="I980" t="s">
-        <v>219</v>
+        <v>2976</v>
       </c>
       <c r="J980" t="s">
-        <v>205</v>
+        <v>2990</v>
       </c>
       <c r="K980" t="s">
         <v>21</v>
       </c>
       <c r="L980" t="s">
-        <v>205</v>
+        <v>2966</v>
       </c>
       <c r="M980" t="s">
-        <v>648</v>
+        <v>23</v>
       </c>
     </row>
     <row r="981" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A981" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B981" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C981" t="s">
         <v>2961</v>
       </c>
-      <c r="B981" t="s">
+      <c r="D981" t="s">
         <v>2962</v>
-      </c>
-      <c r="C981" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D981" t="s">
-        <v>2964</v>
       </c>
       <c r="E981" t="s">
         <v>16</v>
       </c>
       <c r="F981" t="s">
-        <v>2987</v>
+        <v>2991</v>
       </c>
       <c r="G981" t="s">
-        <v>2988</v>
+        <v>2992</v>
       </c>
       <c r="H981">
         <v>3</v>
       </c>
       <c r="I981" t="s">
-        <v>219</v>
+        <v>2972</v>
       </c>
       <c r="J981" t="s">
-        <v>2989</v>
+        <v>2990</v>
       </c>
       <c r="K981" t="s">
         <v>21</v>
       </c>
       <c r="L981" t="s">
-        <v>2250</v>
+        <v>2993</v>
       </c>
       <c r="M981" t="s">
         <v>23</v>
@@ -50135,40 +50129,40 @@
     </row>
     <row r="982" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A982" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B982" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C982" t="s">
         <v>2961</v>
       </c>
-      <c r="B982" t="s">
+      <c r="D982" t="s">
         <v>2962</v>
-      </c>
-      <c r="C982" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D982" t="s">
-        <v>2964</v>
       </c>
       <c r="E982" t="s">
         <v>16</v>
       </c>
       <c r="F982" t="s">
-        <v>2990</v>
+        <v>2994</v>
       </c>
       <c r="G982" t="s">
-        <v>2991</v>
+        <v>2995</v>
       </c>
       <c r="H982">
         <v>3</v>
       </c>
       <c r="I982" t="s">
-        <v>2978</v>
+        <v>213</v>
       </c>
       <c r="J982" t="s">
-        <v>2992</v>
+        <v>2996</v>
       </c>
       <c r="K982" t="s">
         <v>21</v>
       </c>
       <c r="L982" t="s">
-        <v>2968</v>
+        <v>2993</v>
       </c>
       <c r="M982" t="s">
         <v>23</v>
@@ -50176,40 +50170,40 @@
     </row>
     <row r="983" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A983" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B983" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C983" t="s">
         <v>2961</v>
       </c>
-      <c r="B983" t="s">
+      <c r="D983" t="s">
         <v>2962</v>
-      </c>
-      <c r="C983" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D983" t="s">
-        <v>2964</v>
       </c>
       <c r="E983" t="s">
         <v>16</v>
       </c>
       <c r="F983" t="s">
-        <v>2993</v>
+        <v>2997</v>
       </c>
       <c r="G983" t="s">
-        <v>2994</v>
+        <v>2998</v>
       </c>
       <c r="H983">
         <v>3</v>
       </c>
       <c r="I983" t="s">
-        <v>2974</v>
+        <v>216</v>
       </c>
       <c r="J983" t="s">
-        <v>2992</v>
+        <v>2973</v>
       </c>
       <c r="K983" t="s">
         <v>21</v>
       </c>
       <c r="L983" t="s">
-        <v>2995</v>
+        <v>2150</v>
       </c>
       <c r="M983" t="s">
         <v>23</v>
@@ -50217,40 +50211,40 @@
     </row>
     <row r="984" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A984" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B984" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C984" t="s">
         <v>2961</v>
       </c>
-      <c r="B984" t="s">
+      <c r="D984" t="s">
         <v>2962</v>
-      </c>
-      <c r="C984" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D984" t="s">
-        <v>2964</v>
       </c>
       <c r="E984" t="s">
         <v>16</v>
       </c>
       <c r="F984" t="s">
-        <v>2996</v>
+        <v>2999</v>
       </c>
       <c r="G984" t="s">
-        <v>2997</v>
+        <v>3000</v>
       </c>
       <c r="H984">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I984" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="J984" t="s">
-        <v>2998</v>
+        <v>205</v>
       </c>
       <c r="K984" t="s">
         <v>21</v>
       </c>
       <c r="L984" t="s">
-        <v>2995</v>
+        <v>205</v>
       </c>
       <c r="M984" t="s">
         <v>23</v>
@@ -50258,40 +50252,40 @@
     </row>
     <row r="985" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A985" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B985" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C985" t="s">
         <v>2961</v>
       </c>
-      <c r="B985" t="s">
+      <c r="D985" t="s">
         <v>2962</v>
-      </c>
-      <c r="C985" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D985" t="s">
-        <v>2964</v>
       </c>
       <c r="E985" t="s">
         <v>16</v>
       </c>
       <c r="F985" t="s">
-        <v>2999</v>
+        <v>3001</v>
       </c>
       <c r="G985" t="s">
-        <v>3000</v>
+        <v>3002</v>
       </c>
       <c r="H985">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I985" t="s">
-        <v>216</v>
+        <v>3003</v>
       </c>
       <c r="J985" t="s">
-        <v>2975</v>
+        <v>205</v>
       </c>
       <c r="K985" t="s">
         <v>21</v>
       </c>
       <c r="L985" t="s">
-        <v>2150</v>
+        <v>205</v>
       </c>
       <c r="M985" t="s">
         <v>23</v>
@@ -50299,40 +50293,40 @@
     </row>
     <row r="986" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A986" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B986" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C986" t="s">
         <v>2961</v>
       </c>
-      <c r="B986" t="s">
+      <c r="D986" t="s">
         <v>2962</v>
-      </c>
-      <c r="C986" t="s">
-        <v>2963</v>
-      </c>
-      <c r="D986" t="s">
-        <v>2964</v>
       </c>
       <c r="E986" t="s">
         <v>16</v>
       </c>
       <c r="F986" t="s">
-        <v>3001</v>
+        <v>3004</v>
       </c>
       <c r="G986" t="s">
-        <v>3002</v>
+        <v>3005</v>
       </c>
       <c r="H986">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I986" t="s">
-        <v>205</v>
+        <v>3006</v>
       </c>
       <c r="J986" t="s">
-        <v>205</v>
+        <v>2987</v>
       </c>
       <c r="K986" t="s">
         <v>21</v>
       </c>
       <c r="L986" t="s">
-        <v>205</v>
+        <v>2150</v>
       </c>
       <c r="M986" t="s">
         <v>23</v>
@@ -50340,40 +50334,40 @@
     </row>
     <row r="987" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A987" t="s">
-        <v>2961</v>
+        <v>2959</v>
       </c>
       <c r="B987" t="s">
-        <v>2962</v>
+        <v>2960</v>
       </c>
       <c r="C987" t="s">
-        <v>2963</v>
+        <v>3007</v>
       </c>
       <c r="D987" t="s">
-        <v>2964</v>
+        <v>3008</v>
       </c>
       <c r="E987" t="s">
-        <v>16</v>
+        <v>2274</v>
       </c>
       <c r="F987" t="s">
-        <v>3003</v>
+        <v>3009</v>
       </c>
       <c r="G987" t="s">
-        <v>3004</v>
+        <v>2975</v>
       </c>
       <c r="H987">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I987" t="s">
-        <v>3005</v>
+        <v>3010</v>
       </c>
       <c r="J987" t="s">
-        <v>205</v>
+        <v>94</v>
       </c>
       <c r="K987" t="s">
         <v>21</v>
       </c>
       <c r="L987" t="s">
-        <v>205</v>
+        <v>2250</v>
       </c>
       <c r="M987" t="s">
         <v>23</v>
@@ -50381,40 +50375,40 @@
     </row>
     <row r="988" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A988" t="s">
-        <v>2961</v>
+        <v>2959</v>
       </c>
       <c r="B988" t="s">
-        <v>2962</v>
+        <v>2960</v>
       </c>
       <c r="C988" t="s">
-        <v>2963</v>
+        <v>3007</v>
       </c>
       <c r="D988" t="s">
-        <v>2964</v>
+        <v>3008</v>
       </c>
       <c r="E988" t="s">
         <v>16</v>
       </c>
       <c r="F988" t="s">
-        <v>3006</v>
+        <v>3011</v>
       </c>
       <c r="G988" t="s">
-        <v>3007</v>
+        <v>3012</v>
       </c>
       <c r="H988">
         <v>3</v>
       </c>
       <c r="I988" t="s">
-        <v>3008</v>
+        <v>3013</v>
       </c>
       <c r="J988" t="s">
-        <v>2989</v>
+        <v>90</v>
       </c>
       <c r="K988" t="s">
         <v>21</v>
       </c>
       <c r="L988" t="s">
-        <v>2150</v>
+        <v>2250</v>
       </c>
       <c r="M988" t="s">
         <v>23</v>
@@ -50422,34 +50416,34 @@
     </row>
     <row r="989" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A989" t="s">
-        <v>2961</v>
+        <v>2959</v>
       </c>
       <c r="B989" t="s">
-        <v>2962</v>
+        <v>2960</v>
       </c>
       <c r="C989" t="s">
-        <v>3009</v>
+        <v>3007</v>
       </c>
       <c r="D989" t="s">
-        <v>3010</v>
+        <v>3008</v>
       </c>
       <c r="E989" t="s">
-        <v>2274</v>
+        <v>16</v>
       </c>
       <c r="F989" t="s">
-        <v>3011</v>
+        <v>3014</v>
       </c>
       <c r="G989" t="s">
-        <v>2977</v>
+        <v>3015</v>
       </c>
       <c r="H989">
         <v>3</v>
       </c>
       <c r="I989" t="s">
-        <v>3012</v>
+        <v>216</v>
       </c>
       <c r="J989" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="K989" t="s">
         <v>21</v>
@@ -50463,40 +50457,40 @@
     </row>
     <row r="990" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A990" t="s">
-        <v>2961</v>
+        <v>3016</v>
       </c>
       <c r="B990" t="s">
-        <v>2962</v>
+        <v>3017</v>
       </c>
       <c r="C990" t="s">
-        <v>3009</v>
+        <v>3016</v>
       </c>
       <c r="D990" t="s">
-        <v>3010</v>
+        <v>15</v>
       </c>
       <c r="E990" t="s">
         <v>16</v>
       </c>
       <c r="F990" t="s">
-        <v>3013</v>
+        <v>3018</v>
       </c>
       <c r="G990" t="s">
-        <v>3014</v>
+        <v>3019</v>
       </c>
       <c r="H990">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I990" t="s">
-        <v>3015</v>
+        <v>3020</v>
       </c>
       <c r="J990" t="s">
-        <v>90</v>
+        <v>2571</v>
       </c>
       <c r="K990" t="s">
         <v>21</v>
       </c>
       <c r="L990" t="s">
-        <v>2250</v>
+        <v>3021</v>
       </c>
       <c r="M990" t="s">
         <v>23</v>
@@ -50504,40 +50498,40 @@
     </row>
     <row r="991" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A991" t="s">
-        <v>2961</v>
+        <v>3016</v>
       </c>
       <c r="B991" t="s">
-        <v>2962</v>
+        <v>3017</v>
       </c>
       <c r="C991" t="s">
-        <v>3009</v>
+        <v>3016</v>
       </c>
       <c r="D991" t="s">
-        <v>3010</v>
+        <v>15</v>
       </c>
       <c r="E991" t="s">
         <v>16</v>
       </c>
       <c r="F991" t="s">
-        <v>3016</v>
+        <v>3022</v>
       </c>
       <c r="G991" t="s">
-        <v>3017</v>
+        <v>3023</v>
       </c>
       <c r="H991">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I991" t="s">
-        <v>216</v>
+        <v>3024</v>
       </c>
       <c r="J991" t="s">
-        <v>99</v>
+        <v>2389</v>
       </c>
       <c r="K991" t="s">
         <v>21</v>
       </c>
       <c r="L991" t="s">
-        <v>2250</v>
+        <v>3021</v>
       </c>
       <c r="M991" t="s">
         <v>23</v>
@@ -50545,13 +50539,13 @@
     </row>
     <row r="992" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A992" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B992" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C992" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D992" t="s">
         <v>15</v>
@@ -50560,16 +50554,16 @@
         <v>16</v>
       </c>
       <c r="F992" t="s">
-        <v>3020</v>
+        <v>3025</v>
       </c>
       <c r="G992" t="s">
-        <v>3021</v>
+        <v>3026</v>
       </c>
       <c r="H992">
         <v>2</v>
       </c>
       <c r="I992" t="s">
-        <v>3022</v>
+        <v>35</v>
       </c>
       <c r="J992" t="s">
         <v>2571</v>
@@ -50578,7 +50572,7 @@
         <v>21</v>
       </c>
       <c r="L992" t="s">
-        <v>3023</v>
+        <v>3027</v>
       </c>
       <c r="M992" t="s">
         <v>23</v>
@@ -50586,13 +50580,13 @@
     </row>
     <row r="993" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A993" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B993" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C993" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D993" t="s">
         <v>15</v>
@@ -50601,16 +50595,16 @@
         <v>16</v>
       </c>
       <c r="F993" t="s">
-        <v>3024</v>
+        <v>3028</v>
       </c>
       <c r="G993" t="s">
-        <v>3025</v>
+        <v>3029</v>
       </c>
       <c r="H993">
         <v>2</v>
       </c>
       <c r="I993" t="s">
-        <v>3026</v>
+        <v>1357</v>
       </c>
       <c r="J993" t="s">
         <v>2389</v>
@@ -50619,7 +50613,7 @@
         <v>21</v>
       </c>
       <c r="L993" t="s">
-        <v>3023</v>
+        <v>3030</v>
       </c>
       <c r="M993" t="s">
         <v>23</v>
@@ -50627,13 +50621,13 @@
     </row>
     <row r="994" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A994" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B994" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C994" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D994" t="s">
         <v>15</v>
@@ -50642,39 +50636,39 @@
         <v>16</v>
       </c>
       <c r="F994" t="s">
-        <v>3027</v>
+        <v>3028</v>
       </c>
       <c r="G994" t="s">
-        <v>3028</v>
+        <v>3029</v>
       </c>
       <c r="H994">
         <v>2</v>
       </c>
       <c r="I994" t="s">
-        <v>35</v>
+        <v>1827</v>
       </c>
       <c r="J994" t="s">
-        <v>2571</v>
+        <v>2397</v>
       </c>
       <c r="K994" t="s">
         <v>21</v>
       </c>
       <c r="L994" t="s">
-        <v>3029</v>
+        <v>37</v>
       </c>
       <c r="M994" t="s">
-        <v>23</v>
+        <v>640</v>
       </c>
     </row>
     <row r="995" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A995" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B995" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C995" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D995" t="s">
         <v>15</v>
@@ -50683,39 +50677,39 @@
         <v>16</v>
       </c>
       <c r="F995" t="s">
-        <v>3030</v>
+        <v>3028</v>
       </c>
       <c r="G995" t="s">
-        <v>3031</v>
+        <v>3029</v>
       </c>
       <c r="H995">
         <v>2</v>
       </c>
       <c r="I995" t="s">
-        <v>1357</v>
+        <v>3031</v>
       </c>
       <c r="J995" t="s">
-        <v>2389</v>
+        <v>2397</v>
       </c>
       <c r="K995" t="s">
         <v>21</v>
       </c>
       <c r="L995" t="s">
-        <v>3032</v>
+        <v>37</v>
       </c>
       <c r="M995" t="s">
-        <v>23</v>
+        <v>643</v>
       </c>
     </row>
     <row r="996" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A996" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B996" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C996" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D996" t="s">
         <v>15</v>
@@ -50724,39 +50718,39 @@
         <v>16</v>
       </c>
       <c r="F996" t="s">
-        <v>3030</v>
+        <v>3028</v>
       </c>
       <c r="G996" t="s">
-        <v>3031</v>
+        <v>3029</v>
       </c>
       <c r="H996">
         <v>2</v>
       </c>
       <c r="I996" t="s">
-        <v>1827</v>
+        <v>3032</v>
       </c>
       <c r="J996" t="s">
-        <v>2397</v>
+        <v>2389</v>
       </c>
       <c r="K996" t="s">
         <v>21</v>
       </c>
       <c r="L996" t="s">
-        <v>37</v>
+        <v>3030</v>
       </c>
       <c r="M996" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="997" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A997" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B997" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C997" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D997" t="s">
         <v>15</v>
@@ -50765,10 +50759,10 @@
         <v>16</v>
       </c>
       <c r="F997" t="s">
-        <v>3030</v>
+        <v>3028</v>
       </c>
       <c r="G997" t="s">
-        <v>3031</v>
+        <v>3029</v>
       </c>
       <c r="H997">
         <v>2</v>
@@ -50777,27 +50771,27 @@
         <v>3033</v>
       </c>
       <c r="J997" t="s">
-        <v>2397</v>
+        <v>664</v>
       </c>
       <c r="K997" t="s">
         <v>21</v>
       </c>
       <c r="L997" t="s">
-        <v>37</v>
+        <v>3030</v>
       </c>
       <c r="M997" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="998" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A998" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B998" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C998" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D998" t="s">
         <v>15</v>
@@ -50806,10 +50800,10 @@
         <v>16</v>
       </c>
       <c r="F998" t="s">
-        <v>3030</v>
+        <v>3028</v>
       </c>
       <c r="G998" t="s">
-        <v>3031</v>
+        <v>3029</v>
       </c>
       <c r="H998">
         <v>2</v>
@@ -50818,27 +50812,27 @@
         <v>3034</v>
       </c>
       <c r="J998" t="s">
-        <v>2389</v>
+        <v>3035</v>
       </c>
       <c r="K998" t="s">
         <v>21</v>
       </c>
       <c r="L998" t="s">
-        <v>3032</v>
+        <v>3030</v>
       </c>
       <c r="M998" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
     </row>
     <row r="999" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A999" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B999" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C999" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D999" t="s">
         <v>15</v>
@@ -50847,39 +50841,39 @@
         <v>16</v>
       </c>
       <c r="F999" t="s">
-        <v>3030</v>
+        <v>3036</v>
       </c>
       <c r="G999" t="s">
-        <v>3031</v>
+        <v>3037</v>
       </c>
       <c r="H999">
         <v>2</v>
       </c>
       <c r="I999" t="s">
-        <v>3035</v>
+        <v>3032</v>
       </c>
       <c r="J999" t="s">
-        <v>664</v>
+        <v>2548</v>
       </c>
       <c r="K999" t="s">
         <v>21</v>
       </c>
       <c r="L999" t="s">
-        <v>3032</v>
+        <v>3030</v>
       </c>
       <c r="M999" t="s">
-        <v>648</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1000" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1000" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1000" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1000" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="D1000" t="s">
         <v>15</v>
@@ -50888,66 +50882,66 @@
         <v>16</v>
       </c>
       <c r="F1000" t="s">
-        <v>3030</v>
+        <v>3038</v>
       </c>
       <c r="G1000" t="s">
-        <v>3031</v>
+        <v>3039</v>
       </c>
       <c r="H1000">
         <v>2</v>
       </c>
       <c r="I1000" t="s">
-        <v>3036</v>
+        <v>3033</v>
       </c>
       <c r="J1000" t="s">
-        <v>3037</v>
+        <v>3040</v>
       </c>
       <c r="K1000" t="s">
         <v>21</v>
       </c>
       <c r="L1000" t="s">
-        <v>3032</v>
+        <v>3030</v>
       </c>
       <c r="M1000" t="s">
-        <v>651</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1001" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1001" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1001" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1001" t="s">
-        <v>3018</v>
+        <v>3041</v>
       </c>
       <c r="D1001" t="s">
-        <v>15</v>
+        <v>3042</v>
       </c>
       <c r="E1001" t="s">
         <v>16</v>
       </c>
       <c r="F1001" t="s">
-        <v>3038</v>
+        <v>3043</v>
       </c>
       <c r="G1001" t="s">
-        <v>3039</v>
+        <v>3044</v>
       </c>
       <c r="H1001">
         <v>2</v>
       </c>
       <c r="I1001" t="s">
-        <v>3034</v>
+        <v>3032</v>
       </c>
       <c r="J1001" t="s">
-        <v>2548</v>
+        <v>2571</v>
       </c>
       <c r="K1001" t="s">
         <v>21</v>
       </c>
       <c r="L1001" t="s">
-        <v>3032</v>
+        <v>3030</v>
       </c>
       <c r="M1001" t="s">
         <v>23</v>
@@ -50955,40 +50949,40 @@
     </row>
     <row r="1002" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1002" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1002" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1002" t="s">
-        <v>3018</v>
+        <v>3041</v>
       </c>
       <c r="D1002" t="s">
-        <v>15</v>
+        <v>3042</v>
       </c>
       <c r="E1002" t="s">
         <v>16</v>
       </c>
       <c r="F1002" t="s">
-        <v>3040</v>
+        <v>3045</v>
       </c>
       <c r="G1002" t="s">
-        <v>3041</v>
+        <v>3046</v>
       </c>
       <c r="H1002">
         <v>2</v>
       </c>
       <c r="I1002" t="s">
-        <v>3035</v>
+        <v>3047</v>
       </c>
       <c r="J1002" t="s">
-        <v>3042</v>
+        <v>2397</v>
       </c>
       <c r="K1002" t="s">
         <v>21</v>
       </c>
       <c r="L1002" t="s">
-        <v>3032</v>
+        <v>2739</v>
       </c>
       <c r="M1002" t="s">
         <v>23</v>
@@ -50996,40 +50990,40 @@
     </row>
     <row r="1003" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1003" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1003" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1003" t="s">
-        <v>3043</v>
+        <v>3041</v>
       </c>
       <c r="D1003" t="s">
-        <v>3044</v>
+        <v>3042</v>
       </c>
       <c r="E1003" t="s">
         <v>16</v>
       </c>
       <c r="F1003" t="s">
-        <v>3045</v>
+        <v>3048</v>
       </c>
       <c r="G1003" t="s">
-        <v>3046</v>
+        <v>3049</v>
       </c>
       <c r="H1003">
         <v>2</v>
       </c>
       <c r="I1003" t="s">
-        <v>3034</v>
+        <v>3050</v>
       </c>
       <c r="J1003" t="s">
-        <v>2571</v>
+        <v>2548</v>
       </c>
       <c r="K1003" t="s">
         <v>21</v>
       </c>
       <c r="L1003" t="s">
-        <v>3032</v>
+        <v>3021</v>
       </c>
       <c r="M1003" t="s">
         <v>23</v>
@@ -51037,34 +51031,34 @@
     </row>
     <row r="1004" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1004" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1004" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1004" t="s">
-        <v>3043</v>
+        <v>3041</v>
       </c>
       <c r="D1004" t="s">
-        <v>3044</v>
+        <v>3042</v>
       </c>
       <c r="E1004" t="s">
         <v>16</v>
       </c>
       <c r="F1004" t="s">
-        <v>3047</v>
+        <v>3051</v>
       </c>
       <c r="G1004" t="s">
-        <v>3048</v>
+        <v>3052</v>
       </c>
       <c r="H1004">
         <v>2</v>
       </c>
       <c r="I1004" t="s">
-        <v>3049</v>
+        <v>3053</v>
       </c>
       <c r="J1004" t="s">
-        <v>2397</v>
+        <v>2571</v>
       </c>
       <c r="K1004" t="s">
         <v>21</v>
@@ -51078,40 +51072,40 @@
     </row>
     <row r="1005" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1005" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1005" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1005" t="s">
-        <v>3043</v>
+        <v>3041</v>
       </c>
       <c r="D1005" t="s">
-        <v>3044</v>
+        <v>3042</v>
       </c>
       <c r="E1005" t="s">
         <v>16</v>
       </c>
       <c r="F1005" t="s">
-        <v>3050</v>
+        <v>3054</v>
       </c>
       <c r="G1005" t="s">
-        <v>3051</v>
+        <v>3055</v>
       </c>
       <c r="H1005">
         <v>2</v>
       </c>
       <c r="I1005" t="s">
-        <v>3052</v>
+        <v>3056</v>
       </c>
       <c r="J1005" t="s">
-        <v>2548</v>
+        <v>2397</v>
       </c>
       <c r="K1005" t="s">
         <v>21</v>
       </c>
       <c r="L1005" t="s">
-        <v>3023</v>
+        <v>2661</v>
       </c>
       <c r="M1005" t="s">
         <v>23</v>
@@ -51119,31 +51113,31 @@
     </row>
     <row r="1006" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1006" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1006" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1006" t="s">
-        <v>3043</v>
+        <v>3057</v>
       </c>
       <c r="D1006" t="s">
-        <v>3044</v>
+        <v>3058</v>
       </c>
       <c r="E1006" t="s">
         <v>16</v>
       </c>
       <c r="F1006" t="s">
-        <v>3053</v>
+        <v>3059</v>
       </c>
       <c r="G1006" t="s">
-        <v>3054</v>
+        <v>3060</v>
       </c>
       <c r="H1006">
         <v>2</v>
       </c>
       <c r="I1006" t="s">
-        <v>3055</v>
+        <v>3061</v>
       </c>
       <c r="J1006" t="s">
         <v>2571</v>
@@ -51152,7 +51146,7 @@
         <v>21</v>
       </c>
       <c r="L1006" t="s">
-        <v>2739</v>
+        <v>37</v>
       </c>
       <c r="M1006" t="s">
         <v>23</v>
@@ -51160,31 +51154,31 @@
     </row>
     <row r="1007" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1007" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1007" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1007" t="s">
-        <v>3043</v>
+        <v>3057</v>
       </c>
       <c r="D1007" t="s">
-        <v>3044</v>
+        <v>3058</v>
       </c>
       <c r="E1007" t="s">
         <v>16</v>
       </c>
       <c r="F1007" t="s">
-        <v>3056</v>
+        <v>3062</v>
       </c>
       <c r="G1007" t="s">
-        <v>3057</v>
+        <v>3063</v>
       </c>
       <c r="H1007">
         <v>2</v>
       </c>
       <c r="I1007" t="s">
-        <v>3058</v>
+        <v>3024</v>
       </c>
       <c r="J1007" t="s">
         <v>2397</v>
@@ -51193,7 +51187,7 @@
         <v>21</v>
       </c>
       <c r="L1007" t="s">
-        <v>2661</v>
+        <v>3021</v>
       </c>
       <c r="M1007" t="s">
         <v>23</v>
@@ -51201,31 +51195,31 @@
     </row>
     <row r="1008" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1008" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1008" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1008" t="s">
-        <v>3059</v>
+        <v>3057</v>
       </c>
       <c r="D1008" t="s">
-        <v>3060</v>
+        <v>3058</v>
       </c>
       <c r="E1008" t="s">
         <v>16</v>
       </c>
       <c r="F1008" t="s">
-        <v>3061</v>
+        <v>3064</v>
       </c>
       <c r="G1008" t="s">
-        <v>3062</v>
+        <v>3065</v>
       </c>
       <c r="H1008">
         <v>2</v>
       </c>
       <c r="I1008" t="s">
-        <v>3063</v>
+        <v>3066</v>
       </c>
       <c r="J1008" t="s">
         <v>2571</v>
@@ -51234,7 +51228,7 @@
         <v>21</v>
       </c>
       <c r="L1008" t="s">
-        <v>37</v>
+        <v>2661</v>
       </c>
       <c r="M1008" t="s">
         <v>23</v>
@@ -51242,40 +51236,40 @@
     </row>
     <row r="1009" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1009" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1009" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1009" t="s">
-        <v>3059</v>
+        <v>3057</v>
       </c>
       <c r="D1009" t="s">
-        <v>3060</v>
+        <v>3058</v>
       </c>
       <c r="E1009" t="s">
         <v>16</v>
       </c>
       <c r="F1009" t="s">
-        <v>3064</v>
+        <v>3067</v>
       </c>
       <c r="G1009" t="s">
-        <v>3065</v>
+        <v>3068</v>
       </c>
       <c r="H1009">
         <v>2</v>
       </c>
       <c r="I1009" t="s">
-        <v>3026</v>
+        <v>35</v>
       </c>
       <c r="J1009" t="s">
-        <v>2397</v>
+        <v>2548</v>
       </c>
       <c r="K1009" t="s">
         <v>21</v>
       </c>
       <c r="L1009" t="s">
-        <v>3023</v>
+        <v>3027</v>
       </c>
       <c r="M1009" t="s">
         <v>23</v>
@@ -51283,40 +51277,40 @@
     </row>
     <row r="1010" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1010" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1010" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1010" t="s">
-        <v>3059</v>
+        <v>3057</v>
       </c>
       <c r="D1010" t="s">
-        <v>3060</v>
+        <v>3058</v>
       </c>
       <c r="E1010" t="s">
         <v>16</v>
       </c>
       <c r="F1010" t="s">
-        <v>3066</v>
+        <v>3069</v>
       </c>
       <c r="G1010" t="s">
-        <v>3067</v>
+        <v>460</v>
       </c>
       <c r="H1010">
         <v>2</v>
       </c>
       <c r="I1010" t="s">
-        <v>3068</v>
+        <v>3070</v>
       </c>
       <c r="J1010" t="s">
-        <v>2571</v>
+        <v>2389</v>
       </c>
       <c r="K1010" t="s">
         <v>21</v>
       </c>
       <c r="L1010" t="s">
-        <v>2661</v>
+        <v>2739</v>
       </c>
       <c r="M1010" t="s">
         <v>23</v>
@@ -51324,40 +51318,40 @@
     </row>
     <row r="1011" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1011" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1011" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1011" t="s">
-        <v>3059</v>
+        <v>3057</v>
       </c>
       <c r="D1011" t="s">
-        <v>3060</v>
+        <v>3058</v>
       </c>
       <c r="E1011" t="s">
         <v>16</v>
       </c>
       <c r="F1011" t="s">
-        <v>3069</v>
+        <v>3071</v>
       </c>
       <c r="G1011" t="s">
-        <v>3070</v>
+        <v>3072</v>
       </c>
       <c r="H1011">
         <v>2</v>
       </c>
       <c r="I1011" t="s">
-        <v>35</v>
+        <v>3032</v>
       </c>
       <c r="J1011" t="s">
-        <v>2548</v>
+        <v>2397</v>
       </c>
       <c r="K1011" t="s">
         <v>21</v>
       </c>
       <c r="L1011" t="s">
-        <v>3029</v>
+        <v>3030</v>
       </c>
       <c r="M1011" t="s">
         <v>23</v>
@@ -51365,40 +51359,40 @@
     </row>
     <row r="1012" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1012" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1012" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1012" t="s">
-        <v>3059</v>
+        <v>3073</v>
       </c>
       <c r="D1012" t="s">
-        <v>3060</v>
+        <v>3074</v>
       </c>
       <c r="E1012" t="s">
         <v>16</v>
       </c>
       <c r="F1012" t="s">
-        <v>3071</v>
+        <v>3075</v>
       </c>
       <c r="G1012" t="s">
-        <v>460</v>
+        <v>3076</v>
       </c>
       <c r="H1012">
         <v>2</v>
       </c>
       <c r="I1012" t="s">
-        <v>3072</v>
+        <v>3066</v>
       </c>
       <c r="J1012" t="s">
-        <v>2389</v>
+        <v>813</v>
       </c>
       <c r="K1012" t="s">
         <v>21</v>
       </c>
       <c r="L1012" t="s">
-        <v>2739</v>
+        <v>3030</v>
       </c>
       <c r="M1012" t="s">
         <v>23</v>
@@ -51406,40 +51400,40 @@
     </row>
     <row r="1013" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1013" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1013" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1013" t="s">
-        <v>3059</v>
+        <v>3073</v>
       </c>
       <c r="D1013" t="s">
-        <v>3060</v>
+        <v>3074</v>
       </c>
       <c r="E1013" t="s">
         <v>16</v>
       </c>
       <c r="F1013" t="s">
-        <v>3073</v>
+        <v>3077</v>
       </c>
       <c r="G1013" t="s">
-        <v>3074</v>
+        <v>3078</v>
       </c>
       <c r="H1013">
         <v>2</v>
       </c>
       <c r="I1013" t="s">
-        <v>3034</v>
+        <v>3079</v>
       </c>
       <c r="J1013" t="s">
-        <v>2397</v>
+        <v>3080</v>
       </c>
       <c r="K1013" t="s">
         <v>21</v>
       </c>
       <c r="L1013" t="s">
-        <v>3032</v>
+        <v>3030</v>
       </c>
       <c r="M1013" t="s">
         <v>23</v>
@@ -51447,40 +51441,40 @@
     </row>
     <row r="1014" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1014" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1014" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1014" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1014" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1014" t="s">
         <v>16</v>
       </c>
       <c r="F1014" t="s">
-        <v>3077</v>
+        <v>3081</v>
       </c>
       <c r="G1014" t="s">
-        <v>3078</v>
+        <v>3082</v>
       </c>
       <c r="H1014">
         <v>2</v>
       </c>
       <c r="I1014" t="s">
-        <v>3068</v>
+        <v>3061</v>
       </c>
       <c r="J1014" t="s">
-        <v>813</v>
+        <v>664</v>
       </c>
       <c r="K1014" t="s">
         <v>21</v>
       </c>
       <c r="L1014" t="s">
-        <v>3032</v>
+        <v>37</v>
       </c>
       <c r="M1014" t="s">
         <v>23</v>
@@ -51488,40 +51482,40 @@
     </row>
     <row r="1015" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1015" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1015" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1015" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1015" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1015" t="s">
         <v>16</v>
       </c>
       <c r="F1015" t="s">
-        <v>3079</v>
+        <v>3083</v>
       </c>
       <c r="G1015" t="s">
-        <v>3080</v>
+        <v>3084</v>
       </c>
       <c r="H1015">
         <v>2</v>
       </c>
       <c r="I1015" t="s">
-        <v>3081</v>
+        <v>3085</v>
       </c>
       <c r="J1015" t="s">
-        <v>3082</v>
+        <v>2548</v>
       </c>
       <c r="K1015" t="s">
         <v>21</v>
       </c>
       <c r="L1015" t="s">
-        <v>3032</v>
+        <v>3086</v>
       </c>
       <c r="M1015" t="s">
         <v>23</v>
@@ -51529,40 +51523,40 @@
     </row>
     <row r="1016" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1016" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1016" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1016" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1016" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1016" t="s">
         <v>16</v>
       </c>
       <c r="F1016" t="s">
-        <v>3083</v>
+        <v>3087</v>
       </c>
       <c r="G1016" t="s">
-        <v>3084</v>
+        <v>3088</v>
       </c>
       <c r="H1016">
         <v>2</v>
       </c>
       <c r="I1016" t="s">
-        <v>3063</v>
+        <v>3079</v>
       </c>
       <c r="J1016" t="s">
-        <v>664</v>
+        <v>2397</v>
       </c>
       <c r="K1016" t="s">
         <v>21</v>
       </c>
       <c r="L1016" t="s">
-        <v>37</v>
+        <v>3086</v>
       </c>
       <c r="M1016" t="s">
         <v>23</v>
@@ -51570,31 +51564,31 @@
     </row>
     <row r="1017" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1017" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1017" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1017" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1017" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1017" t="s">
         <v>16</v>
       </c>
       <c r="F1017" t="s">
-        <v>3085</v>
+        <v>3089</v>
       </c>
       <c r="G1017" t="s">
-        <v>3086</v>
+        <v>3090</v>
       </c>
       <c r="H1017">
         <v>2</v>
       </c>
       <c r="I1017" t="s">
-        <v>3087</v>
+        <v>3034</v>
       </c>
       <c r="J1017" t="s">
         <v>2548</v>
@@ -51603,7 +51597,7 @@
         <v>21</v>
       </c>
       <c r="L1017" t="s">
-        <v>3088</v>
+        <v>37</v>
       </c>
       <c r="M1017" t="s">
         <v>23</v>
@@ -51611,40 +51605,40 @@
     </row>
     <row r="1018" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1018" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1018" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1018" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1018" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1018" t="s">
         <v>16</v>
       </c>
       <c r="F1018" t="s">
-        <v>3089</v>
+        <v>3091</v>
       </c>
       <c r="G1018" t="s">
-        <v>3090</v>
+        <v>3092</v>
       </c>
       <c r="H1018">
         <v>2</v>
       </c>
       <c r="I1018" t="s">
-        <v>3081</v>
+        <v>3093</v>
       </c>
       <c r="J1018" t="s">
-        <v>2397</v>
+        <v>2389</v>
       </c>
       <c r="K1018" t="s">
         <v>21</v>
       </c>
       <c r="L1018" t="s">
-        <v>3088</v>
+        <v>3086</v>
       </c>
       <c r="M1018" t="s">
         <v>23</v>
@@ -51652,34 +51646,34 @@
     </row>
     <row r="1019" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1019" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1019" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1019" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1019" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1019" t="s">
         <v>16</v>
       </c>
       <c r="F1019" t="s">
-        <v>3091</v>
+        <v>3094</v>
       </c>
       <c r="G1019" t="s">
-        <v>3092</v>
+        <v>3095</v>
       </c>
       <c r="H1019">
         <v>2</v>
       </c>
       <c r="I1019" t="s">
-        <v>3036</v>
+        <v>3047</v>
       </c>
       <c r="J1019" t="s">
-        <v>2548</v>
+        <v>2389</v>
       </c>
       <c r="K1019" t="s">
         <v>21</v>
@@ -51693,40 +51687,40 @@
     </row>
     <row r="1020" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1020" t="s">
-        <v>3018</v>
+        <v>3016</v>
       </c>
       <c r="B1020" t="s">
-        <v>3019</v>
+        <v>3017</v>
       </c>
       <c r="C1020" t="s">
-        <v>3075</v>
+        <v>3073</v>
       </c>
       <c r="D1020" t="s">
-        <v>3076</v>
+        <v>3074</v>
       </c>
       <c r="E1020" t="s">
         <v>16</v>
       </c>
       <c r="F1020" t="s">
-        <v>3093</v>
+        <v>3096</v>
       </c>
       <c r="G1020" t="s">
-        <v>3094</v>
+        <v>3097</v>
       </c>
       <c r="H1020">
         <v>2</v>
       </c>
       <c r="I1020" t="s">
-        <v>3095</v>
+        <v>3034</v>
       </c>
       <c r="J1020" t="s">
-        <v>2389</v>
+        <v>2571</v>
       </c>
       <c r="K1020" t="s">
         <v>21</v>
       </c>
       <c r="L1020" t="s">
-        <v>3088</v>
+        <v>3086</v>
       </c>
       <c r="M1020" t="s">
         <v>23</v>
@@ -51734,40 +51728,40 @@
     </row>
     <row r="1021" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1021" t="s">
-        <v>3018</v>
+        <v>3098</v>
       </c>
       <c r="B1021" t="s">
-        <v>3019</v>
+        <v>3099</v>
       </c>
       <c r="C1021" t="s">
-        <v>3075</v>
+        <v>3098</v>
       </c>
       <c r="D1021" t="s">
-        <v>3076</v>
+        <v>15</v>
       </c>
       <c r="E1021" t="s">
-        <v>16</v>
+        <v>1730</v>
       </c>
       <c r="F1021" t="s">
-        <v>3096</v>
+        <v>3100</v>
       </c>
       <c r="G1021" t="s">
-        <v>3097</v>
+        <v>3101</v>
       </c>
       <c r="H1021">
         <v>2</v>
       </c>
       <c r="I1021" t="s">
-        <v>3049</v>
+        <v>3102</v>
       </c>
       <c r="J1021" t="s">
-        <v>2389</v>
+        <v>2397</v>
       </c>
       <c r="K1021" t="s">
         <v>21</v>
       </c>
       <c r="L1021" t="s">
-        <v>37</v>
+        <v>458</v>
       </c>
       <c r="M1021" t="s">
         <v>23</v>
@@ -51775,40 +51769,40 @@
     </row>
     <row r="1022" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1022" t="s">
-        <v>3018</v>
+        <v>3098</v>
       </c>
       <c r="B1022" t="s">
-        <v>3019</v>
+        <v>3099</v>
       </c>
       <c r="C1022" t="s">
-        <v>3075</v>
+        <v>3103</v>
       </c>
       <c r="D1022" t="s">
-        <v>3076</v>
+        <v>3104</v>
       </c>
       <c r="E1022" t="s">
         <v>16</v>
       </c>
       <c r="F1022" t="s">
-        <v>3098</v>
+        <v>3105</v>
       </c>
       <c r="G1022" t="s">
-        <v>3099</v>
+        <v>3106</v>
       </c>
       <c r="H1022">
         <v>2</v>
       </c>
       <c r="I1022" t="s">
-        <v>3036</v>
+        <v>3107</v>
       </c>
       <c r="J1022" t="s">
-        <v>2571</v>
+        <v>3108</v>
       </c>
       <c r="K1022" t="s">
         <v>21</v>
       </c>
       <c r="L1022" t="s">
-        <v>3088</v>
+        <v>411</v>
       </c>
       <c r="M1022" t="s">
         <v>23</v>
@@ -51816,40 +51810,40 @@
     </row>
     <row r="1023" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1023" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1023" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1023" t="s">
-        <v>3100</v>
+        <v>3109</v>
       </c>
       <c r="D1023" t="s">
-        <v>15</v>
+        <v>3110</v>
       </c>
       <c r="E1023" t="s">
-        <v>1730</v>
+        <v>16</v>
       </c>
       <c r="F1023" t="s">
-        <v>3102</v>
+        <v>3111</v>
       </c>
       <c r="G1023" t="s">
-        <v>3103</v>
+        <v>3112</v>
       </c>
       <c r="H1023">
         <v>2</v>
       </c>
       <c r="I1023" t="s">
-        <v>3104</v>
+        <v>2307</v>
       </c>
       <c r="J1023" t="s">
-        <v>2397</v>
+        <v>1901</v>
       </c>
       <c r="K1023" t="s">
         <v>21</v>
       </c>
       <c r="L1023" t="s">
-        <v>458</v>
+        <v>3113</v>
       </c>
       <c r="M1023" t="s">
         <v>23</v>
@@ -51857,34 +51851,34 @@
     </row>
     <row r="1024" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1024" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1024" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1024" t="s">
-        <v>3105</v>
+        <v>3109</v>
       </c>
       <c r="D1024" t="s">
-        <v>3106</v>
+        <v>3110</v>
       </c>
       <c r="E1024" t="s">
         <v>16</v>
       </c>
       <c r="F1024" t="s">
-        <v>3107</v>
+        <v>3114</v>
       </c>
       <c r="G1024" t="s">
-        <v>3108</v>
+        <v>3115</v>
       </c>
       <c r="H1024">
         <v>2</v>
       </c>
       <c r="I1024" t="s">
-        <v>3109</v>
+        <v>3116</v>
       </c>
       <c r="J1024" t="s">
-        <v>3110</v>
+        <v>2389</v>
       </c>
       <c r="K1024" t="s">
         <v>21</v>
@@ -51898,40 +51892,40 @@
     </row>
     <row r="1025" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1025" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1025" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1025" t="s">
-        <v>3111</v>
+        <v>3109</v>
       </c>
       <c r="D1025" t="s">
-        <v>3112</v>
+        <v>3110</v>
       </c>
       <c r="E1025" t="s">
         <v>16</v>
       </c>
       <c r="F1025" t="s">
-        <v>3113</v>
+        <v>3117</v>
       </c>
       <c r="G1025" t="s">
-        <v>3114</v>
+        <v>3118</v>
       </c>
       <c r="H1025">
         <v>2</v>
       </c>
       <c r="I1025" t="s">
-        <v>2307</v>
+        <v>3119</v>
       </c>
       <c r="J1025" t="s">
-        <v>1901</v>
+        <v>3108</v>
       </c>
       <c r="K1025" t="s">
         <v>21</v>
       </c>
       <c r="L1025" t="s">
-        <v>3115</v>
+        <v>458</v>
       </c>
       <c r="M1025" t="s">
         <v>23</v>
@@ -51939,40 +51933,40 @@
     </row>
     <row r="1026" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1026" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1026" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1026" t="s">
-        <v>3111</v>
+        <v>3109</v>
       </c>
       <c r="D1026" t="s">
-        <v>3112</v>
+        <v>3110</v>
       </c>
       <c r="E1026" t="s">
         <v>16</v>
       </c>
       <c r="F1026" t="s">
-        <v>3116</v>
+        <v>3120</v>
       </c>
       <c r="G1026" t="s">
-        <v>3117</v>
+        <v>3121</v>
       </c>
       <c r="H1026">
         <v>2</v>
       </c>
       <c r="I1026" t="s">
-        <v>3118</v>
+        <v>3122</v>
       </c>
       <c r="J1026" t="s">
-        <v>2389</v>
+        <v>1957</v>
       </c>
       <c r="K1026" t="s">
         <v>21</v>
       </c>
       <c r="L1026" t="s">
-        <v>411</v>
+        <v>3123</v>
       </c>
       <c r="M1026" t="s">
         <v>23</v>
@@ -51980,34 +51974,34 @@
     </row>
     <row r="1027" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1027" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1027" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1027" t="s">
-        <v>3111</v>
+        <v>3124</v>
       </c>
       <c r="D1027" t="s">
-        <v>3112</v>
+        <v>3125</v>
       </c>
       <c r="E1027" t="s">
         <v>16</v>
       </c>
       <c r="F1027" t="s">
-        <v>3119</v>
+        <v>3126</v>
       </c>
       <c r="G1027" t="s">
-        <v>3120</v>
+        <v>3127</v>
       </c>
       <c r="H1027">
         <v>2</v>
       </c>
       <c r="I1027" t="s">
-        <v>3121</v>
+        <v>3128</v>
       </c>
       <c r="J1027" t="s">
-        <v>3110</v>
+        <v>3129</v>
       </c>
       <c r="K1027" t="s">
         <v>21</v>
@@ -52021,40 +52015,40 @@
     </row>
     <row r="1028" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1028" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1028" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1028" t="s">
-        <v>3111</v>
+        <v>3124</v>
       </c>
       <c r="D1028" t="s">
-        <v>3112</v>
+        <v>3125</v>
       </c>
       <c r="E1028" t="s">
         <v>16</v>
       </c>
       <c r="F1028" t="s">
-        <v>3122</v>
+        <v>3130</v>
       </c>
       <c r="G1028" t="s">
-        <v>3123</v>
+        <v>3131</v>
       </c>
       <c r="H1028">
         <v>2</v>
       </c>
       <c r="I1028" t="s">
-        <v>3124</v>
+        <v>3128</v>
       </c>
       <c r="J1028" t="s">
-        <v>1957</v>
+        <v>1901</v>
       </c>
       <c r="K1028" t="s">
         <v>21</v>
       </c>
       <c r="L1028" t="s">
-        <v>3125</v>
+        <v>3123</v>
       </c>
       <c r="M1028" t="s">
         <v>23</v>
@@ -52062,40 +52056,40 @@
     </row>
     <row r="1029" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1029" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1029" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1029" t="s">
-        <v>3126</v>
+        <v>3124</v>
       </c>
       <c r="D1029" t="s">
-        <v>3127</v>
+        <v>3125</v>
       </c>
       <c r="E1029" t="s">
         <v>16</v>
       </c>
       <c r="F1029" t="s">
-        <v>3128</v>
+        <v>3132</v>
       </c>
       <c r="G1029" t="s">
-        <v>3129</v>
+        <v>3133</v>
       </c>
       <c r="H1029">
         <v>2</v>
       </c>
       <c r="I1029" t="s">
-        <v>3130</v>
+        <v>3102</v>
       </c>
       <c r="J1029" t="s">
-        <v>3131</v>
+        <v>3134</v>
       </c>
       <c r="K1029" t="s">
         <v>21</v>
       </c>
       <c r="L1029" t="s">
-        <v>458</v>
+        <v>411</v>
       </c>
       <c r="M1029" t="s">
         <v>23</v>
@@ -52103,40 +52097,40 @@
     </row>
     <row r="1030" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1030" t="s">
-        <v>3100</v>
+        <v>3098</v>
       </c>
       <c r="B1030" t="s">
-        <v>3101</v>
+        <v>3099</v>
       </c>
       <c r="C1030" t="s">
-        <v>3126</v>
+        <v>3124</v>
       </c>
       <c r="D1030" t="s">
-        <v>3127</v>
+        <v>3125</v>
       </c>
       <c r="E1030" t="s">
         <v>16</v>
       </c>
       <c r="F1030" t="s">
-        <v>3132</v>
+        <v>3135</v>
       </c>
       <c r="G1030" t="s">
-        <v>3133</v>
+        <v>3136</v>
       </c>
       <c r="H1030">
         <v>2</v>
       </c>
       <c r="I1030" t="s">
-        <v>3130</v>
+        <v>3137</v>
       </c>
       <c r="J1030" t="s">
-        <v>1901</v>
+        <v>2389</v>
       </c>
       <c r="K1030" t="s">
         <v>21</v>
       </c>
       <c r="L1030" t="s">
-        <v>3125</v>
+        <v>458</v>
       </c>
       <c r="M1030" t="s">
         <v>23</v>
@@ -52144,40 +52138,40 @@
     </row>
     <row r="1031" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1031" t="s">
-        <v>3100</v>
+        <v>3138</v>
       </c>
       <c r="B1031" t="s">
-        <v>3101</v>
+        <v>3139</v>
       </c>
       <c r="C1031" t="s">
-        <v>3126</v>
+        <v>3138</v>
       </c>
       <c r="D1031" t="s">
-        <v>3127</v>
+        <v>15</v>
       </c>
       <c r="E1031" t="s">
-        <v>16</v>
+        <v>1730</v>
       </c>
       <c r="F1031" t="s">
-        <v>3134</v>
+        <v>3140</v>
       </c>
       <c r="G1031" t="s">
-        <v>3135</v>
+        <v>3141</v>
       </c>
       <c r="H1031">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I1031" t="s">
-        <v>3104</v>
+        <v>3142</v>
       </c>
       <c r="J1031" t="s">
-        <v>3136</v>
+        <v>1759</v>
       </c>
       <c r="K1031" t="s">
         <v>21</v>
       </c>
       <c r="L1031" t="s">
-        <v>411</v>
+        <v>3143</v>
       </c>
       <c r="M1031" t="s">
         <v>23</v>
@@ -52185,40 +52179,40 @@
     </row>
     <row r="1032" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1032" t="s">
-        <v>3100</v>
+        <v>3138</v>
       </c>
       <c r="B1032" t="s">
-        <v>3101</v>
+        <v>3139</v>
       </c>
       <c r="C1032" t="s">
-        <v>3126</v>
+        <v>3138</v>
       </c>
       <c r="D1032" t="s">
-        <v>3127</v>
+        <v>15</v>
       </c>
       <c r="E1032" t="s">
         <v>16</v>
       </c>
       <c r="F1032" t="s">
-        <v>3137</v>
+        <v>3144</v>
       </c>
       <c r="G1032" t="s">
-        <v>3138</v>
+        <v>3145</v>
       </c>
       <c r="H1032">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I1032" t="s">
-        <v>3139</v>
+        <v>1151</v>
       </c>
       <c r="J1032" t="s">
-        <v>2389</v>
+        <v>2418</v>
       </c>
       <c r="K1032" t="s">
         <v>21</v>
       </c>
       <c r="L1032" t="s">
-        <v>458</v>
+        <v>3143</v>
       </c>
       <c r="M1032" t="s">
         <v>23</v>
@@ -52226,40 +52220,40 @@
     </row>
     <row r="1033" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1033" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1033" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1033" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="D1033" t="s">
         <v>15</v>
       </c>
       <c r="E1033" t="s">
-        <v>1730</v>
+        <v>16</v>
       </c>
       <c r="F1033" t="s">
-        <v>3142</v>
+        <v>3146</v>
       </c>
       <c r="G1033" t="s">
-        <v>3143</v>
+        <v>3147</v>
       </c>
       <c r="H1033">
         <v>3</v>
       </c>
       <c r="I1033" t="s">
-        <v>3144</v>
+        <v>1425</v>
       </c>
       <c r="J1033" t="s">
-        <v>1759</v>
+        <v>2418</v>
       </c>
       <c r="K1033" t="s">
         <v>21</v>
       </c>
       <c r="L1033" t="s">
-        <v>3145</v>
+        <v>3148</v>
       </c>
       <c r="M1033" t="s">
         <v>23</v>
@@ -52267,25 +52261,25 @@
     </row>
     <row r="1034" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1034" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1034" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1034" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="D1034" t="s">
         <v>15</v>
       </c>
       <c r="E1034" t="s">
-        <v>16</v>
+        <v>1730</v>
       </c>
       <c r="F1034" t="s">
-        <v>3146</v>
+        <v>3149</v>
       </c>
       <c r="G1034" t="s">
-        <v>3147</v>
+        <v>3150</v>
       </c>
       <c r="H1034">
         <v>3</v>
@@ -52294,13 +52288,13 @@
         <v>1151</v>
       </c>
       <c r="J1034" t="s">
-        <v>2418</v>
+        <v>163</v>
       </c>
       <c r="K1034" t="s">
-        <v>21</v>
+        <v>325</v>
       </c>
       <c r="L1034" t="s">
-        <v>3145</v>
+        <v>3151</v>
       </c>
       <c r="M1034" t="s">
         <v>23</v>
@@ -52308,40 +52302,40 @@
     </row>
     <row r="1035" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1035" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1035" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1035" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="D1035" t="s">
         <v>15</v>
       </c>
       <c r="E1035" t="s">
-        <v>16</v>
+        <v>2538</v>
       </c>
       <c r="F1035" t="s">
-        <v>3148</v>
+        <v>3152</v>
       </c>
       <c r="G1035" t="s">
-        <v>3149</v>
+        <v>3153</v>
       </c>
       <c r="H1035">
         <v>3</v>
       </c>
       <c r="I1035" t="s">
-        <v>1425</v>
+        <v>1151</v>
       </c>
       <c r="J1035" t="s">
-        <v>2418</v>
+        <v>289</v>
       </c>
       <c r="K1035" t="s">
-        <v>21</v>
+        <v>325</v>
       </c>
       <c r="L1035" t="s">
-        <v>3150</v>
+        <v>3151</v>
       </c>
       <c r="M1035" t="s">
         <v>23</v>
@@ -52349,13 +52343,13 @@
     </row>
     <row r="1036" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1036" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1036" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1036" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="D1036" t="s">
         <v>15</v>
@@ -52364,25 +52358,25 @@
         <v>1730</v>
       </c>
       <c r="F1036" t="s">
-        <v>3151</v>
+        <v>3154</v>
       </c>
       <c r="G1036" t="s">
-        <v>3152</v>
+        <v>3155</v>
       </c>
       <c r="H1036">
         <v>3</v>
       </c>
       <c r="I1036" t="s">
-        <v>1151</v>
+        <v>1425</v>
       </c>
       <c r="J1036" t="s">
-        <v>163</v>
+        <v>70</v>
       </c>
       <c r="K1036" t="s">
         <v>325</v>
       </c>
       <c r="L1036" t="s">
-        <v>3153</v>
+        <v>3151</v>
       </c>
       <c r="M1036" t="s">
         <v>23</v>
@@ -52390,40 +52384,40 @@
     </row>
     <row r="1037" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1037" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1037" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1037" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="D1037" t="s">
         <v>15</v>
       </c>
       <c r="E1037" t="s">
-        <v>2538</v>
+        <v>1730</v>
       </c>
       <c r="F1037" t="s">
-        <v>3154</v>
+        <v>3156</v>
       </c>
       <c r="G1037" t="s">
-        <v>3155</v>
+        <v>3157</v>
       </c>
       <c r="H1037">
         <v>3</v>
       </c>
       <c r="I1037" t="s">
-        <v>1151</v>
+        <v>1804</v>
       </c>
       <c r="J1037" t="s">
-        <v>289</v>
+        <v>86</v>
       </c>
       <c r="K1037" t="s">
         <v>325</v>
       </c>
       <c r="L1037" t="s">
-        <v>3153</v>
+        <v>3151</v>
       </c>
       <c r="M1037" t="s">
         <v>23</v>
@@ -52431,40 +52425,40 @@
     </row>
     <row r="1038" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1038" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1038" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1038" t="s">
-        <v>3140</v>
+        <v>3158</v>
       </c>
       <c r="D1038" t="s">
-        <v>15</v>
+        <v>3159</v>
       </c>
       <c r="E1038" t="s">
-        <v>1730</v>
+        <v>16</v>
       </c>
       <c r="F1038" t="s">
-        <v>3156</v>
+        <v>3160</v>
       </c>
       <c r="G1038" t="s">
-        <v>3157</v>
+        <v>3161</v>
       </c>
       <c r="H1038">
         <v>3</v>
       </c>
       <c r="I1038" t="s">
-        <v>1425</v>
+        <v>1804</v>
       </c>
       <c r="J1038" t="s">
-        <v>70</v>
+        <v>1345</v>
       </c>
       <c r="K1038" t="s">
-        <v>325</v>
+        <v>21</v>
       </c>
       <c r="L1038" t="s">
-        <v>3153</v>
+        <v>3148</v>
       </c>
       <c r="M1038" t="s">
         <v>23</v>
@@ -52472,40 +52466,40 @@
     </row>
     <row r="1039" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1039" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1039" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1039" t="s">
-        <v>3140</v>
+        <v>3158</v>
       </c>
       <c r="D1039" t="s">
-        <v>15</v>
+        <v>3159</v>
       </c>
       <c r="E1039" t="s">
-        <v>1730</v>
+        <v>16</v>
       </c>
       <c r="F1039" t="s">
-        <v>3158</v>
+        <v>3162</v>
       </c>
       <c r="G1039" t="s">
-        <v>3159</v>
+        <v>3163</v>
       </c>
       <c r="H1039">
         <v>3</v>
       </c>
       <c r="I1039" t="s">
-        <v>1804</v>
+        <v>1151</v>
       </c>
       <c r="J1039" t="s">
-        <v>86</v>
+        <v>1774</v>
       </c>
       <c r="K1039" t="s">
-        <v>325</v>
+        <v>21</v>
       </c>
       <c r="L1039" t="s">
-        <v>3153</v>
+        <v>3148</v>
       </c>
       <c r="M1039" t="s">
         <v>23</v>
@@ -52513,31 +52507,31 @@
     </row>
     <row r="1040" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1040" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1040" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1040" t="s">
-        <v>3160</v>
+        <v>3164</v>
       </c>
       <c r="D1040" t="s">
-        <v>3161</v>
+        <v>3165</v>
       </c>
       <c r="E1040" t="s">
         <v>16</v>
       </c>
       <c r="F1040" t="s">
-        <v>3162</v>
+        <v>3166</v>
       </c>
       <c r="G1040" t="s">
-        <v>3163</v>
+        <v>3167</v>
       </c>
       <c r="H1040">
         <v>3</v>
       </c>
       <c r="I1040" t="s">
-        <v>1804</v>
+        <v>3168</v>
       </c>
       <c r="J1040" t="s">
         <v>1345</v>
@@ -52546,7 +52540,7 @@
         <v>21</v>
       </c>
       <c r="L1040" t="s">
-        <v>3150</v>
+        <v>3143</v>
       </c>
       <c r="M1040" t="s">
         <v>23</v>
@@ -52554,31 +52548,31 @@
     </row>
     <row r="1041" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1041" t="s">
-        <v>3140</v>
+        <v>3138</v>
       </c>
       <c r="B1041" t="s">
-        <v>3141</v>
+        <v>3139</v>
       </c>
       <c r="C1041" t="s">
-        <v>3160</v>
+        <v>3164</v>
       </c>
       <c r="D1041" t="s">
-        <v>3161</v>
+        <v>3165</v>
       </c>
       <c r="E1041" t="s">
         <v>16</v>
       </c>
       <c r="F1041" t="s">
-        <v>3164</v>
+        <v>3169</v>
       </c>
       <c r="G1041" t="s">
-        <v>3165</v>
+        <v>3170</v>
       </c>
       <c r="H1041">
         <v>3</v>
       </c>
       <c r="I1041" t="s">
-        <v>1151</v>
+        <v>3171</v>
       </c>
       <c r="J1041" t="s">
         <v>1774</v>
@@ -52587,91 +52581,9 @@
         <v>21</v>
       </c>
       <c r="L1041" t="s">
-        <v>3150</v>
+        <v>3143</v>
       </c>
       <c r="M1041" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="1042" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1042" t="s">
-        <v>3140</v>
-      </c>
-      <c r="B1042" t="s">
-        <v>3141</v>
-      </c>
-      <c r="C1042" t="s">
-        <v>3166</v>
-      </c>
-      <c r="D1042" t="s">
-        <v>3167</v>
-      </c>
-      <c r="E1042" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1042" t="s">
-        <v>3168</v>
-      </c>
-      <c r="G1042" t="s">
-        <v>3169</v>
-      </c>
-      <c r="H1042">
-        <v>3</v>
-      </c>
-      <c r="I1042" t="s">
-        <v>3170</v>
-      </c>
-      <c r="J1042" t="s">
-        <v>1345</v>
-      </c>
-      <c r="K1042" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1042" t="s">
-        <v>3145</v>
-      </c>
-      <c r="M1042" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="1043" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1043" t="s">
-        <v>3140</v>
-      </c>
-      <c r="B1043" t="s">
-        <v>3141</v>
-      </c>
-      <c r="C1043" t="s">
-        <v>3166</v>
-      </c>
-      <c r="D1043" t="s">
-        <v>3167</v>
-      </c>
-      <c r="E1043" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1043" t="s">
-        <v>3171</v>
-      </c>
-      <c r="G1043" t="s">
-        <v>3172</v>
-      </c>
-      <c r="H1043">
-        <v>3</v>
-      </c>
-      <c r="I1043" t="s">
-        <v>3173</v>
-      </c>
-      <c r="J1043" t="s">
-        <v>1774</v>
-      </c>
-      <c r="K1043" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1043" t="s">
-        <v>3145</v>
-      </c>
-      <c r="M1043" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-09-16T23:46Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12493" uniqueCount="3173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12493" uniqueCount="3172">
   <si>
     <t>campusCode</t>
   </si>
@@ -8740,7 +8740,7 @@
     <t>수 11:00-13:00</t>
   </si>
   <si>
-    <t>예술관지하2층6-2호실</t>
+    <t>예술관지하2층6-1호실</t>
   </si>
   <si>
     <t>36297</t>
@@ -8870,9 +8870,6 @@
   </si>
   <si>
     <t>공연예술사</t>
-  </si>
-  <si>
-    <t>예술관지하2층6-1호실</t>
   </si>
   <si>
     <t>709390a</t>
@@ -49345,7 +49342,7 @@
         <v>21</v>
       </c>
       <c r="L962" t="s">
-        <v>2953</v>
+        <v>2909</v>
       </c>
       <c r="M962" t="s">
         <v>23</v>
@@ -49368,16 +49365,16 @@
         <v>16</v>
       </c>
       <c r="F963" t="s">
+        <v>2953</v>
+      </c>
+      <c r="G963" t="s">
         <v>2954</v>
-      </c>
-      <c r="G963" t="s">
-        <v>2955</v>
       </c>
       <c r="H963">
         <v>2</v>
       </c>
       <c r="I963" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
       <c r="J963" t="s">
         <v>710</v>
@@ -49386,7 +49383,7 @@
         <v>21</v>
       </c>
       <c r="L963" t="s">
-        <v>2953</v>
+        <v>2909</v>
       </c>
       <c r="M963" t="s">
         <v>23</v>
@@ -49409,16 +49406,16 @@
         <v>16</v>
       </c>
       <c r="F964" t="s">
+        <v>2956</v>
+      </c>
+      <c r="G964" t="s">
         <v>2957</v>
-      </c>
-      <c r="G964" t="s">
-        <v>2958</v>
       </c>
       <c r="H964">
         <v>2</v>
       </c>
       <c r="I964" t="s">
-        <v>2959</v>
+        <v>2958</v>
       </c>
       <c r="J964" t="s">
         <v>707</v>
@@ -49427,7 +49424,7 @@
         <v>21</v>
       </c>
       <c r="L964" t="s">
-        <v>2953</v>
+        <v>2909</v>
       </c>
       <c r="M964" t="s">
         <v>23</v>
@@ -49435,25 +49432,25 @@
     </row>
     <row r="965" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A965" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B965" t="s">
         <v>2960</v>
       </c>
-      <c r="B965" t="s">
+      <c r="C965" t="s">
         <v>2961</v>
       </c>
-      <c r="C965" t="s">
+      <c r="D965" t="s">
         <v>2962</v>
-      </c>
-      <c r="D965" t="s">
-        <v>2963</v>
       </c>
       <c r="E965" t="s">
         <v>2276</v>
       </c>
       <c r="F965" t="s">
+        <v>2963</v>
+      </c>
+      <c r="G965" t="s">
         <v>2964</v>
-      </c>
-      <c r="G965" t="s">
-        <v>2965</v>
       </c>
       <c r="H965">
         <v>3</v>
@@ -49462,13 +49459,13 @@
         <v>219</v>
       </c>
       <c r="J965" t="s">
+        <v>2965</v>
+      </c>
+      <c r="K965" t="s">
+        <v>21</v>
+      </c>
+      <c r="L965" t="s">
         <v>2966</v>
-      </c>
-      <c r="K965" t="s">
-        <v>21</v>
-      </c>
-      <c r="L965" t="s">
-        <v>2967</v>
       </c>
       <c r="M965" t="s">
         <v>23</v>
@@ -49476,25 +49473,25 @@
     </row>
     <row r="966" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A966" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B966" t="s">
         <v>2960</v>
       </c>
-      <c r="B966" t="s">
+      <c r="C966" t="s">
         <v>2961</v>
       </c>
-      <c r="C966" t="s">
+      <c r="D966" t="s">
         <v>2962</v>
-      </c>
-      <c r="D966" t="s">
-        <v>2963</v>
       </c>
       <c r="E966" t="s">
         <v>16</v>
       </c>
       <c r="F966" t="s">
+        <v>2967</v>
+      </c>
+      <c r="G966" t="s">
         <v>2968</v>
-      </c>
-      <c r="G966" t="s">
-        <v>2969</v>
       </c>
       <c r="H966">
         <v>3</v>
@@ -49503,7 +49500,7 @@
         <v>219</v>
       </c>
       <c r="J966" t="s">
-        <v>2970</v>
+        <v>2969</v>
       </c>
       <c r="K966" t="s">
         <v>21</v>
@@ -49517,34 +49514,34 @@
     </row>
     <row r="967" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A967" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B967" t="s">
         <v>2960</v>
       </c>
-      <c r="B967" t="s">
+      <c r="C967" t="s">
         <v>2961</v>
       </c>
-      <c r="C967" t="s">
+      <c r="D967" t="s">
         <v>2962</v>
-      </c>
-      <c r="D967" t="s">
-        <v>2963</v>
       </c>
       <c r="E967" t="s">
         <v>16</v>
       </c>
       <c r="F967" t="s">
+        <v>2970</v>
+      </c>
+      <c r="G967" t="s">
         <v>2971</v>
       </c>
-      <c r="G967" t="s">
+      <c r="H967">
+        <v>3</v>
+      </c>
+      <c r="I967" t="s">
         <v>2972</v>
       </c>
-      <c r="H967">
-        <v>3</v>
-      </c>
-      <c r="I967" t="s">
+      <c r="J967" t="s">
         <v>2973</v>
-      </c>
-      <c r="J967" t="s">
-        <v>2974</v>
       </c>
       <c r="K967" t="s">
         <v>21</v>
@@ -49558,34 +49555,34 @@
     </row>
     <row r="968" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A968" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B968" t="s">
         <v>2960</v>
       </c>
-      <c r="B968" t="s">
+      <c r="C968" t="s">
         <v>2961</v>
       </c>
-      <c r="C968" t="s">
+      <c r="D968" t="s">
         <v>2962</v>
-      </c>
-      <c r="D968" t="s">
-        <v>2963</v>
       </c>
       <c r="E968" t="s">
         <v>2276</v>
       </c>
       <c r="F968" t="s">
+        <v>2974</v>
+      </c>
+      <c r="G968" t="s">
         <v>2975</v>
       </c>
-      <c r="G968" t="s">
+      <c r="H968">
+        <v>3</v>
+      </c>
+      <c r="I968" t="s">
         <v>2976</v>
       </c>
-      <c r="H968">
-        <v>3</v>
-      </c>
-      <c r="I968" t="s">
-        <v>2977</v>
-      </c>
       <c r="J968" t="s">
-        <v>2970</v>
+        <v>2969</v>
       </c>
       <c r="K968" t="s">
         <v>21</v>
@@ -49599,34 +49596,34 @@
     </row>
     <row r="969" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A969" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B969" t="s">
         <v>2960</v>
       </c>
-      <c r="B969" t="s">
+      <c r="C969" t="s">
         <v>2961</v>
       </c>
-      <c r="C969" t="s">
+      <c r="D969" t="s">
         <v>2962</v>
-      </c>
-      <c r="D969" t="s">
-        <v>2963</v>
       </c>
       <c r="E969" t="s">
         <v>16</v>
       </c>
       <c r="F969" t="s">
+        <v>2977</v>
+      </c>
+      <c r="G969" t="s">
         <v>2978</v>
       </c>
-      <c r="G969" t="s">
+      <c r="H969">
+        <v>3</v>
+      </c>
+      <c r="I969" t="s">
         <v>2979</v>
       </c>
-      <c r="H969">
-        <v>3</v>
-      </c>
-      <c r="I969" t="s">
+      <c r="J969" t="s">
         <v>2980</v>
-      </c>
-      <c r="J969" t="s">
-        <v>2981</v>
       </c>
       <c r="K969" t="s">
         <v>21</v>
@@ -49640,25 +49637,25 @@
     </row>
     <row r="970" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A970" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B970" t="s">
         <v>2960</v>
       </c>
-      <c r="B970" t="s">
+      <c r="C970" t="s">
         <v>2961</v>
       </c>
-      <c r="C970" t="s">
+      <c r="D970" t="s">
         <v>2962</v>
-      </c>
-      <c r="D970" t="s">
-        <v>2963</v>
       </c>
       <c r="E970" t="s">
         <v>16</v>
       </c>
       <c r="F970" t="s">
+        <v>2981</v>
+      </c>
+      <c r="G970" t="s">
         <v>2982</v>
-      </c>
-      <c r="G970" t="s">
-        <v>2983</v>
       </c>
       <c r="H970">
         <v>3</v>
@@ -49681,31 +49678,31 @@
     </row>
     <row r="971" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A971" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B971" t="s">
         <v>2960</v>
       </c>
-      <c r="B971" t="s">
+      <c r="C971" t="s">
         <v>2961</v>
       </c>
-      <c r="C971" t="s">
+      <c r="D971" t="s">
         <v>2962</v>
-      </c>
-      <c r="D971" t="s">
-        <v>2963</v>
       </c>
       <c r="E971" t="s">
         <v>16</v>
       </c>
       <c r="F971" t="s">
+        <v>2981</v>
+      </c>
+      <c r="G971" t="s">
         <v>2982</v>
       </c>
-      <c r="G971" t="s">
-        <v>2983</v>
-      </c>
       <c r="H971">
         <v>3</v>
       </c>
       <c r="I971" t="s">
-        <v>2977</v>
+        <v>2976</v>
       </c>
       <c r="J971" t="s">
         <v>205</v>
@@ -49722,31 +49719,31 @@
     </row>
     <row r="972" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A972" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B972" t="s">
         <v>2960</v>
       </c>
-      <c r="B972" t="s">
+      <c r="C972" t="s">
         <v>2961</v>
       </c>
-      <c r="C972" t="s">
+      <c r="D972" t="s">
         <v>2962</v>
-      </c>
-      <c r="D972" t="s">
-        <v>2963</v>
       </c>
       <c r="E972" t="s">
         <v>16</v>
       </c>
       <c r="F972" t="s">
+        <v>2981</v>
+      </c>
+      <c r="G972" t="s">
         <v>2982</v>
       </c>
-      <c r="G972" t="s">
-        <v>2983</v>
-      </c>
       <c r="H972">
         <v>3</v>
       </c>
       <c r="I972" t="s">
-        <v>2973</v>
+        <v>2972</v>
       </c>
       <c r="J972" t="s">
         <v>205</v>
@@ -49763,25 +49760,25 @@
     </row>
     <row r="973" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A973" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B973" t="s">
         <v>2960</v>
       </c>
-      <c r="B973" t="s">
+      <c r="C973" t="s">
         <v>2961</v>
       </c>
-      <c r="C973" t="s">
+      <c r="D973" t="s">
         <v>2962</v>
-      </c>
-      <c r="D973" t="s">
-        <v>2963</v>
       </c>
       <c r="E973" t="s">
         <v>16</v>
       </c>
       <c r="F973" t="s">
+        <v>2981</v>
+      </c>
+      <c r="G973" t="s">
         <v>2982</v>
-      </c>
-      <c r="G973" t="s">
-        <v>2983</v>
       </c>
       <c r="H973">
         <v>3</v>
@@ -49804,25 +49801,25 @@
     </row>
     <row r="974" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A974" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B974" t="s">
         <v>2960</v>
       </c>
-      <c r="B974" t="s">
+      <c r="C974" t="s">
         <v>2961</v>
       </c>
-      <c r="C974" t="s">
+      <c r="D974" t="s">
         <v>2962</v>
-      </c>
-      <c r="D974" t="s">
-        <v>2963</v>
       </c>
       <c r="E974" t="s">
         <v>16</v>
       </c>
       <c r="F974" t="s">
+        <v>2981</v>
+      </c>
+      <c r="G974" t="s">
         <v>2982</v>
-      </c>
-      <c r="G974" t="s">
-        <v>2983</v>
       </c>
       <c r="H974">
         <v>3</v>
@@ -49845,25 +49842,25 @@
     </row>
     <row r="975" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A975" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B975" t="s">
         <v>2960</v>
       </c>
-      <c r="B975" t="s">
+      <c r="C975" t="s">
         <v>2961</v>
       </c>
-      <c r="C975" t="s">
+      <c r="D975" t="s">
         <v>2962</v>
-      </c>
-      <c r="D975" t="s">
-        <v>2963</v>
       </c>
       <c r="E975" t="s">
         <v>16</v>
       </c>
       <c r="F975" t="s">
+        <v>2983</v>
+      </c>
+      <c r="G975" t="s">
         <v>2984</v>
-      </c>
-      <c r="G975" t="s">
-        <v>2985</v>
       </c>
       <c r="H975">
         <v>3</v>
@@ -49886,31 +49883,31 @@
     </row>
     <row r="976" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A976" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B976" t="s">
         <v>2960</v>
       </c>
-      <c r="B976" t="s">
+      <c r="C976" t="s">
         <v>2961</v>
       </c>
-      <c r="C976" t="s">
+      <c r="D976" t="s">
         <v>2962</v>
-      </c>
-      <c r="D976" t="s">
-        <v>2963</v>
       </c>
       <c r="E976" t="s">
         <v>16</v>
       </c>
       <c r="F976" t="s">
+        <v>2983</v>
+      </c>
+      <c r="G976" t="s">
         <v>2984</v>
       </c>
-      <c r="G976" t="s">
-        <v>2985</v>
-      </c>
       <c r="H976">
         <v>3</v>
       </c>
       <c r="I976" t="s">
-        <v>2973</v>
+        <v>2972</v>
       </c>
       <c r="J976" t="s">
         <v>205</v>
@@ -49927,31 +49924,31 @@
     </row>
     <row r="977" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A977" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B977" t="s">
         <v>2960</v>
       </c>
-      <c r="B977" t="s">
+      <c r="C977" t="s">
         <v>2961</v>
       </c>
-      <c r="C977" t="s">
+      <c r="D977" t="s">
         <v>2962</v>
-      </c>
-      <c r="D977" t="s">
-        <v>2963</v>
       </c>
       <c r="E977" t="s">
         <v>16</v>
       </c>
       <c r="F977" t="s">
+        <v>2983</v>
+      </c>
+      <c r="G977" t="s">
         <v>2984</v>
       </c>
-      <c r="G977" t="s">
-        <v>2985</v>
-      </c>
       <c r="H977">
         <v>3</v>
       </c>
       <c r="I977" t="s">
-        <v>2977</v>
+        <v>2976</v>
       </c>
       <c r="J977" t="s">
         <v>205</v>
@@ -49968,25 +49965,25 @@
     </row>
     <row r="978" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A978" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B978" t="s">
         <v>2960</v>
       </c>
-      <c r="B978" t="s">
+      <c r="C978" t="s">
         <v>2961</v>
       </c>
-      <c r="C978" t="s">
+      <c r="D978" t="s">
         <v>2962</v>
-      </c>
-      <c r="D978" t="s">
-        <v>2963</v>
       </c>
       <c r="E978" t="s">
         <v>16</v>
       </c>
       <c r="F978" t="s">
+        <v>2983</v>
+      </c>
+      <c r="G978" t="s">
         <v>2984</v>
-      </c>
-      <c r="G978" t="s">
-        <v>2985</v>
       </c>
       <c r="H978">
         <v>3</v>
@@ -50009,25 +50006,25 @@
     </row>
     <row r="979" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A979" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B979" t="s">
         <v>2960</v>
       </c>
-      <c r="B979" t="s">
+      <c r="C979" t="s">
         <v>2961</v>
       </c>
-      <c r="C979" t="s">
+      <c r="D979" t="s">
         <v>2962</v>
-      </c>
-      <c r="D979" t="s">
-        <v>2963</v>
       </c>
       <c r="E979" t="s">
         <v>16</v>
       </c>
       <c r="F979" t="s">
+        <v>2985</v>
+      </c>
+      <c r="G979" t="s">
         <v>2986</v>
-      </c>
-      <c r="G979" t="s">
-        <v>2987</v>
       </c>
       <c r="H979">
         <v>3</v>
@@ -50036,7 +50033,7 @@
         <v>219</v>
       </c>
       <c r="J979" t="s">
-        <v>2988</v>
+        <v>2987</v>
       </c>
       <c r="K979" t="s">
         <v>21</v>
@@ -50050,40 +50047,40 @@
     </row>
     <row r="980" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A980" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B980" t="s">
         <v>2960</v>
       </c>
-      <c r="B980" t="s">
+      <c r="C980" t="s">
         <v>2961</v>
       </c>
-      <c r="C980" t="s">
+      <c r="D980" t="s">
         <v>2962</v>
-      </c>
-      <c r="D980" t="s">
-        <v>2963</v>
       </c>
       <c r="E980" t="s">
         <v>16</v>
       </c>
       <c r="F980" t="s">
+        <v>2988</v>
+      </c>
+      <c r="G980" t="s">
         <v>2989</v>
       </c>
-      <c r="G980" t="s">
+      <c r="H980">
+        <v>3</v>
+      </c>
+      <c r="I980" t="s">
+        <v>2976</v>
+      </c>
+      <c r="J980" t="s">
         <v>2990</v>
       </c>
-      <c r="H980">
-        <v>3</v>
-      </c>
-      <c r="I980" t="s">
-        <v>2977</v>
-      </c>
-      <c r="J980" t="s">
-        <v>2991</v>
-      </c>
       <c r="K980" t="s">
         <v>21</v>
       </c>
       <c r="L980" t="s">
-        <v>2967</v>
+        <v>2966</v>
       </c>
       <c r="M980" t="s">
         <v>23</v>
@@ -50091,40 +50088,40 @@
     </row>
     <row r="981" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A981" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B981" t="s">
         <v>2960</v>
       </c>
-      <c r="B981" t="s">
+      <c r="C981" t="s">
         <v>2961</v>
       </c>
-      <c r="C981" t="s">
+      <c r="D981" t="s">
         <v>2962</v>
-      </c>
-      <c r="D981" t="s">
-        <v>2963</v>
       </c>
       <c r="E981" t="s">
         <v>16</v>
       </c>
       <c r="F981" t="s">
+        <v>2991</v>
+      </c>
+      <c r="G981" t="s">
         <v>2992</v>
       </c>
-      <c r="G981" t="s">
+      <c r="H981">
+        <v>3</v>
+      </c>
+      <c r="I981" t="s">
+        <v>2972</v>
+      </c>
+      <c r="J981" t="s">
+        <v>2990</v>
+      </c>
+      <c r="K981" t="s">
+        <v>21</v>
+      </c>
+      <c r="L981" t="s">
         <v>2993</v>
-      </c>
-      <c r="H981">
-        <v>3</v>
-      </c>
-      <c r="I981" t="s">
-        <v>2973</v>
-      </c>
-      <c r="J981" t="s">
-        <v>2991</v>
-      </c>
-      <c r="K981" t="s">
-        <v>21</v>
-      </c>
-      <c r="L981" t="s">
-        <v>2994</v>
       </c>
       <c r="M981" t="s">
         <v>23</v>
@@ -50132,25 +50129,25 @@
     </row>
     <row r="982" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A982" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B982" t="s">
         <v>2960</v>
       </c>
-      <c r="B982" t="s">
+      <c r="C982" t="s">
         <v>2961</v>
       </c>
-      <c r="C982" t="s">
+      <c r="D982" t="s">
         <v>2962</v>
-      </c>
-      <c r="D982" t="s">
-        <v>2963</v>
       </c>
       <c r="E982" t="s">
         <v>16</v>
       </c>
       <c r="F982" t="s">
+        <v>2994</v>
+      </c>
+      <c r="G982" t="s">
         <v>2995</v>
-      </c>
-      <c r="G982" t="s">
-        <v>2996</v>
       </c>
       <c r="H982">
         <v>3</v>
@@ -50159,13 +50156,13 @@
         <v>213</v>
       </c>
       <c r="J982" t="s">
-        <v>2997</v>
+        <v>2996</v>
       </c>
       <c r="K982" t="s">
         <v>21</v>
       </c>
       <c r="L982" t="s">
-        <v>2994</v>
+        <v>2993</v>
       </c>
       <c r="M982" t="s">
         <v>23</v>
@@ -50173,25 +50170,25 @@
     </row>
     <row r="983" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A983" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B983" t="s">
         <v>2960</v>
       </c>
-      <c r="B983" t="s">
+      <c r="C983" t="s">
         <v>2961</v>
       </c>
-      <c r="C983" t="s">
+      <c r="D983" t="s">
         <v>2962</v>
-      </c>
-      <c r="D983" t="s">
-        <v>2963</v>
       </c>
       <c r="E983" t="s">
         <v>16</v>
       </c>
       <c r="F983" t="s">
+        <v>2997</v>
+      </c>
+      <c r="G983" t="s">
         <v>2998</v>
-      </c>
-      <c r="G983" t="s">
-        <v>2999</v>
       </c>
       <c r="H983">
         <v>3</v>
@@ -50200,7 +50197,7 @@
         <v>216</v>
       </c>
       <c r="J983" t="s">
-        <v>2974</v>
+        <v>2973</v>
       </c>
       <c r="K983" t="s">
         <v>21</v>
@@ -50214,25 +50211,25 @@
     </row>
     <row r="984" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A984" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B984" t="s">
         <v>2960</v>
       </c>
-      <c r="B984" t="s">
+      <c r="C984" t="s">
         <v>2961</v>
       </c>
-      <c r="C984" t="s">
+      <c r="D984" t="s">
         <v>2962</v>
-      </c>
-      <c r="D984" t="s">
-        <v>2963</v>
       </c>
       <c r="E984" t="s">
         <v>16</v>
       </c>
       <c r="F984" t="s">
+        <v>2999</v>
+      </c>
+      <c r="G984" t="s">
         <v>3000</v>
-      </c>
-      <c r="G984" t="s">
-        <v>3001</v>
       </c>
       <c r="H984">
         <v>6</v>
@@ -50255,31 +50252,31 @@
     </row>
     <row r="985" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A985" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B985" t="s">
         <v>2960</v>
       </c>
-      <c r="B985" t="s">
+      <c r="C985" t="s">
         <v>2961</v>
       </c>
-      <c r="C985" t="s">
+      <c r="D985" t="s">
         <v>2962</v>
-      </c>
-      <c r="D985" t="s">
-        <v>2963</v>
       </c>
       <c r="E985" t="s">
         <v>16</v>
       </c>
       <c r="F985" t="s">
+        <v>3001</v>
+      </c>
+      <c r="G985" t="s">
         <v>3002</v>
-      </c>
-      <c r="G985" t="s">
-        <v>3003</v>
       </c>
       <c r="H985">
         <v>6</v>
       </c>
       <c r="I985" t="s">
-        <v>3004</v>
+        <v>3003</v>
       </c>
       <c r="J985" t="s">
         <v>205</v>
@@ -50296,34 +50293,34 @@
     </row>
     <row r="986" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A986" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B986" t="s">
         <v>2960</v>
       </c>
-      <c r="B986" t="s">
+      <c r="C986" t="s">
         <v>2961</v>
       </c>
-      <c r="C986" t="s">
+      <c r="D986" t="s">
         <v>2962</v>
-      </c>
-      <c r="D986" t="s">
-        <v>2963</v>
       </c>
       <c r="E986" t="s">
         <v>16</v>
       </c>
       <c r="F986" t="s">
+        <v>3004</v>
+      </c>
+      <c r="G986" t="s">
         <v>3005</v>
       </c>
-      <c r="G986" t="s">
+      <c r="H986">
+        <v>3</v>
+      </c>
+      <c r="I986" t="s">
         <v>3006</v>
       </c>
-      <c r="H986">
-        <v>3</v>
-      </c>
-      <c r="I986" t="s">
-        <v>3007</v>
-      </c>
       <c r="J986" t="s">
-        <v>2988</v>
+        <v>2987</v>
       </c>
       <c r="K986" t="s">
         <v>21</v>
@@ -50337,31 +50334,31 @@
     </row>
     <row r="987" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A987" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B987" t="s">
         <v>2960</v>
       </c>
-      <c r="B987" t="s">
-        <v>2961</v>
-      </c>
       <c r="C987" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D987" t="s">
         <v>3008</v>
-      </c>
-      <c r="D987" t="s">
-        <v>3009</v>
       </c>
       <c r="E987" t="s">
         <v>2276</v>
       </c>
       <c r="F987" t="s">
+        <v>3009</v>
+      </c>
+      <c r="G987" t="s">
+        <v>2975</v>
+      </c>
+      <c r="H987">
+        <v>3</v>
+      </c>
+      <c r="I987" t="s">
         <v>3010</v>
-      </c>
-      <c r="G987" t="s">
-        <v>2976</v>
-      </c>
-      <c r="H987">
-        <v>3</v>
-      </c>
-      <c r="I987" t="s">
-        <v>3011</v>
       </c>
       <c r="J987" t="s">
         <v>94</v>
@@ -50378,31 +50375,31 @@
     </row>
     <row r="988" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A988" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B988" t="s">
         <v>2960</v>
       </c>
-      <c r="B988" t="s">
-        <v>2961</v>
-      </c>
       <c r="C988" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D988" t="s">
         <v>3008</v>
-      </c>
-      <c r="D988" t="s">
-        <v>3009</v>
       </c>
       <c r="E988" t="s">
         <v>16</v>
       </c>
       <c r="F988" t="s">
+        <v>3011</v>
+      </c>
+      <c r="G988" t="s">
         <v>3012</v>
       </c>
-      <c r="G988" t="s">
+      <c r="H988">
+        <v>3</v>
+      </c>
+      <c r="I988" t="s">
         <v>3013</v>
-      </c>
-      <c r="H988">
-        <v>3</v>
-      </c>
-      <c r="I988" t="s">
-        <v>3014</v>
       </c>
       <c r="J988" t="s">
         <v>90</v>
@@ -50419,25 +50416,25 @@
     </row>
     <row r="989" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A989" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B989" t="s">
         <v>2960</v>
       </c>
-      <c r="B989" t="s">
-        <v>2961</v>
-      </c>
       <c r="C989" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D989" t="s">
         <v>3008</v>
-      </c>
-      <c r="D989" t="s">
-        <v>3009</v>
       </c>
       <c r="E989" t="s">
         <v>16</v>
       </c>
       <c r="F989" t="s">
+        <v>3014</v>
+      </c>
+      <c r="G989" t="s">
         <v>3015</v>
-      </c>
-      <c r="G989" t="s">
-        <v>3016</v>
       </c>
       <c r="H989">
         <v>3</v>
@@ -50460,13 +50457,13 @@
     </row>
     <row r="990" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A990" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B990" t="s">
         <v>3017</v>
       </c>
-      <c r="B990" t="s">
-        <v>3018</v>
-      </c>
       <c r="C990" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D990" t="s">
         <v>15</v>
@@ -50475,16 +50472,16 @@
         <v>16</v>
       </c>
       <c r="F990" t="s">
+        <v>3018</v>
+      </c>
+      <c r="G990" t="s">
         <v>3019</v>
-      </c>
-      <c r="G990" t="s">
-        <v>3020</v>
       </c>
       <c r="H990">
         <v>2</v>
       </c>
       <c r="I990" t="s">
-        <v>3021</v>
+        <v>3020</v>
       </c>
       <c r="J990" t="s">
         <v>2572</v>
@@ -50493,7 +50490,7 @@
         <v>21</v>
       </c>
       <c r="L990" t="s">
-        <v>3022</v>
+        <v>3021</v>
       </c>
       <c r="M990" t="s">
         <v>23</v>
@@ -50501,13 +50498,13 @@
     </row>
     <row r="991" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A991" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B991" t="s">
         <v>3017</v>
       </c>
-      <c r="B991" t="s">
-        <v>3018</v>
-      </c>
       <c r="C991" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D991" t="s">
         <v>15</v>
@@ -50516,16 +50513,16 @@
         <v>16</v>
       </c>
       <c r="F991" t="s">
+        <v>3022</v>
+      </c>
+      <c r="G991" t="s">
         <v>3023</v>
-      </c>
-      <c r="G991" t="s">
-        <v>3024</v>
       </c>
       <c r="H991">
         <v>2</v>
       </c>
       <c r="I991" t="s">
-        <v>3025</v>
+        <v>3024</v>
       </c>
       <c r="J991" t="s">
         <v>2391</v>
@@ -50534,7 +50531,7 @@
         <v>21</v>
       </c>
       <c r="L991" t="s">
-        <v>3022</v>
+        <v>3021</v>
       </c>
       <c r="M991" t="s">
         <v>23</v>
@@ -50542,13 +50539,13 @@
     </row>
     <row r="992" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A992" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B992" t="s">
         <v>3017</v>
       </c>
-      <c r="B992" t="s">
-        <v>3018</v>
-      </c>
       <c r="C992" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D992" t="s">
         <v>15</v>
@@ -50557,10 +50554,10 @@
         <v>16</v>
       </c>
       <c r="F992" t="s">
+        <v>3025</v>
+      </c>
+      <c r="G992" t="s">
         <v>3026</v>
-      </c>
-      <c r="G992" t="s">
-        <v>3027</v>
       </c>
       <c r="H992">
         <v>2</v>
@@ -50575,7 +50572,7 @@
         <v>21</v>
       </c>
       <c r="L992" t="s">
-        <v>3028</v>
+        <v>3027</v>
       </c>
       <c r="M992" t="s">
         <v>23</v>
@@ -50583,13 +50580,13 @@
     </row>
     <row r="993" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A993" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B993" t="s">
         <v>3017</v>
       </c>
-      <c r="B993" t="s">
-        <v>3018</v>
-      </c>
       <c r="C993" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D993" t="s">
         <v>15</v>
@@ -50598,10 +50595,10 @@
         <v>16</v>
       </c>
       <c r="F993" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G993" t="s">
         <v>3029</v>
-      </c>
-      <c r="G993" t="s">
-        <v>3030</v>
       </c>
       <c r="H993">
         <v>2</v>
@@ -50616,7 +50613,7 @@
         <v>21</v>
       </c>
       <c r="L993" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M993" t="s">
         <v>23</v>
@@ -50624,13 +50621,13 @@
     </row>
     <row r="994" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A994" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B994" t="s">
         <v>3017</v>
       </c>
-      <c r="B994" t="s">
-        <v>3018</v>
-      </c>
       <c r="C994" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D994" t="s">
         <v>15</v>
@@ -50639,10 +50636,10 @@
         <v>16</v>
       </c>
       <c r="F994" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G994" t="s">
         <v>3029</v>
-      </c>
-      <c r="G994" t="s">
-        <v>3030</v>
       </c>
       <c r="H994">
         <v>2</v>
@@ -50665,13 +50662,13 @@
     </row>
     <row r="995" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A995" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B995" t="s">
         <v>3017</v>
       </c>
-      <c r="B995" t="s">
-        <v>3018</v>
-      </c>
       <c r="C995" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D995" t="s">
         <v>15</v>
@@ -50680,16 +50677,16 @@
         <v>16</v>
       </c>
       <c r="F995" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G995" t="s">
         <v>3029</v>
-      </c>
-      <c r="G995" t="s">
-        <v>3030</v>
       </c>
       <c r="H995">
         <v>2</v>
       </c>
       <c r="I995" t="s">
-        <v>3032</v>
+        <v>3031</v>
       </c>
       <c r="J995" t="s">
         <v>2399</v>
@@ -50706,13 +50703,13 @@
     </row>
     <row r="996" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A996" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B996" t="s">
         <v>3017</v>
       </c>
-      <c r="B996" t="s">
-        <v>3018</v>
-      </c>
       <c r="C996" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D996" t="s">
         <v>15</v>
@@ -50721,16 +50718,16 @@
         <v>16</v>
       </c>
       <c r="F996" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G996" t="s">
         <v>3029</v>
-      </c>
-      <c r="G996" t="s">
-        <v>3030</v>
       </c>
       <c r="H996">
         <v>2</v>
       </c>
       <c r="I996" t="s">
-        <v>3033</v>
+        <v>3032</v>
       </c>
       <c r="J996" t="s">
         <v>2391</v>
@@ -50739,7 +50736,7 @@
         <v>21</v>
       </c>
       <c r="L996" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M996" t="s">
         <v>646</v>
@@ -50747,13 +50744,13 @@
     </row>
     <row r="997" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A997" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B997" t="s">
         <v>3017</v>
       </c>
-      <c r="B997" t="s">
-        <v>3018</v>
-      </c>
       <c r="C997" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D997" t="s">
         <v>15</v>
@@ -50762,16 +50759,16 @@
         <v>16</v>
       </c>
       <c r="F997" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G997" t="s">
         <v>3029</v>
-      </c>
-      <c r="G997" t="s">
-        <v>3030</v>
       </c>
       <c r="H997">
         <v>2</v>
       </c>
       <c r="I997" t="s">
-        <v>3034</v>
+        <v>3033</v>
       </c>
       <c r="J997" t="s">
         <v>664</v>
@@ -50780,7 +50777,7 @@
         <v>21</v>
       </c>
       <c r="L997" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M997" t="s">
         <v>648</v>
@@ -50788,13 +50785,13 @@
     </row>
     <row r="998" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A998" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B998" t="s">
         <v>3017</v>
       </c>
-      <c r="B998" t="s">
-        <v>3018</v>
-      </c>
       <c r="C998" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D998" t="s">
         <v>15</v>
@@ -50803,25 +50800,25 @@
         <v>16</v>
       </c>
       <c r="F998" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G998" t="s">
         <v>3029</v>
-      </c>
-      <c r="G998" t="s">
-        <v>3030</v>
       </c>
       <c r="H998">
         <v>2</v>
       </c>
       <c r="I998" t="s">
+        <v>3034</v>
+      </c>
+      <c r="J998" t="s">
         <v>3035</v>
       </c>
-      <c r="J998" t="s">
-        <v>3036</v>
-      </c>
       <c r="K998" t="s">
         <v>21</v>
       </c>
       <c r="L998" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M998" t="s">
         <v>651</v>
@@ -50829,13 +50826,13 @@
     </row>
     <row r="999" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A999" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B999" t="s">
         <v>3017</v>
       </c>
-      <c r="B999" t="s">
-        <v>3018</v>
-      </c>
       <c r="C999" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D999" t="s">
         <v>15</v>
@@ -50844,16 +50841,16 @@
         <v>16</v>
       </c>
       <c r="F999" t="s">
+        <v>3036</v>
+      </c>
+      <c r="G999" t="s">
         <v>3037</v>
-      </c>
-      <c r="G999" t="s">
-        <v>3038</v>
       </c>
       <c r="H999">
         <v>2</v>
       </c>
       <c r="I999" t="s">
-        <v>3033</v>
+        <v>3032</v>
       </c>
       <c r="J999" t="s">
         <v>2549</v>
@@ -50862,7 +50859,7 @@
         <v>21</v>
       </c>
       <c r="L999" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M999" t="s">
         <v>23</v>
@@ -50870,13 +50867,13 @@
     </row>
     <row r="1000" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1000" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1000" t="s">
         <v>3017</v>
       </c>
-      <c r="B1000" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1000" t="s">
-        <v>3017</v>
+        <v>3016</v>
       </c>
       <c r="D1000" t="s">
         <v>15</v>
@@ -50885,25 +50882,25 @@
         <v>16</v>
       </c>
       <c r="F1000" t="s">
+        <v>3038</v>
+      </c>
+      <c r="G1000" t="s">
         <v>3039</v>
-      </c>
-      <c r="G1000" t="s">
-        <v>3040</v>
       </c>
       <c r="H1000">
         <v>2</v>
       </c>
       <c r="I1000" t="s">
-        <v>3034</v>
+        <v>3033</v>
       </c>
       <c r="J1000" t="s">
-        <v>3041</v>
+        <v>3040</v>
       </c>
       <c r="K1000" t="s">
         <v>21</v>
       </c>
       <c r="L1000" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M1000" t="s">
         <v>23</v>
@@ -50911,31 +50908,31 @@
     </row>
     <row r="1001" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1001" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1001" t="s">
         <v>3017</v>
       </c>
-      <c r="B1001" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1001" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1001" t="s">
         <v>3042</v>
-      </c>
-      <c r="D1001" t="s">
-        <v>3043</v>
       </c>
       <c r="E1001" t="s">
         <v>16</v>
       </c>
       <c r="F1001" t="s">
+        <v>3043</v>
+      </c>
+      <c r="G1001" t="s">
         <v>3044</v>
-      </c>
-      <c r="G1001" t="s">
-        <v>3045</v>
       </c>
       <c r="H1001">
         <v>2</v>
       </c>
       <c r="I1001" t="s">
-        <v>3033</v>
+        <v>3032</v>
       </c>
       <c r="J1001" t="s">
         <v>2572</v>
@@ -50944,7 +50941,7 @@
         <v>21</v>
       </c>
       <c r="L1001" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M1001" t="s">
         <v>23</v>
@@ -50952,31 +50949,31 @@
     </row>
     <row r="1002" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1002" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1002" t="s">
         <v>3017</v>
       </c>
-      <c r="B1002" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1002" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1002" t="s">
         <v>3042</v>
-      </c>
-      <c r="D1002" t="s">
-        <v>3043</v>
       </c>
       <c r="E1002" t="s">
         <v>16</v>
       </c>
       <c r="F1002" t="s">
+        <v>3045</v>
+      </c>
+      <c r="G1002" t="s">
         <v>3046</v>
-      </c>
-      <c r="G1002" t="s">
-        <v>3047</v>
       </c>
       <c r="H1002">
         <v>2</v>
       </c>
       <c r="I1002" t="s">
-        <v>3048</v>
+        <v>3047</v>
       </c>
       <c r="J1002" t="s">
         <v>2399</v>
@@ -50993,31 +50990,31 @@
     </row>
     <row r="1003" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1003" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1003" t="s">
         <v>3017</v>
       </c>
-      <c r="B1003" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1003" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1003" t="s">
         <v>3042</v>
-      </c>
-      <c r="D1003" t="s">
-        <v>3043</v>
       </c>
       <c r="E1003" t="s">
         <v>16</v>
       </c>
       <c r="F1003" t="s">
+        <v>3048</v>
+      </c>
+      <c r="G1003" t="s">
         <v>3049</v>
-      </c>
-      <c r="G1003" t="s">
-        <v>3050</v>
       </c>
       <c r="H1003">
         <v>2</v>
       </c>
       <c r="I1003" t="s">
-        <v>3051</v>
+        <v>3050</v>
       </c>
       <c r="J1003" t="s">
         <v>2549</v>
@@ -51026,7 +51023,7 @@
         <v>21</v>
       </c>
       <c r="L1003" t="s">
-        <v>3022</v>
+        <v>3021</v>
       </c>
       <c r="M1003" t="s">
         <v>23</v>
@@ -51034,31 +51031,31 @@
     </row>
     <row r="1004" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1004" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1004" t="s">
         <v>3017</v>
       </c>
-      <c r="B1004" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1004" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1004" t="s">
         <v>3042</v>
-      </c>
-      <c r="D1004" t="s">
-        <v>3043</v>
       </c>
       <c r="E1004" t="s">
         <v>16</v>
       </c>
       <c r="F1004" t="s">
+        <v>3051</v>
+      </c>
+      <c r="G1004" t="s">
         <v>3052</v>
-      </c>
-      <c r="G1004" t="s">
-        <v>3053</v>
       </c>
       <c r="H1004">
         <v>2</v>
       </c>
       <c r="I1004" t="s">
-        <v>3054</v>
+        <v>3053</v>
       </c>
       <c r="J1004" t="s">
         <v>2572</v>
@@ -51075,31 +51072,31 @@
     </row>
     <row r="1005" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1005" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1005" t="s">
         <v>3017</v>
       </c>
-      <c r="B1005" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1005" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1005" t="s">
         <v>3042</v>
-      </c>
-      <c r="D1005" t="s">
-        <v>3043</v>
       </c>
       <c r="E1005" t="s">
         <v>16</v>
       </c>
       <c r="F1005" t="s">
+        <v>3054</v>
+      </c>
+      <c r="G1005" t="s">
         <v>3055</v>
-      </c>
-      <c r="G1005" t="s">
-        <v>3056</v>
       </c>
       <c r="H1005">
         <v>2</v>
       </c>
       <c r="I1005" t="s">
-        <v>3057</v>
+        <v>3056</v>
       </c>
       <c r="J1005" t="s">
         <v>2399</v>
@@ -51116,31 +51113,31 @@
     </row>
     <row r="1006" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1006" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1006" t="s">
         <v>3017</v>
       </c>
-      <c r="B1006" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1006" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D1006" t="s">
         <v>3058</v>
-      </c>
-      <c r="D1006" t="s">
-        <v>3059</v>
       </c>
       <c r="E1006" t="s">
         <v>16</v>
       </c>
       <c r="F1006" t="s">
+        <v>3059</v>
+      </c>
+      <c r="G1006" t="s">
         <v>3060</v>
-      </c>
-      <c r="G1006" t="s">
-        <v>3061</v>
       </c>
       <c r="H1006">
         <v>2</v>
       </c>
       <c r="I1006" t="s">
-        <v>3062</v>
+        <v>3061</v>
       </c>
       <c r="J1006" t="s">
         <v>2572</v>
@@ -51157,31 +51154,31 @@
     </row>
     <row r="1007" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1007" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1007" t="s">
         <v>3017</v>
       </c>
-      <c r="B1007" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1007" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D1007" t="s">
         <v>3058</v>
-      </c>
-      <c r="D1007" t="s">
-        <v>3059</v>
       </c>
       <c r="E1007" t="s">
         <v>16</v>
       </c>
       <c r="F1007" t="s">
+        <v>3062</v>
+      </c>
+      <c r="G1007" t="s">
         <v>3063</v>
-      </c>
-      <c r="G1007" t="s">
-        <v>3064</v>
       </c>
       <c r="H1007">
         <v>2</v>
       </c>
       <c r="I1007" t="s">
-        <v>3025</v>
+        <v>3024</v>
       </c>
       <c r="J1007" t="s">
         <v>2399</v>
@@ -51190,7 +51187,7 @@
         <v>21</v>
       </c>
       <c r="L1007" t="s">
-        <v>3022</v>
+        <v>3021</v>
       </c>
       <c r="M1007" t="s">
         <v>23</v>
@@ -51198,31 +51195,31 @@
     </row>
     <row r="1008" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1008" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1008" t="s">
         <v>3017</v>
       </c>
-      <c r="B1008" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1008" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D1008" t="s">
         <v>3058</v>
-      </c>
-      <c r="D1008" t="s">
-        <v>3059</v>
       </c>
       <c r="E1008" t="s">
         <v>16</v>
       </c>
       <c r="F1008" t="s">
+        <v>3064</v>
+      </c>
+      <c r="G1008" t="s">
         <v>3065</v>
-      </c>
-      <c r="G1008" t="s">
-        <v>3066</v>
       </c>
       <c r="H1008">
         <v>2</v>
       </c>
       <c r="I1008" t="s">
-        <v>3067</v>
+        <v>3066</v>
       </c>
       <c r="J1008" t="s">
         <v>2572</v>
@@ -51239,25 +51236,25 @@
     </row>
     <row r="1009" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1009" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1009" t="s">
         <v>3017</v>
       </c>
-      <c r="B1009" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1009" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D1009" t="s">
         <v>3058</v>
-      </c>
-      <c r="D1009" t="s">
-        <v>3059</v>
       </c>
       <c r="E1009" t="s">
         <v>16</v>
       </c>
       <c r="F1009" t="s">
+        <v>3067</v>
+      </c>
+      <c r="G1009" t="s">
         <v>3068</v>
-      </c>
-      <c r="G1009" t="s">
-        <v>3069</v>
       </c>
       <c r="H1009">
         <v>2</v>
@@ -51272,7 +51269,7 @@
         <v>21</v>
       </c>
       <c r="L1009" t="s">
-        <v>3028</v>
+        <v>3027</v>
       </c>
       <c r="M1009" t="s">
         <v>23</v>
@@ -51280,22 +51277,22 @@
     </row>
     <row r="1010" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1010" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1010" t="s">
         <v>3017</v>
       </c>
-      <c r="B1010" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1010" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D1010" t="s">
         <v>3058</v>
-      </c>
-      <c r="D1010" t="s">
-        <v>3059</v>
       </c>
       <c r="E1010" t="s">
         <v>16</v>
       </c>
       <c r="F1010" t="s">
-        <v>3070</v>
+        <v>3069</v>
       </c>
       <c r="G1010" t="s">
         <v>460</v>
@@ -51304,7 +51301,7 @@
         <v>2</v>
       </c>
       <c r="I1010" t="s">
-        <v>3071</v>
+        <v>3070</v>
       </c>
       <c r="J1010" t="s">
         <v>2391</v>
@@ -51321,31 +51318,31 @@
     </row>
     <row r="1011" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1011" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1011" t="s">
         <v>3017</v>
       </c>
-      <c r="B1011" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1011" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D1011" t="s">
         <v>3058</v>
-      </c>
-      <c r="D1011" t="s">
-        <v>3059</v>
       </c>
       <c r="E1011" t="s">
         <v>16</v>
       </c>
       <c r="F1011" t="s">
+        <v>3071</v>
+      </c>
+      <c r="G1011" t="s">
         <v>3072</v>
-      </c>
-      <c r="G1011" t="s">
-        <v>3073</v>
       </c>
       <c r="H1011">
         <v>2</v>
       </c>
       <c r="I1011" t="s">
-        <v>3033</v>
+        <v>3032</v>
       </c>
       <c r="J1011" t="s">
         <v>2399</v>
@@ -51354,7 +51351,7 @@
         <v>21</v>
       </c>
       <c r="L1011" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M1011" t="s">
         <v>23</v>
@@ -51362,31 +51359,31 @@
     </row>
     <row r="1012" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1012" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1012" t="s">
         <v>3017</v>
       </c>
-      <c r="B1012" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1012" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1012" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1012" t="s">
-        <v>3075</v>
       </c>
       <c r="E1012" t="s">
         <v>16</v>
       </c>
       <c r="F1012" t="s">
+        <v>3075</v>
+      </c>
+      <c r="G1012" t="s">
         <v>3076</v>
-      </c>
-      <c r="G1012" t="s">
-        <v>3077</v>
       </c>
       <c r="H1012">
         <v>2</v>
       </c>
       <c r="I1012" t="s">
-        <v>3067</v>
+        <v>3066</v>
       </c>
       <c r="J1012" t="s">
         <v>813</v>
@@ -51395,7 +51392,7 @@
         <v>21</v>
       </c>
       <c r="L1012" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M1012" t="s">
         <v>23</v>
@@ -51403,40 +51400,40 @@
     </row>
     <row r="1013" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1013" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1013" t="s">
         <v>3017</v>
       </c>
-      <c r="B1013" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1013" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1013" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1013" t="s">
-        <v>3075</v>
       </c>
       <c r="E1013" t="s">
         <v>16</v>
       </c>
       <c r="F1013" t="s">
+        <v>3077</v>
+      </c>
+      <c r="G1013" t="s">
         <v>3078</v>
-      </c>
-      <c r="G1013" t="s">
-        <v>3079</v>
       </c>
       <c r="H1013">
         <v>2</v>
       </c>
       <c r="I1013" t="s">
+        <v>3079</v>
+      </c>
+      <c r="J1013" t="s">
         <v>3080</v>
       </c>
-      <c r="J1013" t="s">
-        <v>3081</v>
-      </c>
       <c r="K1013" t="s">
         <v>21</v>
       </c>
       <c r="L1013" t="s">
-        <v>3031</v>
+        <v>3030</v>
       </c>
       <c r="M1013" t="s">
         <v>23</v>
@@ -51444,31 +51441,31 @@
     </row>
     <row r="1014" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1014" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1014" t="s">
         <v>3017</v>
       </c>
-      <c r="B1014" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1014" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1014" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1014" t="s">
-        <v>3075</v>
       </c>
       <c r="E1014" t="s">
         <v>16</v>
       </c>
       <c r="F1014" t="s">
+        <v>3081</v>
+      </c>
+      <c r="G1014" t="s">
         <v>3082</v>
-      </c>
-      <c r="G1014" t="s">
-        <v>3083</v>
       </c>
       <c r="H1014">
         <v>2</v>
       </c>
       <c r="I1014" t="s">
-        <v>3062</v>
+        <v>3061</v>
       </c>
       <c r="J1014" t="s">
         <v>664</v>
@@ -51485,31 +51482,31 @@
     </row>
     <row r="1015" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1015" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1015" t="s">
         <v>3017</v>
       </c>
-      <c r="B1015" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1015" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1015" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1015" t="s">
-        <v>3075</v>
       </c>
       <c r="E1015" t="s">
         <v>16</v>
       </c>
       <c r="F1015" t="s">
+        <v>3083</v>
+      </c>
+      <c r="G1015" t="s">
         <v>3084</v>
-      </c>
-      <c r="G1015" t="s">
-        <v>3085</v>
       </c>
       <c r="H1015">
         <v>2</v>
       </c>
       <c r="I1015" t="s">
-        <v>3086</v>
+        <v>3085</v>
       </c>
       <c r="J1015" t="s">
         <v>2549</v>
@@ -51518,7 +51515,7 @@
         <v>21</v>
       </c>
       <c r="L1015" t="s">
-        <v>3087</v>
+        <v>3086</v>
       </c>
       <c r="M1015" t="s">
         <v>23</v>
@@ -51526,31 +51523,31 @@
     </row>
     <row r="1016" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1016" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1016" t="s">
         <v>3017</v>
       </c>
-      <c r="B1016" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1016" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1016" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1016" t="s">
-        <v>3075</v>
       </c>
       <c r="E1016" t="s">
         <v>16</v>
       </c>
       <c r="F1016" t="s">
+        <v>3087</v>
+      </c>
+      <c r="G1016" t="s">
         <v>3088</v>
-      </c>
-      <c r="G1016" t="s">
-        <v>3089</v>
       </c>
       <c r="H1016">
         <v>2</v>
       </c>
       <c r="I1016" t="s">
-        <v>3080</v>
+        <v>3079</v>
       </c>
       <c r="J1016" t="s">
         <v>2399</v>
@@ -51559,7 +51556,7 @@
         <v>21</v>
       </c>
       <c r="L1016" t="s">
-        <v>3087</v>
+        <v>3086</v>
       </c>
       <c r="M1016" t="s">
         <v>23</v>
@@ -51567,31 +51564,31 @@
     </row>
     <row r="1017" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1017" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1017" t="s">
         <v>3017</v>
       </c>
-      <c r="B1017" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1017" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1017" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1017" t="s">
-        <v>3075</v>
       </c>
       <c r="E1017" t="s">
         <v>16</v>
       </c>
       <c r="F1017" t="s">
+        <v>3089</v>
+      </c>
+      <c r="G1017" t="s">
         <v>3090</v>
-      </c>
-      <c r="G1017" t="s">
-        <v>3091</v>
       </c>
       <c r="H1017">
         <v>2</v>
       </c>
       <c r="I1017" t="s">
-        <v>3035</v>
+        <v>3034</v>
       </c>
       <c r="J1017" t="s">
         <v>2549</v>
@@ -51608,31 +51605,31 @@
     </row>
     <row r="1018" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1018" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1018" t="s">
         <v>3017</v>
       </c>
-      <c r="B1018" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1018" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1018" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1018" t="s">
-        <v>3075</v>
       </c>
       <c r="E1018" t="s">
         <v>16</v>
       </c>
       <c r="F1018" t="s">
+        <v>3091</v>
+      </c>
+      <c r="G1018" t="s">
         <v>3092</v>
-      </c>
-      <c r="G1018" t="s">
-        <v>3093</v>
       </c>
       <c r="H1018">
         <v>2</v>
       </c>
       <c r="I1018" t="s">
-        <v>3094</v>
+        <v>3093</v>
       </c>
       <c r="J1018" t="s">
         <v>2391</v>
@@ -51641,7 +51638,7 @@
         <v>21</v>
       </c>
       <c r="L1018" t="s">
-        <v>3087</v>
+        <v>3086</v>
       </c>
       <c r="M1018" t="s">
         <v>23</v>
@@ -51649,31 +51646,31 @@
     </row>
     <row r="1019" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1019" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1019" t="s">
         <v>3017</v>
       </c>
-      <c r="B1019" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1019" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1019" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1019" t="s">
-        <v>3075</v>
       </c>
       <c r="E1019" t="s">
         <v>16</v>
       </c>
       <c r="F1019" t="s">
+        <v>3094</v>
+      </c>
+      <c r="G1019" t="s">
         <v>3095</v>
-      </c>
-      <c r="G1019" t="s">
-        <v>3096</v>
       </c>
       <c r="H1019">
         <v>2</v>
       </c>
       <c r="I1019" t="s">
-        <v>3048</v>
+        <v>3047</v>
       </c>
       <c r="J1019" t="s">
         <v>2391</v>
@@ -51690,31 +51687,31 @@
     </row>
     <row r="1020" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1020" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B1020" t="s">
         <v>3017</v>
       </c>
-      <c r="B1020" t="s">
-        <v>3018</v>
-      </c>
       <c r="C1020" t="s">
+        <v>3073</v>
+      </c>
+      <c r="D1020" t="s">
         <v>3074</v>
-      </c>
-      <c r="D1020" t="s">
-        <v>3075</v>
       </c>
       <c r="E1020" t="s">
         <v>16</v>
       </c>
       <c r="F1020" t="s">
+        <v>3096</v>
+      </c>
+      <c r="G1020" t="s">
         <v>3097</v>
-      </c>
-      <c r="G1020" t="s">
-        <v>3098</v>
       </c>
       <c r="H1020">
         <v>2</v>
       </c>
       <c r="I1020" t="s">
-        <v>3035</v>
+        <v>3034</v>
       </c>
       <c r="J1020" t="s">
         <v>2572</v>
@@ -51723,7 +51720,7 @@
         <v>21</v>
       </c>
       <c r="L1020" t="s">
-        <v>3087</v>
+        <v>3086</v>
       </c>
       <c r="M1020" t="s">
         <v>23</v>
@@ -51731,13 +51728,13 @@
     </row>
     <row r="1021" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1021" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1021" t="s">
         <v>3099</v>
       </c>
-      <c r="B1021" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1021" t="s">
-        <v>3099</v>
+        <v>3098</v>
       </c>
       <c r="D1021" t="s">
         <v>15</v>
@@ -51746,16 +51743,16 @@
         <v>1732</v>
       </c>
       <c r="F1021" t="s">
+        <v>3100</v>
+      </c>
+      <c r="G1021" t="s">
         <v>3101</v>
-      </c>
-      <c r="G1021" t="s">
-        <v>3102</v>
       </c>
       <c r="H1021">
         <v>2</v>
       </c>
       <c r="I1021" t="s">
-        <v>3103</v>
+        <v>3102</v>
       </c>
       <c r="J1021" t="s">
         <v>2399</v>
@@ -51772,34 +51769,34 @@
     </row>
     <row r="1022" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1022" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1022" t="s">
         <v>3099</v>
       </c>
-      <c r="B1022" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1022" t="s">
+        <v>3103</v>
+      </c>
+      <c r="D1022" t="s">
         <v>3104</v>
-      </c>
-      <c r="D1022" t="s">
-        <v>3105</v>
       </c>
       <c r="E1022" t="s">
         <v>16</v>
       </c>
       <c r="F1022" t="s">
+        <v>3105</v>
+      </c>
+      <c r="G1022" t="s">
         <v>3106</v>
-      </c>
-      <c r="G1022" t="s">
-        <v>3107</v>
       </c>
       <c r="H1022">
         <v>2</v>
       </c>
       <c r="I1022" t="s">
+        <v>3107</v>
+      </c>
+      <c r="J1022" t="s">
         <v>3108</v>
-      </c>
-      <c r="J1022" t="s">
-        <v>3109</v>
       </c>
       <c r="K1022" t="s">
         <v>21</v>
@@ -51813,25 +51810,25 @@
     </row>
     <row r="1023" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1023" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1023" t="s">
         <v>3099</v>
       </c>
-      <c r="B1023" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1023" t="s">
+        <v>3109</v>
+      </c>
+      <c r="D1023" t="s">
         <v>3110</v>
-      </c>
-      <c r="D1023" t="s">
-        <v>3111</v>
       </c>
       <c r="E1023" t="s">
         <v>16</v>
       </c>
       <c r="F1023" t="s">
+        <v>3111</v>
+      </c>
+      <c r="G1023" t="s">
         <v>3112</v>
-      </c>
-      <c r="G1023" t="s">
-        <v>3113</v>
       </c>
       <c r="H1023">
         <v>2</v>
@@ -51846,7 +51843,7 @@
         <v>21</v>
       </c>
       <c r="L1023" t="s">
-        <v>3114</v>
+        <v>3113</v>
       </c>
       <c r="M1023" t="s">
         <v>23</v>
@@ -51854,31 +51851,31 @@
     </row>
     <row r="1024" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1024" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1024" t="s">
         <v>3099</v>
       </c>
-      <c r="B1024" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1024" t="s">
+        <v>3109</v>
+      </c>
+      <c r="D1024" t="s">
         <v>3110</v>
-      </c>
-      <c r="D1024" t="s">
-        <v>3111</v>
       </c>
       <c r="E1024" t="s">
         <v>16</v>
       </c>
       <c r="F1024" t="s">
+        <v>3114</v>
+      </c>
+      <c r="G1024" t="s">
         <v>3115</v>
-      </c>
-      <c r="G1024" t="s">
-        <v>3116</v>
       </c>
       <c r="H1024">
         <v>2</v>
       </c>
       <c r="I1024" t="s">
-        <v>3117</v>
+        <v>3116</v>
       </c>
       <c r="J1024" t="s">
         <v>2391</v>
@@ -51895,34 +51892,34 @@
     </row>
     <row r="1025" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1025" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1025" t="s">
         <v>3099</v>
       </c>
-      <c r="B1025" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1025" t="s">
+        <v>3109</v>
+      </c>
+      <c r="D1025" t="s">
         <v>3110</v>
-      </c>
-      <c r="D1025" t="s">
-        <v>3111</v>
       </c>
       <c r="E1025" t="s">
         <v>16</v>
       </c>
       <c r="F1025" t="s">
+        <v>3117</v>
+      </c>
+      <c r="G1025" t="s">
         <v>3118</v>
-      </c>
-      <c r="G1025" t="s">
-        <v>3119</v>
       </c>
       <c r="H1025">
         <v>2</v>
       </c>
       <c r="I1025" t="s">
-        <v>3120</v>
+        <v>3119</v>
       </c>
       <c r="J1025" t="s">
-        <v>3109</v>
+        <v>3108</v>
       </c>
       <c r="K1025" t="s">
         <v>21</v>
@@ -51936,31 +51933,31 @@
     </row>
     <row r="1026" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1026" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1026" t="s">
         <v>3099</v>
       </c>
-      <c r="B1026" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1026" t="s">
+        <v>3109</v>
+      </c>
+      <c r="D1026" t="s">
         <v>3110</v>
-      </c>
-      <c r="D1026" t="s">
-        <v>3111</v>
       </c>
       <c r="E1026" t="s">
         <v>16</v>
       </c>
       <c r="F1026" t="s">
+        <v>3120</v>
+      </c>
+      <c r="G1026" t="s">
         <v>3121</v>
-      </c>
-      <c r="G1026" t="s">
-        <v>3122</v>
       </c>
       <c r="H1026">
         <v>2</v>
       </c>
       <c r="I1026" t="s">
-        <v>3123</v>
+        <v>3122</v>
       </c>
       <c r="J1026" t="s">
         <v>1959</v>
@@ -51969,7 +51966,7 @@
         <v>21</v>
       </c>
       <c r="L1026" t="s">
-        <v>3124</v>
+        <v>3123</v>
       </c>
       <c r="M1026" t="s">
         <v>23</v>
@@ -51977,34 +51974,34 @@
     </row>
     <row r="1027" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1027" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1027" t="s">
         <v>3099</v>
       </c>
-      <c r="B1027" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1027" t="s">
+        <v>3124</v>
+      </c>
+      <c r="D1027" t="s">
         <v>3125</v>
-      </c>
-      <c r="D1027" t="s">
-        <v>3126</v>
       </c>
       <c r="E1027" t="s">
         <v>16</v>
       </c>
       <c r="F1027" t="s">
+        <v>3126</v>
+      </c>
+      <c r="G1027" t="s">
         <v>3127</v>
-      </c>
-      <c r="G1027" t="s">
-        <v>3128</v>
       </c>
       <c r="H1027">
         <v>2</v>
       </c>
       <c r="I1027" t="s">
+        <v>3128</v>
+      </c>
+      <c r="J1027" t="s">
         <v>3129</v>
-      </c>
-      <c r="J1027" t="s">
-        <v>3130</v>
       </c>
       <c r="K1027" t="s">
         <v>21</v>
@@ -52018,31 +52015,31 @@
     </row>
     <row r="1028" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1028" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1028" t="s">
         <v>3099</v>
       </c>
-      <c r="B1028" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1028" t="s">
+        <v>3124</v>
+      </c>
+      <c r="D1028" t="s">
         <v>3125</v>
-      </c>
-      <c r="D1028" t="s">
-        <v>3126</v>
       </c>
       <c r="E1028" t="s">
         <v>16</v>
       </c>
       <c r="F1028" t="s">
+        <v>3130</v>
+      </c>
+      <c r="G1028" t="s">
         <v>3131</v>
-      </c>
-      <c r="G1028" t="s">
-        <v>3132</v>
       </c>
       <c r="H1028">
         <v>2</v>
       </c>
       <c r="I1028" t="s">
-        <v>3129</v>
+        <v>3128</v>
       </c>
       <c r="J1028" t="s">
         <v>1903</v>
@@ -52051,7 +52048,7 @@
         <v>21</v>
       </c>
       <c r="L1028" t="s">
-        <v>3124</v>
+        <v>3123</v>
       </c>
       <c r="M1028" t="s">
         <v>23</v>
@@ -52059,34 +52056,34 @@
     </row>
     <row r="1029" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1029" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1029" t="s">
         <v>3099</v>
       </c>
-      <c r="B1029" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1029" t="s">
+        <v>3124</v>
+      </c>
+      <c r="D1029" t="s">
         <v>3125</v>
-      </c>
-      <c r="D1029" t="s">
-        <v>3126</v>
       </c>
       <c r="E1029" t="s">
         <v>16</v>
       </c>
       <c r="F1029" t="s">
+        <v>3132</v>
+      </c>
+      <c r="G1029" t="s">
         <v>3133</v>
-      </c>
-      <c r="G1029" t="s">
-        <v>3134</v>
       </c>
       <c r="H1029">
         <v>2</v>
       </c>
       <c r="I1029" t="s">
-        <v>3103</v>
+        <v>3102</v>
       </c>
       <c r="J1029" t="s">
-        <v>3135</v>
+        <v>3134</v>
       </c>
       <c r="K1029" t="s">
         <v>21</v>
@@ -52100,31 +52097,31 @@
     </row>
     <row r="1030" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1030" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1030" t="s">
         <v>3099</v>
       </c>
-      <c r="B1030" t="s">
-        <v>3100</v>
-      </c>
       <c r="C1030" t="s">
+        <v>3124</v>
+      </c>
+      <c r="D1030" t="s">
         <v>3125</v>
-      </c>
-      <c r="D1030" t="s">
-        <v>3126</v>
       </c>
       <c r="E1030" t="s">
         <v>16</v>
       </c>
       <c r="F1030" t="s">
+        <v>3135</v>
+      </c>
+      <c r="G1030" t="s">
         <v>3136</v>
-      </c>
-      <c r="G1030" t="s">
-        <v>3137</v>
       </c>
       <c r="H1030">
         <v>2</v>
       </c>
       <c r="I1030" t="s">
-        <v>3138</v>
+        <v>3137</v>
       </c>
       <c r="J1030" t="s">
         <v>2391</v>
@@ -52141,13 +52138,13 @@
     </row>
     <row r="1031" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1031" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1031" t="s">
         <v>3139</v>
       </c>
-      <c r="B1031" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1031" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1031" t="s">
         <v>15</v>
@@ -52156,16 +52153,16 @@
         <v>1732</v>
       </c>
       <c r="F1031" t="s">
+        <v>3140</v>
+      </c>
+      <c r="G1031" t="s">
         <v>3141</v>
       </c>
-      <c r="G1031" t="s">
+      <c r="H1031">
+        <v>3</v>
+      </c>
+      <c r="I1031" t="s">
         <v>3142</v>
-      </c>
-      <c r="H1031">
-        <v>3</v>
-      </c>
-      <c r="I1031" t="s">
-        <v>3143</v>
       </c>
       <c r="J1031" t="s">
         <v>1761</v>
@@ -52174,7 +52171,7 @@
         <v>21</v>
       </c>
       <c r="L1031" t="s">
-        <v>3144</v>
+        <v>3143</v>
       </c>
       <c r="M1031" t="s">
         <v>23</v>
@@ -52182,13 +52179,13 @@
     </row>
     <row r="1032" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1032" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1032" t="s">
         <v>3139</v>
       </c>
-      <c r="B1032" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1032" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1032" t="s">
         <v>15</v>
@@ -52197,10 +52194,10 @@
         <v>16</v>
       </c>
       <c r="F1032" t="s">
+        <v>3144</v>
+      </c>
+      <c r="G1032" t="s">
         <v>3145</v>
-      </c>
-      <c r="G1032" t="s">
-        <v>3146</v>
       </c>
       <c r="H1032">
         <v>3</v>
@@ -52215,7 +52212,7 @@
         <v>21</v>
       </c>
       <c r="L1032" t="s">
-        <v>3144</v>
+        <v>3143</v>
       </c>
       <c r="M1032" t="s">
         <v>23</v>
@@ -52223,13 +52220,13 @@
     </row>
     <row r="1033" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1033" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1033" t="s">
         <v>3139</v>
       </c>
-      <c r="B1033" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1033" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1033" t="s">
         <v>15</v>
@@ -52238,10 +52235,10 @@
         <v>16</v>
       </c>
       <c r="F1033" t="s">
+        <v>3146</v>
+      </c>
+      <c r="G1033" t="s">
         <v>3147</v>
-      </c>
-      <c r="G1033" t="s">
-        <v>3148</v>
       </c>
       <c r="H1033">
         <v>3</v>
@@ -52256,7 +52253,7 @@
         <v>21</v>
       </c>
       <c r="L1033" t="s">
-        <v>3149</v>
+        <v>3148</v>
       </c>
       <c r="M1033" t="s">
         <v>23</v>
@@ -52264,13 +52261,13 @@
     </row>
     <row r="1034" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1034" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1034" t="s">
         <v>3139</v>
       </c>
-      <c r="B1034" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1034" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1034" t="s">
         <v>15</v>
@@ -52279,10 +52276,10 @@
         <v>1732</v>
       </c>
       <c r="F1034" t="s">
+        <v>3149</v>
+      </c>
+      <c r="G1034" t="s">
         <v>3150</v>
-      </c>
-      <c r="G1034" t="s">
-        <v>3151</v>
       </c>
       <c r="H1034">
         <v>3</v>
@@ -52297,7 +52294,7 @@
         <v>325</v>
       </c>
       <c r="L1034" t="s">
-        <v>3152</v>
+        <v>3151</v>
       </c>
       <c r="M1034" t="s">
         <v>23</v>
@@ -52305,13 +52302,13 @@
     </row>
     <row r="1035" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1035" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1035" t="s">
         <v>3139</v>
       </c>
-      <c r="B1035" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1035" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1035" t="s">
         <v>15</v>
@@ -52320,10 +52317,10 @@
         <v>2539</v>
       </c>
       <c r="F1035" t="s">
+        <v>3152</v>
+      </c>
+      <c r="G1035" t="s">
         <v>3153</v>
-      </c>
-      <c r="G1035" t="s">
-        <v>3154</v>
       </c>
       <c r="H1035">
         <v>3</v>
@@ -52338,7 +52335,7 @@
         <v>325</v>
       </c>
       <c r="L1035" t="s">
-        <v>3152</v>
+        <v>3151</v>
       </c>
       <c r="M1035" t="s">
         <v>23</v>
@@ -52346,13 +52343,13 @@
     </row>
     <row r="1036" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1036" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1036" t="s">
         <v>3139</v>
       </c>
-      <c r="B1036" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1036" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1036" t="s">
         <v>15</v>
@@ -52361,10 +52358,10 @@
         <v>1732</v>
       </c>
       <c r="F1036" t="s">
+        <v>3154</v>
+      </c>
+      <c r="G1036" t="s">
         <v>3155</v>
-      </c>
-      <c r="G1036" t="s">
-        <v>3156</v>
       </c>
       <c r="H1036">
         <v>3</v>
@@ -52379,7 +52376,7 @@
         <v>325</v>
       </c>
       <c r="L1036" t="s">
-        <v>3152</v>
+        <v>3151</v>
       </c>
       <c r="M1036" t="s">
         <v>23</v>
@@ -52387,13 +52384,13 @@
     </row>
     <row r="1037" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1037" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1037" t="s">
         <v>3139</v>
       </c>
-      <c r="B1037" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1037" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="D1037" t="s">
         <v>15</v>
@@ -52402,10 +52399,10 @@
         <v>1732</v>
       </c>
       <c r="F1037" t="s">
+        <v>3156</v>
+      </c>
+      <c r="G1037" t="s">
         <v>3157</v>
-      </c>
-      <c r="G1037" t="s">
-        <v>3158</v>
       </c>
       <c r="H1037">
         <v>3</v>
@@ -52420,7 +52417,7 @@
         <v>325</v>
       </c>
       <c r="L1037" t="s">
-        <v>3152</v>
+        <v>3151</v>
       </c>
       <c r="M1037" t="s">
         <v>23</v>
@@ -52428,25 +52425,25 @@
     </row>
     <row r="1038" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1038" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1038" t="s">
         <v>3139</v>
       </c>
-      <c r="B1038" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1038" t="s">
+        <v>3158</v>
+      </c>
+      <c r="D1038" t="s">
         <v>3159</v>
-      </c>
-      <c r="D1038" t="s">
-        <v>3160</v>
       </c>
       <c r="E1038" t="s">
         <v>16</v>
       </c>
       <c r="F1038" t="s">
+        <v>3160</v>
+      </c>
+      <c r="G1038" t="s">
         <v>3161</v>
-      </c>
-      <c r="G1038" t="s">
-        <v>3162</v>
       </c>
       <c r="H1038">
         <v>3</v>
@@ -52461,7 +52458,7 @@
         <v>21</v>
       </c>
       <c r="L1038" t="s">
-        <v>3149</v>
+        <v>3148</v>
       </c>
       <c r="M1038" t="s">
         <v>23</v>
@@ -52469,25 +52466,25 @@
     </row>
     <row r="1039" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1039" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1039" t="s">
         <v>3139</v>
       </c>
-      <c r="B1039" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1039" t="s">
+        <v>3158</v>
+      </c>
+      <c r="D1039" t="s">
         <v>3159</v>
-      </c>
-      <c r="D1039" t="s">
-        <v>3160</v>
       </c>
       <c r="E1039" t="s">
         <v>16</v>
       </c>
       <c r="F1039" t="s">
+        <v>3162</v>
+      </c>
+      <c r="G1039" t="s">
         <v>3163</v>
-      </c>
-      <c r="G1039" t="s">
-        <v>3164</v>
       </c>
       <c r="H1039">
         <v>3</v>
@@ -52502,7 +52499,7 @@
         <v>21</v>
       </c>
       <c r="L1039" t="s">
-        <v>3149</v>
+        <v>3148</v>
       </c>
       <c r="M1039" t="s">
         <v>23</v>
@@ -52510,31 +52507,31 @@
     </row>
     <row r="1040" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1040" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1040" t="s">
         <v>3139</v>
       </c>
-      <c r="B1040" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1040" t="s">
+        <v>3164</v>
+      </c>
+      <c r="D1040" t="s">
         <v>3165</v>
-      </c>
-      <c r="D1040" t="s">
-        <v>3166</v>
       </c>
       <c r="E1040" t="s">
         <v>16</v>
       </c>
       <c r="F1040" t="s">
+        <v>3166</v>
+      </c>
+      <c r="G1040" t="s">
         <v>3167</v>
       </c>
-      <c r="G1040" t="s">
+      <c r="H1040">
+        <v>3</v>
+      </c>
+      <c r="I1040" t="s">
         <v>3168</v>
-      </c>
-      <c r="H1040">
-        <v>3</v>
-      </c>
-      <c r="I1040" t="s">
-        <v>3169</v>
       </c>
       <c r="J1040" t="s">
         <v>1345</v>
@@ -52543,7 +52540,7 @@
         <v>21</v>
       </c>
       <c r="L1040" t="s">
-        <v>3144</v>
+        <v>3143</v>
       </c>
       <c r="M1040" t="s">
         <v>23</v>
@@ -52551,31 +52548,31 @@
     </row>
     <row r="1041" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1041" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1041" t="s">
         <v>3139</v>
       </c>
-      <c r="B1041" t="s">
-        <v>3140</v>
-      </c>
       <c r="C1041" t="s">
+        <v>3164</v>
+      </c>
+      <c r="D1041" t="s">
         <v>3165</v>
-      </c>
-      <c r="D1041" t="s">
-        <v>3166</v>
       </c>
       <c r="E1041" t="s">
         <v>16</v>
       </c>
       <c r="F1041" t="s">
+        <v>3169</v>
+      </c>
+      <c r="G1041" t="s">
         <v>3170</v>
       </c>
-      <c r="G1041" t="s">
+      <c r="H1041">
+        <v>3</v>
+      </c>
+      <c r="I1041" t="s">
         <v>3171</v>
-      </c>
-      <c r="H1041">
-        <v>3</v>
-      </c>
-      <c r="I1041" t="s">
-        <v>3172</v>
       </c>
       <c r="J1041" t="s">
         <v>1776</v>
@@ -52584,7 +52581,7 @@
         <v>21</v>
       </c>
       <c r="L1041" t="s">
-        <v>3144</v>
+        <v>3143</v>
       </c>
       <c r="M1041" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-09-17T23:38Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -4531,7 +4531,7 @@
     <t>홍성지</t>
   </si>
   <si>
-    <t>월 10:30-12:00,수 10:00-12:00</t>
+    <t>월 10:30-12:00,수 10:30-12:00</t>
   </si>
   <si>
     <t>조형관별관3층6호실</t>
@@ -4543,7 +4543,7 @@
     <t>초급한국어2</t>
   </si>
   <si>
-    <t>화 10:30-12:00,목 10:00-12:00</t>
+    <t>화 10:30-12:00,목 10:30-12:00</t>
   </si>
   <si>
     <t>조형관별관2층2호실</t>
@@ -32573,7 +32573,7 @@
         <v>21</v>
       </c>
       <c r="L553" t="s">
-        <v>1624</v>
+        <v>1550</v>
       </c>
       <c r="M553" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-10-09T01:21Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -4630,352 +4630,352 @@
     <t>진황가</t>
   </si>
   <si>
+    <t>조형관별관3층5호실</t>
+  </si>
+  <si>
+    <t>36277</t>
+  </si>
+  <si>
+    <t>스마트경험디자인학과</t>
+  </si>
+  <si>
+    <t>704140b</t>
+  </si>
+  <si>
+    <t>논문ㆍ작품지도</t>
+  </si>
+  <si>
+    <t>연명흠</t>
+  </si>
+  <si>
+    <t>수 18:55-21:35</t>
+  </si>
+  <si>
+    <t>조형관별관1층5호실</t>
+  </si>
+  <si>
+    <t>704150a</t>
+  </si>
+  <si>
+    <t>논문지도1</t>
+  </si>
+  <si>
+    <t>목 18:55-21:35</t>
+  </si>
+  <si>
+    <t>조형관별관3층4호실</t>
+  </si>
+  <si>
+    <t>704160a</t>
+  </si>
+  <si>
+    <t>논문지도2</t>
+  </si>
+  <si>
+    <t>임진호</t>
+  </si>
+  <si>
+    <t>689070a</t>
+  </si>
+  <si>
+    <t>인터랙션디자인2</t>
+  </si>
+  <si>
+    <t>김수진</t>
+  </si>
+  <si>
+    <t>조형관별관3층3호실</t>
+  </si>
+  <si>
+    <t>689430a</t>
+  </si>
+  <si>
+    <t>서비스디자인2</t>
+  </si>
+  <si>
+    <t>정진열</t>
+  </si>
+  <si>
+    <t>화 18:55-21:35</t>
+  </si>
+  <si>
+    <t>696070a</t>
+  </si>
+  <si>
+    <t>디자인조사분석연습</t>
+  </si>
+  <si>
+    <t>조형관별관3층2호실</t>
+  </si>
+  <si>
+    <t>스튜디오</t>
+  </si>
+  <si>
+    <t>7204501</t>
+  </si>
+  <si>
+    <t>로컬플래닝 스튜디오 2</t>
+  </si>
+  <si>
+    <t>토 10:00-16:00</t>
+  </si>
+  <si>
+    <t>7204601</t>
+  </si>
+  <si>
+    <t>기술융합디자인논제 2</t>
+  </si>
+  <si>
+    <t>정치훈</t>
+  </si>
+  <si>
+    <t>7219501</t>
+  </si>
+  <si>
+    <t>도시공간론2</t>
+  </si>
+  <si>
+    <t>이용원</t>
+  </si>
+  <si>
+    <t>월 18:55-21:35</t>
+  </si>
+  <si>
+    <t>7231401</t>
+  </si>
+  <si>
+    <t>인공지능 활용 디자인</t>
+  </si>
+  <si>
+    <t>7244101</t>
+  </si>
+  <si>
+    <t>AI-XR 디자인</t>
+  </si>
+  <si>
+    <t>한주현</t>
+  </si>
+  <si>
+    <t>7249001</t>
+  </si>
+  <si>
+    <t>로컬혁신세미나2</t>
+  </si>
+  <si>
+    <t>7253701</t>
+  </si>
+  <si>
+    <t>기후변화와 서비스디자인</t>
+  </si>
+  <si>
+    <t>유채문</t>
+  </si>
+  <si>
+    <t>7260501</t>
+  </si>
+  <si>
+    <t>인클루시브 디자인</t>
+  </si>
+  <si>
+    <t>7286301</t>
+  </si>
+  <si>
+    <t>인간-인공지능 협업디자인 스튜디오2</t>
+  </si>
+  <si>
+    <t>허정윤</t>
+  </si>
+  <si>
+    <t>월 14:00-17:00,수 10:00-13:00</t>
+  </si>
+  <si>
+    <t>조형관별관3층10호실,조형관별관3층2호실</t>
+  </si>
+  <si>
+    <t>7295401</t>
+  </si>
+  <si>
+    <t>AI콘텐츠디자인스튜디오1</t>
+  </si>
+  <si>
+    <t>권주영</t>
+  </si>
+  <si>
+    <t>월 14:00-19:45</t>
+  </si>
+  <si>
+    <t>김진영</t>
+  </si>
+  <si>
+    <t>월 10:00-13:00,목 10:00-13:00</t>
+  </si>
+  <si>
+    <t>7295501</t>
+  </si>
+  <si>
+    <t>AI 시대의 인간이해</t>
+  </si>
+  <si>
+    <t>7295601</t>
+  </si>
+  <si>
+    <t>Agentic UX디자인</t>
+  </si>
+  <si>
+    <t>7295701</t>
+  </si>
+  <si>
+    <t>서비스디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>조만수</t>
+  </si>
+  <si>
+    <t>월 10:00-13:00,수 10:00-13:00</t>
+  </si>
+  <si>
+    <t>7295901</t>
+  </si>
+  <si>
+    <t>사운드경험디자인</t>
+  </si>
+  <si>
+    <t>남궁기찬</t>
+  </si>
+  <si>
+    <t>월 11:00-14:00</t>
+  </si>
+  <si>
+    <t>7296001</t>
+  </si>
+  <si>
+    <t>제품서비스시스템디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>심유리</t>
+  </si>
+  <si>
+    <t>월 10:00-17:00</t>
+  </si>
+  <si>
+    <t>7296101</t>
+  </si>
+  <si>
+    <t>정보디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>허정현</t>
+  </si>
+  <si>
+    <t>월 18:00-20:40,수 14:30-17:30</t>
+  </si>
+  <si>
+    <t>조형관별관3층3호실,조형관별관3층10호실</t>
+  </si>
+  <si>
+    <t>7296201</t>
+  </si>
+  <si>
+    <t>공공서비스디자인</t>
+  </si>
+  <si>
+    <t>박순정</t>
+  </si>
+  <si>
+    <t>조형관별관3층9호실</t>
+  </si>
+  <si>
+    <t>7296301</t>
+  </si>
+  <si>
+    <t>정량연구방법</t>
+  </si>
+  <si>
+    <t>36320</t>
+  </si>
+  <si>
+    <t>공간ㆍ문화디자인학과</t>
+  </si>
+  <si>
+    <t>704200b</t>
+  </si>
+  <si>
+    <t>7243701</t>
+  </si>
+  <si>
+    <t>특수연구과제2</t>
+  </si>
+  <si>
+    <t>윤성호</t>
+  </si>
+  <si>
+    <t>조형관별관3층14호실</t>
+  </si>
+  <si>
+    <t>7294501</t>
+  </si>
+  <si>
+    <t>7295101</t>
+  </si>
+  <si>
+    <t>강민선</t>
+  </si>
+  <si>
+    <t>707590a</t>
+  </si>
+  <si>
+    <t>소재 융합 개발 연구</t>
+  </si>
+  <si>
+    <t>이순정</t>
+  </si>
+  <si>
+    <t>토 10:00-13:00</t>
+  </si>
+  <si>
+    <t>7129001</t>
+  </si>
+  <si>
+    <t>디자인리서치&amp;방법론</t>
+  </si>
+  <si>
+    <t>7192201</t>
+  </si>
+  <si>
+    <t>글로벌 디자인 워크샵</t>
+  </si>
+  <si>
+    <t>정상엽</t>
+  </si>
+  <si>
+    <t>7192301</t>
+  </si>
+  <si>
+    <t>공간디자인 리서치 1</t>
+  </si>
+  <si>
+    <t>고은주</t>
+  </si>
+  <si>
+    <t>7243801</t>
+  </si>
+  <si>
+    <t>현대도시디자인</t>
+  </si>
+  <si>
+    <t>김상호</t>
+  </si>
+  <si>
+    <t>7262401</t>
+  </si>
+  <si>
+    <t>사진과 문화공간</t>
+  </si>
+  <si>
+    <t>김규랑</t>
+  </si>
+  <si>
     <t>조형관별관3층7호실</t>
-  </si>
-  <si>
-    <t>36277</t>
-  </si>
-  <si>
-    <t>스마트경험디자인학과</t>
-  </si>
-  <si>
-    <t>704140b</t>
-  </si>
-  <si>
-    <t>논문ㆍ작품지도</t>
-  </si>
-  <si>
-    <t>연명흠</t>
-  </si>
-  <si>
-    <t>수 18:55-21:35</t>
-  </si>
-  <si>
-    <t>조형관별관1층5호실</t>
-  </si>
-  <si>
-    <t>704150a</t>
-  </si>
-  <si>
-    <t>논문지도1</t>
-  </si>
-  <si>
-    <t>목 18:55-21:35</t>
-  </si>
-  <si>
-    <t>조형관별관3층4호실</t>
-  </si>
-  <si>
-    <t>704160a</t>
-  </si>
-  <si>
-    <t>논문지도2</t>
-  </si>
-  <si>
-    <t>임진호</t>
-  </si>
-  <si>
-    <t>조형관별관3층5호실</t>
-  </si>
-  <si>
-    <t>689070a</t>
-  </si>
-  <si>
-    <t>인터랙션디자인2</t>
-  </si>
-  <si>
-    <t>김수진</t>
-  </si>
-  <si>
-    <t>조형관별관3층3호실</t>
-  </si>
-  <si>
-    <t>689430a</t>
-  </si>
-  <si>
-    <t>서비스디자인2</t>
-  </si>
-  <si>
-    <t>정진열</t>
-  </si>
-  <si>
-    <t>화 18:55-21:35</t>
-  </si>
-  <si>
-    <t>696070a</t>
-  </si>
-  <si>
-    <t>디자인조사분석연습</t>
-  </si>
-  <si>
-    <t>조형관별관3층2호실</t>
-  </si>
-  <si>
-    <t>스튜디오</t>
-  </si>
-  <si>
-    <t>7204501</t>
-  </si>
-  <si>
-    <t>로컬플래닝 스튜디오 2</t>
-  </si>
-  <si>
-    <t>토 10:00-16:00</t>
-  </si>
-  <si>
-    <t>7204601</t>
-  </si>
-  <si>
-    <t>기술융합디자인논제 2</t>
-  </si>
-  <si>
-    <t>정치훈</t>
-  </si>
-  <si>
-    <t>7219501</t>
-  </si>
-  <si>
-    <t>도시공간론2</t>
-  </si>
-  <si>
-    <t>이용원</t>
-  </si>
-  <si>
-    <t>월 18:55-21:35</t>
-  </si>
-  <si>
-    <t>7231401</t>
-  </si>
-  <si>
-    <t>인공지능 활용 디자인</t>
-  </si>
-  <si>
-    <t>7244101</t>
-  </si>
-  <si>
-    <t>AI-XR 디자인</t>
-  </si>
-  <si>
-    <t>한주현</t>
-  </si>
-  <si>
-    <t>7249001</t>
-  </si>
-  <si>
-    <t>로컬혁신세미나2</t>
-  </si>
-  <si>
-    <t>7253701</t>
-  </si>
-  <si>
-    <t>기후변화와 서비스디자인</t>
-  </si>
-  <si>
-    <t>유채문</t>
-  </si>
-  <si>
-    <t>7260501</t>
-  </si>
-  <si>
-    <t>인클루시브 디자인</t>
-  </si>
-  <si>
-    <t>7286301</t>
-  </si>
-  <si>
-    <t>인간-인공지능 협업디자인 스튜디오2</t>
-  </si>
-  <si>
-    <t>허정윤</t>
-  </si>
-  <si>
-    <t>월 14:00-17:00,수 10:00-13:00</t>
-  </si>
-  <si>
-    <t>조형관별관3층10호실,조형관별관3층2호실</t>
-  </si>
-  <si>
-    <t>7295401</t>
-  </si>
-  <si>
-    <t>AI콘텐츠디자인스튜디오1</t>
-  </si>
-  <si>
-    <t>권주영</t>
-  </si>
-  <si>
-    <t>월 14:00-19:45</t>
-  </si>
-  <si>
-    <t>김진영</t>
-  </si>
-  <si>
-    <t>월 10:00-13:00,목 10:00-13:00</t>
-  </si>
-  <si>
-    <t>7295501</t>
-  </si>
-  <si>
-    <t>AI 시대의 인간이해</t>
-  </si>
-  <si>
-    <t>7295601</t>
-  </si>
-  <si>
-    <t>Agentic UX디자인</t>
-  </si>
-  <si>
-    <t>7295701</t>
-  </si>
-  <si>
-    <t>서비스디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>조만수</t>
-  </si>
-  <si>
-    <t>월 10:00-13:00,수 10:00-13:00</t>
-  </si>
-  <si>
-    <t>7295901</t>
-  </si>
-  <si>
-    <t>사운드경험디자인</t>
-  </si>
-  <si>
-    <t>남궁기찬</t>
-  </si>
-  <si>
-    <t>월 11:00-14:00</t>
-  </si>
-  <si>
-    <t>7296001</t>
-  </si>
-  <si>
-    <t>제품서비스시스템디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>심유리</t>
-  </si>
-  <si>
-    <t>월 10:00-17:00</t>
-  </si>
-  <si>
-    <t>7296101</t>
-  </si>
-  <si>
-    <t>정보디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>허정현</t>
-  </si>
-  <si>
-    <t>월 18:00-20:40,수 14:30-17:30</t>
-  </si>
-  <si>
-    <t>조형관별관3층3호실,조형관별관3층10호실</t>
-  </si>
-  <si>
-    <t>7296201</t>
-  </si>
-  <si>
-    <t>공공서비스디자인</t>
-  </si>
-  <si>
-    <t>박순정</t>
-  </si>
-  <si>
-    <t>조형관별관3층9호실</t>
-  </si>
-  <si>
-    <t>7296301</t>
-  </si>
-  <si>
-    <t>정량연구방법</t>
-  </si>
-  <si>
-    <t>36320</t>
-  </si>
-  <si>
-    <t>공간ㆍ문화디자인학과</t>
-  </si>
-  <si>
-    <t>704200b</t>
-  </si>
-  <si>
-    <t>7243701</t>
-  </si>
-  <si>
-    <t>특수연구과제2</t>
-  </si>
-  <si>
-    <t>윤성호</t>
-  </si>
-  <si>
-    <t>조형관별관3층14호실</t>
-  </si>
-  <si>
-    <t>7294501</t>
-  </si>
-  <si>
-    <t>7295101</t>
-  </si>
-  <si>
-    <t>강민선</t>
-  </si>
-  <si>
-    <t>707590a</t>
-  </si>
-  <si>
-    <t>소재 융합 개발 연구</t>
-  </si>
-  <si>
-    <t>이순정</t>
-  </si>
-  <si>
-    <t>토 10:00-13:00</t>
-  </si>
-  <si>
-    <t>7129001</t>
-  </si>
-  <si>
-    <t>디자인리서치&amp;방법론</t>
-  </si>
-  <si>
-    <t>7192201</t>
-  </si>
-  <si>
-    <t>글로벌 디자인 워크샵</t>
-  </si>
-  <si>
-    <t>정상엽</t>
-  </si>
-  <si>
-    <t>7192301</t>
-  </si>
-  <si>
-    <t>공간디자인 리서치 1</t>
-  </si>
-  <si>
-    <t>고은주</t>
-  </si>
-  <si>
-    <t>7243801</t>
-  </si>
-  <si>
-    <t>현대도시디자인</t>
-  </si>
-  <si>
-    <t>김상호</t>
-  </si>
-  <si>
-    <t>7262401</t>
-  </si>
-  <si>
-    <t>사진과 문화공간</t>
-  </si>
-  <si>
-    <t>김규랑</t>
   </si>
   <si>
     <t>7294101</t>
@@ -31015,7 +31015,7 @@
         <v>21</v>
       </c>
       <c r="L515" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M515" t="s">
         <v>23</v>
@@ -31038,16 +31038,16 @@
         <v>52</v>
       </c>
       <c r="F516" t="s">
+        <v>1554</v>
+      </c>
+      <c r="G516" t="s">
         <v>1555</v>
       </c>
-      <c r="G516" t="s">
+      <c r="H516">
+        <v>3</v>
+      </c>
+      <c r="I516" t="s">
         <v>1556</v>
-      </c>
-      <c r="H516">
-        <v>3</v>
-      </c>
-      <c r="I516" t="s">
-        <v>1557</v>
       </c>
       <c r="J516" t="s">
         <v>163</v>
@@ -31056,7 +31056,7 @@
         <v>21</v>
       </c>
       <c r="L516" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M516" t="s">
         <v>23</v>
@@ -31079,25 +31079,25 @@
         <v>52</v>
       </c>
       <c r="F517" t="s">
+        <v>1558</v>
+      </c>
+      <c r="G517" t="s">
         <v>1559</v>
       </c>
-      <c r="G517" t="s">
+      <c r="H517">
+        <v>3</v>
+      </c>
+      <c r="I517" t="s">
         <v>1560</v>
       </c>
-      <c r="H517">
-        <v>3</v>
-      </c>
-      <c r="I517" t="s">
+      <c r="J517" t="s">
         <v>1561</v>
       </c>
-      <c r="J517" t="s">
-        <v>1562</v>
-      </c>
       <c r="K517" t="s">
         <v>21</v>
       </c>
       <c r="L517" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M517" t="s">
         <v>23</v>
@@ -31120,10 +31120,10 @@
         <v>52</v>
       </c>
       <c r="F518" t="s">
+        <v>1562</v>
+      </c>
+      <c r="G518" t="s">
         <v>1563</v>
-      </c>
-      <c r="G518" t="s">
-        <v>1564</v>
       </c>
       <c r="H518">
         <v>3</v>
@@ -31138,7 +31138,7 @@
         <v>21</v>
       </c>
       <c r="L518" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M518" t="s">
         <v>23</v>
@@ -31158,13 +31158,13 @@
         <v>1541</v>
       </c>
       <c r="E519" t="s">
+        <v>1565</v>
+      </c>
+      <c r="F519" t="s">
         <v>1566</v>
       </c>
-      <c r="F519" t="s">
+      <c r="G519" t="s">
         <v>1567</v>
-      </c>
-      <c r="G519" t="s">
-        <v>1568</v>
       </c>
       <c r="H519">
         <v>6</v>
@@ -31173,13 +31173,13 @@
         <v>205</v>
       </c>
       <c r="J519" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="K519" t="s">
         <v>21</v>
       </c>
       <c r="L519" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M519" t="s">
         <v>23</v>
@@ -31202,16 +31202,16 @@
         <v>52</v>
       </c>
       <c r="F520" t="s">
+        <v>1569</v>
+      </c>
+      <c r="G520" t="s">
         <v>1570</v>
       </c>
-      <c r="G520" t="s">
+      <c r="H520">
+        <v>3</v>
+      </c>
+      <c r="I520" t="s">
         <v>1571</v>
-      </c>
-      <c r="H520">
-        <v>3</v>
-      </c>
-      <c r="I520" t="s">
-        <v>1572</v>
       </c>
       <c r="J520" t="s">
         <v>359</v>
@@ -31243,19 +31243,19 @@
         <v>52</v>
       </c>
       <c r="F521" t="s">
+        <v>1572</v>
+      </c>
+      <c r="G521" t="s">
         <v>1573</v>
       </c>
-      <c r="G521" t="s">
+      <c r="H521">
+        <v>3</v>
+      </c>
+      <c r="I521" t="s">
         <v>1574</v>
       </c>
-      <c r="H521">
-        <v>3</v>
-      </c>
-      <c r="I521" t="s">
+      <c r="J521" t="s">
         <v>1575</v>
-      </c>
-      <c r="J521" t="s">
-        <v>1576</v>
       </c>
       <c r="K521" t="s">
         <v>21</v>
@@ -31284,16 +31284,16 @@
         <v>52</v>
       </c>
       <c r="F522" t="s">
+        <v>1576</v>
+      </c>
+      <c r="G522" t="s">
         <v>1577</v>
       </c>
-      <c r="G522" t="s">
-        <v>1578</v>
-      </c>
       <c r="H522">
         <v>3</v>
       </c>
       <c r="I522" t="s">
-        <v>1557</v>
+        <v>1556</v>
       </c>
       <c r="J522" t="s">
         <v>863</v>
@@ -31302,7 +31302,7 @@
         <v>21</v>
       </c>
       <c r="L522" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M522" t="s">
         <v>23</v>
@@ -31325,16 +31325,16 @@
         <v>52</v>
       </c>
       <c r="F523" t="s">
+        <v>1578</v>
+      </c>
+      <c r="G523" t="s">
         <v>1579</v>
       </c>
-      <c r="G523" t="s">
+      <c r="H523">
+        <v>3</v>
+      </c>
+      <c r="I523" t="s">
         <v>1580</v>
-      </c>
-      <c r="H523">
-        <v>3</v>
-      </c>
-      <c r="I523" t="s">
-        <v>1581</v>
       </c>
       <c r="J523" t="s">
         <v>567</v>
@@ -31343,7 +31343,7 @@
         <v>21</v>
       </c>
       <c r="L523" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M523" t="s">
         <v>23</v>
@@ -31366,16 +31366,16 @@
         <v>52</v>
       </c>
       <c r="F524" t="s">
+        <v>1581</v>
+      </c>
+      <c r="G524" t="s">
         <v>1582</v>
       </c>
-      <c r="G524" t="s">
-        <v>1583</v>
-      </c>
       <c r="H524">
         <v>3</v>
       </c>
       <c r="I524" t="s">
-        <v>1561</v>
+        <v>1560</v>
       </c>
       <c r="J524" t="s">
         <v>1549</v>
@@ -31407,16 +31407,16 @@
         <v>52</v>
       </c>
       <c r="F525" t="s">
+        <v>1583</v>
+      </c>
+      <c r="G525" t="s">
         <v>1584</v>
       </c>
-      <c r="G525" t="s">
+      <c r="H525">
+        <v>3</v>
+      </c>
+      <c r="I525" t="s">
         <v>1585</v>
-      </c>
-      <c r="H525">
-        <v>3</v>
-      </c>
-      <c r="I525" t="s">
-        <v>1586</v>
       </c>
       <c r="J525" t="s">
         <v>908</v>
@@ -31425,7 +31425,7 @@
         <v>21</v>
       </c>
       <c r="L525" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M525" t="s">
         <v>23</v>
@@ -31448,10 +31448,10 @@
         <v>52</v>
       </c>
       <c r="F526" t="s">
+        <v>1586</v>
+      </c>
+      <c r="G526" t="s">
         <v>1587</v>
-      </c>
-      <c r="G526" t="s">
-        <v>1588</v>
       </c>
       <c r="H526">
         <v>3</v>
@@ -31486,28 +31486,28 @@
         <v>1541</v>
       </c>
       <c r="E527" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F527" t="s">
+        <v>1588</v>
+      </c>
+      <c r="G527" t="s">
         <v>1589</v>
-      </c>
-      <c r="G527" t="s">
-        <v>1590</v>
       </c>
       <c r="H527">
         <v>6</v>
       </c>
       <c r="I527" t="s">
+        <v>1590</v>
+      </c>
+      <c r="J527" t="s">
         <v>1591</v>
       </c>
-      <c r="J527" t="s">
+      <c r="K527" t="s">
+        <v>21</v>
+      </c>
+      <c r="L527" t="s">
         <v>1592</v>
-      </c>
-      <c r="K527" t="s">
-        <v>21</v>
-      </c>
-      <c r="L527" t="s">
-        <v>1593</v>
       </c>
       <c r="M527" t="s">
         <v>23</v>
@@ -31527,28 +31527,28 @@
         <v>1541</v>
       </c>
       <c r="E528" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F528" t="s">
+        <v>1593</v>
+      </c>
+      <c r="G528" t="s">
         <v>1594</v>
-      </c>
-      <c r="G528" t="s">
-        <v>1595</v>
       </c>
       <c r="H528">
         <v>6</v>
       </c>
       <c r="I528" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J528" t="s">
         <v>1596</v>
       </c>
-      <c r="J528" t="s">
-        <v>1597</v>
-      </c>
       <c r="K528" t="s">
         <v>21</v>
       </c>
       <c r="L528" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M528" t="s">
         <v>23</v>
@@ -31568,28 +31568,28 @@
         <v>1541</v>
       </c>
       <c r="E529" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F529" t="s">
+        <v>1593</v>
+      </c>
+      <c r="G529" t="s">
         <v>1594</v>
-      </c>
-      <c r="G529" t="s">
-        <v>1595</v>
       </c>
       <c r="H529">
         <v>6</v>
       </c>
       <c r="I529" t="s">
+        <v>1597</v>
+      </c>
+      <c r="J529" t="s">
         <v>1598</v>
       </c>
-      <c r="J529" t="s">
-        <v>1599</v>
-      </c>
       <c r="K529" t="s">
         <v>21</v>
       </c>
       <c r="L529" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M529" t="s">
         <v>640</v>
@@ -31612,16 +31612,16 @@
         <v>52</v>
       </c>
       <c r="F530" t="s">
+        <v>1599</v>
+      </c>
+      <c r="G530" t="s">
         <v>1600</v>
       </c>
-      <c r="G530" t="s">
-        <v>1601</v>
-      </c>
       <c r="H530">
         <v>3</v>
       </c>
       <c r="I530" t="s">
-        <v>1591</v>
+        <v>1590</v>
       </c>
       <c r="J530" t="s">
         <v>86</v>
@@ -31653,16 +31653,16 @@
         <v>52</v>
       </c>
       <c r="F531" t="s">
+        <v>1601</v>
+      </c>
+      <c r="G531" t="s">
         <v>1602</v>
       </c>
-      <c r="G531" t="s">
-        <v>1603</v>
-      </c>
       <c r="H531">
         <v>3</v>
       </c>
       <c r="I531" t="s">
-        <v>1591</v>
+        <v>1590</v>
       </c>
       <c r="J531" t="s">
         <v>117</v>
@@ -31691,22 +31691,22 @@
         <v>1541</v>
       </c>
       <c r="E532" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F532" t="s">
+        <v>1603</v>
+      </c>
+      <c r="G532" t="s">
         <v>1604</v>
-      </c>
-      <c r="G532" t="s">
-        <v>1605</v>
       </c>
       <c r="H532">
         <v>6</v>
       </c>
       <c r="I532" t="s">
+        <v>1605</v>
+      </c>
+      <c r="J532" t="s">
         <v>1606</v>
-      </c>
-      <c r="J532" t="s">
-        <v>1607</v>
       </c>
       <c r="K532" t="s">
         <v>21</v>
@@ -31735,25 +31735,25 @@
         <v>52</v>
       </c>
       <c r="F533" t="s">
+        <v>1607</v>
+      </c>
+      <c r="G533" t="s">
         <v>1608</v>
       </c>
-      <c r="G533" t="s">
+      <c r="H533">
+        <v>3</v>
+      </c>
+      <c r="I533" t="s">
         <v>1609</v>
       </c>
-      <c r="H533">
-        <v>3</v>
-      </c>
-      <c r="I533" t="s">
+      <c r="J533" t="s">
         <v>1610</v>
       </c>
-      <c r="J533" t="s">
-        <v>1611</v>
-      </c>
       <c r="K533" t="s">
         <v>21</v>
       </c>
       <c r="L533" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M533" t="s">
         <v>23</v>
@@ -31773,22 +31773,22 @@
         <v>1541</v>
       </c>
       <c r="E534" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F534" t="s">
+        <v>1611</v>
+      </c>
+      <c r="G534" t="s">
         <v>1612</v>
-      </c>
-      <c r="G534" t="s">
-        <v>1613</v>
       </c>
       <c r="H534">
         <v>6</v>
       </c>
       <c r="I534" t="s">
+        <v>1613</v>
+      </c>
+      <c r="J534" t="s">
         <v>1614</v>
-      </c>
-      <c r="J534" t="s">
-        <v>1615</v>
       </c>
       <c r="K534" t="s">
         <v>21</v>
@@ -31814,28 +31814,28 @@
         <v>1541</v>
       </c>
       <c r="E535" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F535" t="s">
+        <v>1615</v>
+      </c>
+      <c r="G535" t="s">
         <v>1616</v>
-      </c>
-      <c r="G535" t="s">
-        <v>1617</v>
       </c>
       <c r="H535">
         <v>6</v>
       </c>
       <c r="I535" t="s">
+        <v>1617</v>
+      </c>
+      <c r="J535" t="s">
         <v>1618</v>
       </c>
-      <c r="J535" t="s">
+      <c r="K535" t="s">
+        <v>21</v>
+      </c>
+      <c r="L535" t="s">
         <v>1619</v>
-      </c>
-      <c r="K535" t="s">
-        <v>21</v>
-      </c>
-      <c r="L535" t="s">
-        <v>1620</v>
       </c>
       <c r="M535" t="s">
         <v>23</v>
@@ -31858,16 +31858,16 @@
         <v>52</v>
       </c>
       <c r="F536" t="s">
+        <v>1620</v>
+      </c>
+      <c r="G536" t="s">
         <v>1621</v>
       </c>
-      <c r="G536" t="s">
+      <c r="H536">
+        <v>3</v>
+      </c>
+      <c r="I536" t="s">
         <v>1622</v>
-      </c>
-      <c r="H536">
-        <v>3</v>
-      </c>
-      <c r="I536" t="s">
-        <v>1623</v>
       </c>
       <c r="J536" t="s">
         <v>86</v>
@@ -31876,7 +31876,7 @@
         <v>21</v>
       </c>
       <c r="L536" t="s">
-        <v>1624</v>
+        <v>1623</v>
       </c>
       <c r="M536" t="s">
         <v>23</v>
@@ -31899,16 +31899,16 @@
         <v>52</v>
       </c>
       <c r="F537" t="s">
+        <v>1624</v>
+      </c>
+      <c r="G537" t="s">
         <v>1625</v>
       </c>
-      <c r="G537" t="s">
-        <v>1626</v>
-      </c>
       <c r="H537">
         <v>3</v>
       </c>
       <c r="I537" t="s">
-        <v>1596</v>
+        <v>1595</v>
       </c>
       <c r="J537" t="s">
         <v>163</v>
@@ -31917,7 +31917,7 @@
         <v>21</v>
       </c>
       <c r="L537" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M537" t="s">
         <v>23</v>
@@ -31931,16 +31931,16 @@
         <v>1501</v>
       </c>
       <c r="C538" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D538" t="s">
         <v>1627</v>
-      </c>
-      <c r="D538" t="s">
-        <v>1628</v>
       </c>
       <c r="E538" t="s">
         <v>52</v>
       </c>
       <c r="F538" t="s">
-        <v>1629</v>
+        <v>1628</v>
       </c>
       <c r="G538" t="s">
         <v>1543</v>
@@ -31972,25 +31972,25 @@
         <v>1501</v>
       </c>
       <c r="C539" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D539" t="s">
         <v>1627</v>
-      </c>
-      <c r="D539" t="s">
-        <v>1628</v>
       </c>
       <c r="E539" t="s">
         <v>52</v>
       </c>
       <c r="F539" t="s">
+        <v>1629</v>
+      </c>
+      <c r="G539" t="s">
         <v>1630</v>
       </c>
-      <c r="G539" t="s">
+      <c r="H539">
+        <v>3</v>
+      </c>
+      <c r="I539" t="s">
         <v>1631</v>
-      </c>
-      <c r="H539">
-        <v>3</v>
-      </c>
-      <c r="I539" t="s">
-        <v>1632</v>
       </c>
       <c r="J539" t="s">
         <v>70</v>
@@ -31999,7 +31999,7 @@
         <v>21</v>
       </c>
       <c r="L539" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="M539" t="s">
         <v>23</v>
@@ -32013,16 +32013,16 @@
         <v>1501</v>
       </c>
       <c r="C540" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D540" t="s">
         <v>1627</v>
-      </c>
-      <c r="D540" t="s">
-        <v>1628</v>
       </c>
       <c r="E540" t="s">
         <v>52</v>
       </c>
       <c r="F540" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="G540" t="s">
         <v>1552</v>
@@ -32054,16 +32054,16 @@
         <v>1501</v>
       </c>
       <c r="C541" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D541" t="s">
         <v>1627</v>
-      </c>
-      <c r="D541" t="s">
-        <v>1628</v>
       </c>
       <c r="E541" t="s">
         <v>52</v>
       </c>
       <c r="F541" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="G541" t="s">
         <v>1548</v>
@@ -32072,7 +32072,7 @@
         <v>3</v>
       </c>
       <c r="I541" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J541" t="s">
         <v>359</v>
@@ -32095,34 +32095,34 @@
         <v>1501</v>
       </c>
       <c r="C542" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D542" t="s">
         <v>1627</v>
-      </c>
-      <c r="D542" t="s">
-        <v>1628</v>
       </c>
       <c r="E542" t="s">
         <v>52</v>
       </c>
       <c r="F542" t="s">
+        <v>1636</v>
+      </c>
+      <c r="G542" t="s">
         <v>1637</v>
       </c>
-      <c r="G542" t="s">
+      <c r="H542">
+        <v>3</v>
+      </c>
+      <c r="I542" t="s">
         <v>1638</v>
       </c>
-      <c r="H542">
-        <v>3</v>
-      </c>
-      <c r="I542" t="s">
+      <c r="J542" t="s">
         <v>1639</v>
       </c>
-      <c r="J542" t="s">
-        <v>1640</v>
-      </c>
       <c r="K542" t="s">
         <v>21</v>
       </c>
       <c r="L542" t="s">
-        <v>1624</v>
+        <v>1623</v>
       </c>
       <c r="M542" t="s">
         <v>23</v>
@@ -32136,19 +32136,19 @@
         <v>1501</v>
       </c>
       <c r="C543" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D543" t="s">
         <v>1627</v>
-      </c>
-      <c r="D543" t="s">
-        <v>1628</v>
       </c>
       <c r="E543" t="s">
         <v>52</v>
       </c>
       <c r="F543" t="s">
+        <v>1640</v>
+      </c>
+      <c r="G543" t="s">
         <v>1641</v>
-      </c>
-      <c r="G543" t="s">
-        <v>1642</v>
       </c>
       <c r="H543">
         <v>3</v>
@@ -32177,25 +32177,25 @@
         <v>1501</v>
       </c>
       <c r="C544" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D544" t="s">
         <v>1627</v>
       </c>
-      <c r="D544" t="s">
-        <v>1628</v>
-      </c>
       <c r="E544" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F544" t="s">
+        <v>1642</v>
+      </c>
+      <c r="G544" t="s">
         <v>1643</v>
       </c>
-      <c r="G544" t="s">
+      <c r="H544">
+        <v>3</v>
+      </c>
+      <c r="I544" t="s">
         <v>1644</v>
-      </c>
-      <c r="H544">
-        <v>3</v>
-      </c>
-      <c r="I544" t="s">
-        <v>1645</v>
       </c>
       <c r="J544" t="s">
         <v>854</v>
@@ -32204,7 +32204,7 @@
         <v>21</v>
       </c>
       <c r="L544" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M544" t="s">
         <v>23</v>
@@ -32218,25 +32218,25 @@
         <v>1501</v>
       </c>
       <c r="C545" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D545" t="s">
         <v>1627</v>
-      </c>
-      <c r="D545" t="s">
-        <v>1628</v>
       </c>
       <c r="E545" t="s">
         <v>52</v>
       </c>
       <c r="F545" t="s">
+        <v>1645</v>
+      </c>
+      <c r="G545" t="s">
         <v>1646</v>
       </c>
-      <c r="G545" t="s">
+      <c r="H545">
+        <v>3</v>
+      </c>
+      <c r="I545" t="s">
         <v>1647</v>
-      </c>
-      <c r="H545">
-        <v>3</v>
-      </c>
-      <c r="I545" t="s">
-        <v>1648</v>
       </c>
       <c r="J545" t="s">
         <v>163</v>
@@ -32259,25 +32259,25 @@
         <v>1501</v>
       </c>
       <c r="C546" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D546" t="s">
         <v>1627</v>
-      </c>
-      <c r="D546" t="s">
-        <v>1628</v>
       </c>
       <c r="E546" t="s">
         <v>52</v>
       </c>
       <c r="F546" t="s">
+        <v>1648</v>
+      </c>
+      <c r="G546" t="s">
         <v>1649</v>
       </c>
-      <c r="G546" t="s">
+      <c r="H546">
+        <v>3</v>
+      </c>
+      <c r="I546" t="s">
         <v>1650</v>
-      </c>
-      <c r="H546">
-        <v>3</v>
-      </c>
-      <c r="I546" t="s">
-        <v>1651</v>
       </c>
       <c r="J546" t="s">
         <v>99</v>
@@ -32286,7 +32286,7 @@
         <v>21</v>
       </c>
       <c r="L546" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="M546" t="s">
         <v>23</v>
@@ -32300,25 +32300,25 @@
         <v>1501</v>
       </c>
       <c r="C547" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D547" t="s">
         <v>1627</v>
-      </c>
-      <c r="D547" t="s">
-        <v>1628</v>
       </c>
       <c r="E547" t="s">
         <v>52</v>
       </c>
       <c r="F547" t="s">
+        <v>1651</v>
+      </c>
+      <c r="G547" t="s">
         <v>1652</v>
       </c>
-      <c r="G547" t="s">
+      <c r="H547">
+        <v>3</v>
+      </c>
+      <c r="I547" t="s">
         <v>1653</v>
-      </c>
-      <c r="H547">
-        <v>3</v>
-      </c>
-      <c r="I547" t="s">
-        <v>1654</v>
       </c>
       <c r="J547" t="s">
         <v>271</v>
@@ -32327,7 +32327,7 @@
         <v>21</v>
       </c>
       <c r="L547" t="s">
-        <v>1539</v>
+        <v>1654</v>
       </c>
       <c r="M547" t="s">
         <v>23</v>
@@ -32341,10 +32341,10 @@
         <v>1501</v>
       </c>
       <c r="C548" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D548" t="s">
         <v>1627</v>
-      </c>
-      <c r="D548" t="s">
-        <v>1628</v>
       </c>
       <c r="E548" t="s">
         <v>52</v>
@@ -32362,7 +32362,7 @@
         <v>1657</v>
       </c>
       <c r="J548" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="K548" t="s">
         <v>21</v>
@@ -32382,10 +32382,10 @@
         <v>1501</v>
       </c>
       <c r="C549" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D549" t="s">
         <v>1627</v>
-      </c>
-      <c r="D549" t="s">
-        <v>1628</v>
       </c>
       <c r="E549" t="s">
         <v>52</v>
@@ -32423,13 +32423,13 @@
         <v>1501</v>
       </c>
       <c r="C550" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D550" t="s">
         <v>1627</v>
       </c>
-      <c r="D550" t="s">
-        <v>1628</v>
-      </c>
       <c r="E550" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F550" t="s">
         <v>1660</v>
@@ -32464,13 +32464,13 @@
         <v>1501</v>
       </c>
       <c r="C551" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D551" t="s">
         <v>1627</v>
       </c>
-      <c r="D551" t="s">
-        <v>1628</v>
-      </c>
       <c r="E551" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F551" t="s">
         <v>1664</v>
@@ -32482,7 +32482,7 @@
         <v>3</v>
       </c>
       <c r="I551" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J551" t="s">
         <v>148</v>
@@ -32491,7 +32491,7 @@
         <v>21</v>
       </c>
       <c r="L551" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M551" t="s">
         <v>23</v>
@@ -32505,10 +32505,10 @@
         <v>1501</v>
       </c>
       <c r="C552" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D552" t="s">
         <v>1627</v>
-      </c>
-      <c r="D552" t="s">
-        <v>1628</v>
       </c>
       <c r="E552" t="s">
         <v>52</v>
@@ -32532,7 +32532,7 @@
         <v>21</v>
       </c>
       <c r="L552" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M552" t="s">
         <v>23</v>
@@ -32546,13 +32546,13 @@
         <v>1501</v>
       </c>
       <c r="C553" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D553" t="s">
         <v>1627</v>
       </c>
-      <c r="D553" t="s">
-        <v>1628</v>
-      </c>
       <c r="E553" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F553" t="s">
         <v>1669</v>
@@ -32587,10 +32587,10 @@
         <v>1501</v>
       </c>
       <c r="C554" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D554" t="s">
         <v>1627</v>
-      </c>
-      <c r="D554" t="s">
-        <v>1628</v>
       </c>
       <c r="E554" t="s">
         <v>52</v>
@@ -32614,7 +32614,7 @@
         <v>21</v>
       </c>
       <c r="L554" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M554" t="s">
         <v>23</v>
@@ -32628,13 +32628,13 @@
         <v>1501</v>
       </c>
       <c r="C555" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D555" t="s">
         <v>1627</v>
       </c>
-      <c r="D555" t="s">
-        <v>1628</v>
-      </c>
       <c r="E555" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F555" t="s">
         <v>1674</v>
@@ -32655,7 +32655,7 @@
         <v>21</v>
       </c>
       <c r="L555" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="M555" t="s">
         <v>23</v>
@@ -32669,13 +32669,13 @@
         <v>1501</v>
       </c>
       <c r="C556" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D556" t="s">
         <v>1627</v>
       </c>
-      <c r="D556" t="s">
-        <v>1628</v>
-      </c>
       <c r="E556" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F556" t="s">
         <v>1676</v>
@@ -32696,7 +32696,7 @@
         <v>21</v>
       </c>
       <c r="L556" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M556" t="s">
         <v>23</v>
@@ -32710,13 +32710,13 @@
         <v>1501</v>
       </c>
       <c r="C557" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D557" t="s">
         <v>1627</v>
       </c>
-      <c r="D557" t="s">
-        <v>1628</v>
-      </c>
       <c r="E557" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F557" t="s">
         <v>1678</v>
@@ -32728,7 +32728,7 @@
         <v>3</v>
       </c>
       <c r="I557" t="s">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="J557" t="s">
         <v>908</v>
@@ -32737,7 +32737,7 @@
         <v>21</v>
       </c>
       <c r="L557" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="M557" t="s">
         <v>23</v>
@@ -32751,13 +32751,13 @@
         <v>1501</v>
       </c>
       <c r="C558" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D558" t="s">
         <v>1627</v>
       </c>
-      <c r="D558" t="s">
-        <v>1628</v>
-      </c>
       <c r="E558" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F558" t="s">
         <v>1680</v>
@@ -32769,7 +32769,7 @@
         <v>3</v>
       </c>
       <c r="I558" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="J558" t="s">
         <v>854</v>
@@ -32778,7 +32778,7 @@
         <v>21</v>
       </c>
       <c r="L558" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M558" t="s">
         <v>23</v>
@@ -32860,7 +32860,7 @@
         <v>21</v>
       </c>
       <c r="L560" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M560" t="s">
         <v>23</v>
@@ -32901,7 +32901,7 @@
         <v>21</v>
       </c>
       <c r="L561" t="s">
-        <v>1539</v>
+        <v>1654</v>
       </c>
       <c r="M561" t="s">
         <v>23</v>
@@ -32921,7 +32921,7 @@
         <v>1683</v>
       </c>
       <c r="E562" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F562" t="s">
         <v>1690</v>
@@ -32962,7 +32962,7 @@
         <v>1683</v>
       </c>
       <c r="E563" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F563" t="s">
         <v>1694</v>
@@ -32983,7 +32983,7 @@
         <v>21</v>
       </c>
       <c r="L563" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="M563" t="s">
         <v>23</v>
@@ -33024,7 +33024,7 @@
         <v>21</v>
       </c>
       <c r="L564" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M564" t="s">
         <v>23</v>
@@ -33065,7 +33065,7 @@
         <v>21</v>
       </c>
       <c r="L565" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M565" t="s">
         <v>23</v>
@@ -33085,7 +33085,7 @@
         <v>1683</v>
       </c>
       <c r="E566" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F566" t="s">
         <v>1701</v>
@@ -33147,7 +33147,7 @@
         <v>21</v>
       </c>
       <c r="L567" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M567" t="s">
         <v>23</v>
@@ -33188,7 +33188,7 @@
         <v>21</v>
       </c>
       <c r="L568" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M568" t="s">
         <v>23</v>
@@ -33229,7 +33229,7 @@
         <v>21</v>
       </c>
       <c r="L569" t="s">
-        <v>1554</v>
+        <v>1539</v>
       </c>
       <c r="M569" t="s">
         <v>23</v>
@@ -33331,7 +33331,7 @@
         <v>1683</v>
       </c>
       <c r="E572" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F572" t="s">
         <v>1716</v>
@@ -33393,7 +33393,7 @@
         <v>21</v>
       </c>
       <c r="L573" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="M573" t="s">
         <v>23</v>
@@ -33413,7 +33413,7 @@
         <v>1683</v>
       </c>
       <c r="E574" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F574" t="s">
         <v>1722</v>
@@ -33454,7 +33454,7 @@
         <v>1683</v>
       </c>
       <c r="E575" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="F575" t="s">
         <v>1725</v>
@@ -33674,7 +33674,7 @@
         <v>1735</v>
       </c>
       <c r="J580" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="K580" t="s">
         <v>21</v>
@@ -34002,7 +34002,7 @@
         <v>1773</v>
       </c>
       <c r="J588" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="K588" t="s">
         <v>21</v>
@@ -34289,7 +34289,7 @@
         <v>1794</v>
       </c>
       <c r="J595" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="K595" t="s">
         <v>21</v>
@@ -34412,7 +34412,7 @@
         <v>1803</v>
       </c>
       <c r="J598" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="K598" t="s">
         <v>21</v>
@@ -34617,7 +34617,7 @@
         <v>1819</v>
       </c>
       <c r="J603" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="K603" t="s">
         <v>21</v>
@@ -42653,7 +42653,7 @@
         <v>2427</v>
       </c>
       <c r="J799" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="K799" t="s">
         <v>21</v>
@@ -42773,7 +42773,7 @@
         <v>3</v>
       </c>
       <c r="I802" t="s">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="J802" t="s">
         <v>355</v>
@@ -42814,7 +42814,7 @@
         <v>3</v>
       </c>
       <c r="I803" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J803" t="s">
         <v>2420</v>
@@ -43511,7 +43511,7 @@
         <v>3</v>
       </c>
       <c r="I820" t="s">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="J820" t="s">
         <v>355</v>
@@ -43520,7 +43520,7 @@
         <v>21</v>
       </c>
       <c r="L820" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="M820" t="s">
         <v>23</v>
@@ -43552,7 +43552,7 @@
         <v>3</v>
       </c>
       <c r="I821" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="J821" t="s">
         <v>2420</v>
@@ -47652,7 +47652,7 @@
         <v>2</v>
       </c>
       <c r="I921" t="s">
-        <v>1596</v>
+        <v>1595</v>
       </c>
       <c r="J921" t="s">
         <v>678</v>
@@ -48103,7 +48103,7 @@
         <v>2</v>
       </c>
       <c r="I932" t="s">
-        <v>1557</v>
+        <v>1556</v>
       </c>
       <c r="J932" t="s">
         <v>2642</v>

</xml_diff>